<commit_message>
use official data for stock analysis
</commit_message>
<xml_diff>
--- a/output/stock_analysis_result.xlsx
+++ b/output/stock_analysis_result.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T27"/>
+  <dimension ref="A1:T33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -521,52 +521,52 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2609.TW</t>
+          <t>2383.TW</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>陽明</t>
+          <t>台光電</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>53</v>
+        <v>5505</v>
       </c>
       <c r="D2" t="n">
-        <v>50.49</v>
+        <v>4826</v>
       </c>
       <c r="E2" t="n">
-        <v>49.92</v>
+        <v>4804</v>
       </c>
       <c r="F2" t="n">
-        <v>49.9</v>
+        <v>4756.25</v>
       </c>
       <c r="G2" t="n">
-        <v>44114173</v>
+        <v>1801298</v>
       </c>
       <c r="H2" t="n">
-        <v>24067636</v>
+        <v>2244504</v>
       </c>
       <c r="I2" t="n">
-        <v>53.9</v>
+        <v>5505</v>
       </c>
       <c r="J2" t="n">
-        <v>47.35</v>
+        <v>4160</v>
       </c>
       <c r="K2" t="n">
-        <v>10000</v>
+        <v>359818</v>
       </c>
       <c r="L2" t="n">
-        <v>20000</v>
+        <v>1354542</v>
       </c>
       <c r="M2" t="n">
-        <v>35000</v>
+        <v>1447903</v>
       </c>
       <c r="N2" t="n">
-        <v>50000</v>
+        <v>2950399</v>
       </c>
       <c r="O2" t="n">
-        <v>130</v>
+        <v>155</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
@@ -580,69 +580,69 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>站上5日線、多頭排列、黃金交叉、爆量、接近20日高點</t>
+          <t>站上5日線、多頭排列、黃金交叉、量能未放大、突破20日高點</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>籌碼轉強</t>
+          <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>短線偏強，站上5日線、多頭排列、黃金交叉、爆量、接近20日高點，可以列入觀察，但仍要注意是否追高。</t>
+          <t>強勢偏多：站上5日線、多頭排列、黃金交叉、量能未放大、突破20日高點、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2409.TW</t>
+          <t>2317.TW</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>友達</t>
+          <t>鴻海</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>22.2</v>
+        <v>261</v>
       </c>
       <c r="D3" t="n">
-        <v>19.91</v>
+        <v>248.7</v>
       </c>
       <c r="E3" t="n">
-        <v>19.79</v>
+        <v>248.6</v>
       </c>
       <c r="F3" t="n">
-        <v>18.66</v>
+        <v>242.93</v>
       </c>
       <c r="G3" t="n">
-        <v>392811029</v>
+        <v>122990174</v>
       </c>
       <c r="H3" t="n">
-        <v>254953321</v>
+        <v>72731564</v>
       </c>
       <c r="I3" t="n">
-        <v>22.2</v>
+        <v>263.5</v>
       </c>
       <c r="J3" t="n">
-        <v>16.6</v>
+        <v>219.5</v>
       </c>
       <c r="K3" t="n">
-        <v>8000</v>
+        <v>55787312</v>
       </c>
       <c r="L3" t="n">
-        <v>12000</v>
+        <v>101690979</v>
       </c>
       <c r="M3" t="n">
-        <v>20000</v>
+        <v>84630201</v>
       </c>
       <c r="N3" t="n">
-        <v>35000</v>
+        <v>160089561</v>
       </c>
       <c r="O3" t="n">
-        <v>115</v>
+        <v>135</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
@@ -656,17 +656,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>站上5日線、多頭排列、爆量、突破20日高點</t>
+          <t>站上5日線、多頭排列、成交量放大、接近20日高點</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>籌碼轉強</t>
+          <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>短線偏強，站上5日線、多頭排列、爆量、突破20日高點，可以列入觀察，但仍要注意是否追高。</t>
+          <t>強勢偏多：站上5日線、多頭排列、成交量放大、接近20日高點、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
@@ -682,43 +682,43 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>11.85</v>
+        <v>13</v>
       </c>
       <c r="D4" t="n">
-        <v>10.6</v>
+        <v>11.13</v>
       </c>
       <c r="E4" t="n">
-        <v>10.53</v>
+        <v>10.86</v>
       </c>
       <c r="F4" t="n">
-        <v>9.52</v>
+        <v>9.75</v>
       </c>
       <c r="G4" t="n">
-        <v>100795639</v>
+        <v>43724582</v>
       </c>
       <c r="H4" t="n">
-        <v>63097678</v>
+        <v>60470183</v>
       </c>
       <c r="I4" t="n">
-        <v>11.85</v>
+        <v>13</v>
       </c>
       <c r="J4" t="n">
         <v>8.119999999999999</v>
       </c>
       <c r="K4" t="n">
-        <v>3000</v>
+        <v>2108293</v>
       </c>
       <c r="L4" t="n">
-        <v>5000</v>
+        <v>59515291</v>
       </c>
       <c r="M4" t="n">
-        <v>8000</v>
+        <v>56282808</v>
       </c>
       <c r="N4" t="n">
-        <v>12000</v>
+        <v>50628800</v>
       </c>
       <c r="O4" t="n">
-        <v>115</v>
+        <v>130</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
@@ -732,69 +732,69 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>站上5日線、多頭排列、爆量、突破20日高點</t>
+          <t>站上5日線、多頭排列、量能未放大、突破20日高點</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>籌碼轉強</t>
+          <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>短線偏強，站上5日線、多頭排列、爆量、突破20日高點，可以列入觀察，但仍要注意是否追高。</t>
+          <t>強勢偏多：站上5日線、多頭排列、量能未放大、突破20日高點、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>4958.TW</t>
+          <t>2409.TW</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>臻鼎-KY</t>
+          <t>友達</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>516</v>
+        <v>24.4</v>
       </c>
       <c r="D5" t="n">
-        <v>444.3</v>
+        <v>20.94</v>
       </c>
       <c r="E5" t="n">
-        <v>432.05</v>
+        <v>20.35</v>
       </c>
       <c r="F5" t="n">
-        <v>416.18</v>
+        <v>19.02</v>
       </c>
       <c r="G5" t="n">
-        <v>50890468</v>
+        <v>82302936</v>
       </c>
       <c r="H5" t="n">
-        <v>46138661</v>
+        <v>230537458</v>
       </c>
       <c r="I5" t="n">
-        <v>516</v>
+        <v>24.4</v>
       </c>
       <c r="J5" t="n">
-        <v>331</v>
+        <v>16.6</v>
       </c>
       <c r="K5" t="n">
-        <v>12000</v>
+        <v>18947923</v>
       </c>
       <c r="L5" t="n">
-        <v>25000</v>
+        <v>211604454</v>
       </c>
       <c r="M5" t="n">
-        <v>45000</v>
+        <v>192942642</v>
       </c>
       <c r="N5" t="n">
-        <v>80000</v>
+        <v>353520387</v>
       </c>
       <c r="O5" t="n">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
@@ -808,69 +808,69 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>站上5日線、多頭排列、成交量放大、突破20日高點</t>
+          <t>站上5日線、多頭排列、量能未放大、突破20日高點</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>籌碼轉強</t>
+          <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>短線偏強，站上5日線、多頭排列、成交量放大、突破20日高點，可以列入觀察，但仍要注意是否追高。</t>
+          <t>強勢偏多：站上5日線、多頭排列、量能未放大、突破20日高點、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2327.TW</t>
+          <t>2312.TW</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>國巨</t>
+          <t>金寶</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>629</v>
+        <v>36.4</v>
       </c>
       <c r="D6" t="n">
-        <v>543.8</v>
+        <v>31.13</v>
       </c>
       <c r="E6" t="n">
-        <v>486.75</v>
+        <v>29.88</v>
       </c>
       <c r="F6" t="n">
-        <v>411.23</v>
+        <v>29.14</v>
       </c>
       <c r="G6" t="n">
-        <v>72182688</v>
+        <v>66663284</v>
       </c>
       <c r="H6" t="n">
-        <v>71442747</v>
+        <v>67343380</v>
       </c>
       <c r="I6" t="n">
-        <v>629</v>
+        <v>36.4</v>
       </c>
       <c r="J6" t="n">
-        <v>290</v>
+        <v>25.45</v>
       </c>
       <c r="K6" t="n">
-        <v>15000</v>
+        <v>10178504</v>
       </c>
       <c r="L6" t="n">
-        <v>25000</v>
+        <v>70925202</v>
       </c>
       <c r="M6" t="n">
-        <v>40000</v>
+        <v>76924762</v>
       </c>
       <c r="N6" t="n">
-        <v>70000</v>
+        <v>66944449</v>
       </c>
       <c r="O6" t="n">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
@@ -884,69 +884,69 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>站上5日線、多頭排列、成交量放大、突破20日高點</t>
+          <t>站上5日線、多頭排列、量能未放大、突破20日高點</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>籌碼轉強</t>
+          <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>短線偏強，站上5日線、多頭排列、成交量放大、突破20日高點，可以列入觀察，但仍要注意是否追高。</t>
+          <t>強勢偏多：站上5日線、多頭排列、量能未放大、突破20日高點、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>6239.TW</t>
+          <t>3189.TW</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>力成</t>
+          <t>景碩</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>283</v>
+        <v>669</v>
       </c>
       <c r="D7" t="n">
-        <v>250.4</v>
+        <v>569.8</v>
       </c>
       <c r="E7" t="n">
-        <v>241.3</v>
+        <v>535.35</v>
       </c>
       <c r="F7" t="n">
-        <v>230.18</v>
+        <v>520.33</v>
       </c>
       <c r="G7" t="n">
-        <v>6909104</v>
+        <v>8536899</v>
       </c>
       <c r="H7" t="n">
-        <v>25802698</v>
+        <v>26502334</v>
       </c>
       <c r="I7" t="n">
-        <v>283</v>
+        <v>669</v>
       </c>
       <c r="J7" t="n">
-        <v>201</v>
+        <v>445.5</v>
       </c>
       <c r="K7" t="n">
-        <v>6000</v>
+        <v>964619</v>
       </c>
       <c r="L7" t="n">
-        <v>12000</v>
+        <v>17496756</v>
       </c>
       <c r="M7" t="n">
-        <v>18000</v>
+        <v>19603616</v>
       </c>
       <c r="N7" t="n">
-        <v>25000</v>
+        <v>18095930</v>
       </c>
       <c r="O7" t="n">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
@@ -960,69 +960,69 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>站上5日線、多頭排列、成交量未放大、突破20日高點</t>
+          <t>站上5日線、多頭排列、量能未放大、突破20日高點</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>籌碼轉強</t>
+          <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>短線偏強，站上5日線、多頭排列、成交量未放大、突破20日高點，可以列入觀察，但仍要注意是否追高。</t>
+          <t>強勢偏多：站上5日線、多頭排列、量能未放大、突破20日高點、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>3189.TW</t>
+          <t>2338.TW</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>景碩</t>
+          <t>光罩</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>609</v>
+        <v>57.1</v>
       </c>
       <c r="D8" t="n">
-        <v>537</v>
+        <v>52.56</v>
       </c>
       <c r="E8" t="n">
-        <v>518.75</v>
+        <v>50.76</v>
       </c>
       <c r="F8" t="n">
-        <v>513.17</v>
+        <v>50.01</v>
       </c>
       <c r="G8" t="n">
-        <v>10417136</v>
+        <v>16550566</v>
       </c>
       <c r="H8" t="n">
-        <v>27927013</v>
+        <v>8831247</v>
       </c>
       <c r="I8" t="n">
-        <v>609</v>
+        <v>58.5</v>
       </c>
       <c r="J8" t="n">
-        <v>445.5</v>
+        <v>45.45</v>
       </c>
       <c r="K8" t="n">
-        <v>8000</v>
+        <v>3454745</v>
       </c>
       <c r="L8" t="n">
-        <v>15000</v>
+        <v>13009409</v>
       </c>
       <c r="M8" t="n">
-        <v>25000</v>
+        <v>14246624</v>
       </c>
       <c r="N8" t="n">
-        <v>40000</v>
+        <v>12266815</v>
       </c>
       <c r="O8" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
@@ -1036,69 +1036,69 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>站上5日線、多頭排列、成交量未放大、突破20日高點</t>
+          <t>站上5日線、多頭排列、成交量放大</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>籌碼轉強</t>
+          <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>短線偏強，站上5日線、多頭排列、成交量未放大、突破20日高點，可以列入觀察，但仍要注意是否追高。</t>
+          <t>強勢偏多：站上5日線、多頭排列、成交量放大、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>8358.TWO</t>
+          <t>6274.TWO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>金居</t>
+          <t>台燿</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>522</v>
+        <v>1600</v>
       </c>
       <c r="D9" t="n">
-        <v>467.4</v>
+        <v>1362</v>
       </c>
       <c r="E9" t="n">
-        <v>454.85</v>
+        <v>1372.5</v>
       </c>
       <c r="F9" t="n">
-        <v>429.05</v>
+        <v>1279.05</v>
       </c>
       <c r="G9" t="n">
-        <v>4202780</v>
+        <v>1486000</v>
       </c>
       <c r="H9" t="n">
-        <v>4332139</v>
+        <v>1401800</v>
       </c>
       <c r="I9" t="n">
-        <v>528</v>
+        <v>1600</v>
       </c>
       <c r="J9" t="n">
-        <v>324.5</v>
+        <v>941</v>
       </c>
       <c r="K9" t="n">
-        <v>2000</v>
+        <v>282254</v>
       </c>
       <c r="L9" t="n">
-        <v>6000</v>
+        <v>969253</v>
       </c>
       <c r="M9" t="n">
-        <v>9000</v>
+        <v>1221688</v>
       </c>
       <c r="N9" t="n">
-        <v>12000</v>
+        <v>2123947</v>
       </c>
       <c r="O9" t="n">
-        <v>90</v>
+        <v>115</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
@@ -1112,69 +1112,69 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>站上5日線、多頭排列、成交量未放大、接近20日高點</t>
+          <t>站上5日線、量能溫和放大、突破20日高點</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>籌碼轉強</t>
+          <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>短線偏強，站上5日線、多頭排列、成交量未放大、接近20日高點，可以列入觀察，但仍要注意是否追高。</t>
+          <t>強勢偏多：站上5日線、量能溫和放大、突破20日高點、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>3035.TW</t>
+          <t>3037.TW</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>智原</t>
+          <t>欣興</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>211</v>
+        <v>990</v>
       </c>
       <c r="D10" t="n">
-        <v>198</v>
+        <v>901.2</v>
       </c>
       <c r="E10" t="n">
-        <v>197.65</v>
+        <v>879.1</v>
       </c>
       <c r="F10" t="n">
-        <v>187.38</v>
+        <v>869.4</v>
       </c>
       <c r="G10" t="n">
-        <v>27951666</v>
+        <v>24465071</v>
       </c>
       <c r="H10" t="n">
-        <v>16214445</v>
+        <v>28813042</v>
       </c>
       <c r="I10" t="n">
-        <v>216.5</v>
+        <v>1030</v>
       </c>
       <c r="J10" t="n">
-        <v>167</v>
+        <v>776</v>
       </c>
       <c r="K10" t="n">
-        <v>10000</v>
+        <v>1191293</v>
       </c>
       <c r="L10" t="n">
-        <v>18000</v>
+        <v>14796086</v>
       </c>
       <c r="M10" t="n">
-        <v>30000</v>
+        <v>14042095</v>
       </c>
       <c r="N10" t="n">
-        <v>50000</v>
+        <v>12040296</v>
       </c>
       <c r="O10" t="n">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
@@ -1188,69 +1188,69 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>站上5日線、多頭排列、爆量</t>
+          <t>站上5日線、多頭排列、量能未放大</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>籌碼轉強</t>
+          <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>短線偏強，站上5日線、多頭排列、爆量，可以列入觀察，但仍要注意是否追高。</t>
+          <t>強勢偏多：站上5日線、多頭排列、量能未放大、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2338.TW</t>
+          <t>8358.TWO</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>光罩</t>
+          <t>金居</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>54.4</v>
+        <v>545</v>
       </c>
       <c r="D11" t="n">
-        <v>51.07</v>
+        <v>490.8</v>
       </c>
       <c r="E11" t="n">
-        <v>50.05</v>
+        <v>463.15</v>
       </c>
       <c r="F11" t="n">
-        <v>49.52</v>
+        <v>438.32</v>
       </c>
       <c r="G11" t="n">
-        <v>9214268</v>
+        <v>2767000</v>
       </c>
       <c r="H11" t="n">
-        <v>6313989</v>
+        <v>4459600</v>
       </c>
       <c r="I11" t="n">
-        <v>57</v>
+        <v>558</v>
       </c>
       <c r="J11" t="n">
-        <v>45.45</v>
+        <v>324.5</v>
       </c>
       <c r="K11" t="n">
-        <v>3000</v>
+        <v>434414</v>
       </c>
       <c r="L11" t="n">
-        <v>5000</v>
+        <v>4299788</v>
       </c>
       <c r="M11" t="n">
-        <v>8000</v>
+        <v>9649180</v>
       </c>
       <c r="N11" t="n">
-        <v>10000</v>
+        <v>9535283</v>
       </c>
       <c r="O11" t="n">
-        <v>85</v>
+        <v>105</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
@@ -1264,73 +1264,73 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>站上5日線、多頭排列、成交量放大</t>
+          <t>站上5日線、多頭排列、量能未放大</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>籌碼轉強</t>
+          <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>短線偏強，站上5日線、多頭排列、成交量放大，可以列入觀察，但仍要注意是否追高。</t>
+          <t>強勢偏多：站上5日線、多頭排列、量能未放大、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>6274.TWO</t>
+          <t>2344.TW</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>台燿</t>
+          <t>華邦電</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1455</v>
+        <v>128.5</v>
       </c>
       <c r="D12" t="n">
-        <v>1294</v>
+        <v>120.1</v>
       </c>
       <c r="E12" t="n">
-        <v>1358</v>
+        <v>123.8</v>
       </c>
       <c r="F12" t="n">
-        <v>1251.3</v>
+        <v>117.83</v>
       </c>
       <c r="G12" t="n">
-        <v>1582543</v>
+        <v>357612926</v>
       </c>
       <c r="H12" t="n">
-        <v>1588253</v>
+        <v>219239775</v>
       </c>
       <c r="I12" t="n">
-        <v>1480</v>
+        <v>136.5</v>
       </c>
       <c r="J12" t="n">
-        <v>941</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="K12" t="n">
-        <v>5000</v>
+        <v>77651903</v>
       </c>
       <c r="L12" t="n">
-        <v>10000</v>
+        <v>96687402</v>
       </c>
       <c r="M12" t="n">
-        <v>20000</v>
+        <v>61728965</v>
       </c>
       <c r="N12" t="n">
-        <v>35000</v>
+        <v>182119556</v>
       </c>
       <c r="O12" t="n">
-        <v>65</v>
+        <v>95</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>👀觀察</t>
+          <t>🔥強勢</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -1340,73 +1340,73 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>站上5日線、成交量未放大、接近20日高點</t>
+          <t>站上5日線、成交量放大</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>籌碼轉強</t>
+          <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>短線偏強，站上5日線、成交量未放大、接近20日高點，可以列入觀察，但仍要注意是否追高。</t>
+          <t>強勢偏多：站上5日線、成交量放大、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2312.TW</t>
+          <t>1802.TW</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>金寶</t>
+          <t>台玻</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>33.1</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="D13" t="n">
-        <v>29.54</v>
+        <v>67.73999999999999</v>
       </c>
       <c r="E13" t="n">
-        <v>29.23</v>
+        <v>67.45</v>
       </c>
       <c r="F13" t="n">
-        <v>28.62</v>
+        <v>68.11</v>
       </c>
       <c r="G13" t="n">
-        <v>134312480</v>
+        <v>185285181</v>
       </c>
       <c r="H13" t="n">
-        <v>58293636</v>
+        <v>96433207</v>
       </c>
       <c r="I13" t="n">
-        <v>33.1</v>
+        <v>76.8</v>
       </c>
       <c r="J13" t="n">
-        <v>25.35</v>
+        <v>61.7</v>
       </c>
       <c r="K13" t="n">
-        <v>-2000</v>
+        <v>44538498</v>
       </c>
       <c r="L13" t="n">
-        <v>-5000</v>
+        <v>88202486</v>
       </c>
       <c r="M13" t="n">
-        <v>-8000</v>
+        <v>75247740</v>
       </c>
       <c r="N13" t="n">
-        <v>-12000</v>
+        <v>32596649</v>
       </c>
       <c r="O13" t="n">
-        <v>65</v>
+        <v>95</v>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>👀觀察</t>
+          <t>🔥強勢</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -1416,73 +1416,73 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>站上5日線、多頭排列、超級爆量、突破20日高點</t>
+          <t>站上5日線、成交量放大</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>短線賣壓重</t>
+          <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>短線偏強，站上5日線、多頭排列、超級爆量、突破20日高點，可以列入觀察，但仍要注意是否追高。</t>
+          <t>強勢偏多：站上5日線、成交量放大、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>6669.TW</t>
+          <t>3711.TW</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>緯穎</t>
+          <t>日月光投控</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>5525</v>
+        <v>617</v>
       </c>
       <c r="D14" t="n">
-        <v>5152</v>
+        <v>527.2</v>
       </c>
       <c r="E14" t="n">
-        <v>5302</v>
+        <v>534.4</v>
       </c>
       <c r="F14" t="n">
-        <v>5076.5</v>
+        <v>523.17</v>
       </c>
       <c r="G14" t="n">
-        <v>1829705</v>
+        <v>26609382</v>
       </c>
       <c r="H14" t="n">
-        <v>1681714</v>
+        <v>28063686</v>
       </c>
       <c r="I14" t="n">
-        <v>5870</v>
+        <v>617</v>
       </c>
       <c r="J14" t="n">
-        <v>4320</v>
+        <v>465</v>
       </c>
       <c r="K14" t="n">
-        <v>15000</v>
+        <v>-1946569</v>
       </c>
       <c r="L14" t="n">
-        <v>30000</v>
+        <v>4398628</v>
       </c>
       <c r="M14" t="n">
-        <v>50000</v>
+        <v>375095</v>
       </c>
       <c r="N14" t="n">
-        <v>80000</v>
+        <v>-4267040</v>
       </c>
       <c r="O14" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>👀觀察</t>
+          <t>🔥強勢</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -1492,73 +1492,73 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>站上5日線、成交量放大</t>
+          <t>站上5日線、黃金交叉、量能未放大、突破20日高點</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>籌碼轉強</t>
+          <t>5日法人買超</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>短線偏強，站上5日線、成交量放大，可以列入觀察，但仍要注意是否追高。</t>
+          <t>強勢偏多：站上5日線、黃金交叉、量能未放大、突破20日高點、5日法人買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2374.TW</t>
+          <t>2609.TW</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>佳能</t>
+          <t>陽明</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>83.40000000000001</v>
+        <v>51.8</v>
       </c>
       <c r="D15" t="n">
-        <v>80.98</v>
+        <v>51.14</v>
       </c>
       <c r="E15" t="n">
-        <v>81.02</v>
+        <v>50.02</v>
       </c>
       <c r="F15" t="n">
-        <v>78.97</v>
+        <v>49.98</v>
       </c>
       <c r="G15" t="n">
-        <v>15239585</v>
+        <v>29869029</v>
       </c>
       <c r="H15" t="n">
-        <v>11366488</v>
+        <v>27481089</v>
       </c>
       <c r="I15" t="n">
-        <v>85.5</v>
+        <v>53.9</v>
       </c>
       <c r="J15" t="n">
-        <v>70.2</v>
+        <v>47.35</v>
       </c>
       <c r="K15" t="n">
-        <v>2000</v>
+        <v>-7838235</v>
       </c>
       <c r="L15" t="n">
-        <v>4000</v>
+        <v>21017772</v>
       </c>
       <c r="M15" t="n">
-        <v>6000</v>
+        <v>26241510</v>
       </c>
       <c r="N15" t="n">
-        <v>10000</v>
+        <v>-434219</v>
       </c>
       <c r="O15" t="n">
-        <v>60</v>
+        <v>85</v>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>👀觀察</t>
+          <t>🔥強勢</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -1568,73 +1568,73 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>站上5日線、成交量放大</t>
+          <t>站上5日線、多頭排列、量能溫和放大</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>籌碼轉強</t>
+          <t>5日法人明顯買超</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>短線偏強，站上5日線、成交量放大，可以列入觀察，但仍要注意是否追高。</t>
+          <t>強勢偏多：站上5日線、多頭排列、量能溫和放大、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2344.TW</t>
+          <t>3035.TW</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>華邦電</t>
+          <t>智原</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>125</v>
+        <v>218.5</v>
       </c>
       <c r="D16" t="n">
-        <v>120.5</v>
+        <v>203.1</v>
       </c>
       <c r="E16" t="n">
-        <v>122.7</v>
+        <v>199.95</v>
       </c>
       <c r="F16" t="n">
-        <v>110.54</v>
+        <v>189.05</v>
       </c>
       <c r="G16" t="n">
-        <v>190947918</v>
+        <v>30348381</v>
       </c>
       <c r="H16" t="n">
-        <v>184433553</v>
+        <v>20400910</v>
       </c>
       <c r="I16" t="n">
-        <v>136.5</v>
+        <v>231</v>
       </c>
       <c r="J16" t="n">
-        <v>84</v>
+        <v>167</v>
       </c>
       <c r="K16" t="n">
-        <v>2000</v>
+        <v>-1076740</v>
       </c>
       <c r="L16" t="n">
-        <v>5000</v>
+        <v>6371419</v>
       </c>
       <c r="M16" t="n">
-        <v>12000</v>
+        <v>6997630</v>
       </c>
       <c r="N16" t="n">
-        <v>15000</v>
+        <v>194327</v>
       </c>
       <c r="O16" t="n">
-        <v>60</v>
+        <v>85</v>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>👀觀察</t>
+          <t>🔥強勢</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -1644,73 +1644,73 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>站上5日線、成交量放大</t>
+          <t>站上5日線、多頭排列、量能溫和放大</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>籌碼轉強</t>
+          <t>5日法人明顯買超</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>短線偏強，站上5日線、成交量放大，可以列入觀察，但仍要注意是否追高。</t>
+          <t>強勢偏多：站上5日線、多頭排列、量能溫和放大、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2330.TW</t>
+          <t>2327.TW</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>台積電</t>
+          <t>國巨</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2255</v>
+        <v>317</v>
       </c>
       <c r="D17" t="n">
-        <v>2223</v>
+        <v>313.5</v>
       </c>
       <c r="E17" t="n">
-        <v>2236</v>
+        <v>313.7</v>
       </c>
       <c r="F17" t="n">
-        <v>2235.75</v>
+        <v>299.55</v>
       </c>
       <c r="G17" t="n">
-        <v>24437825</v>
+        <v>35517666</v>
       </c>
       <c r="H17" t="n">
-        <v>27484516</v>
+        <v>36150847</v>
       </c>
       <c r="I17" t="n">
-        <v>2345</v>
+        <v>336.5</v>
       </c>
       <c r="J17" t="n">
-        <v>2105</v>
+        <v>245</v>
       </c>
       <c r="K17" t="n">
-        <v>5000</v>
+        <v>2231528</v>
       </c>
       <c r="L17" t="n">
-        <v>12000</v>
+        <v>3889908</v>
       </c>
       <c r="M17" t="n">
-        <v>25000</v>
+        <v>9359269</v>
       </c>
       <c r="N17" t="n">
-        <v>40000</v>
+        <v>20009905</v>
       </c>
       <c r="O17" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>👀觀察</t>
+          <t>🔥強勢</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -1720,73 +1720,73 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>站上5日線、成交量未放大</t>
+          <t>站上5日線、量能未放大</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>籌碼轉強</t>
+          <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>短線偏強，站上5日線、成交量未放大，可以列入觀察，但仍要注意是否追高。</t>
+          <t>強勢偏多：站上5日線、量能未放大、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>3163.TWO</t>
+          <t>4958.TW</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>波若威</t>
+          <t>臻鼎-KY</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1145</v>
+        <v>529</v>
       </c>
       <c r="D18" t="n">
-        <v>988.4</v>
+        <v>472.4</v>
       </c>
       <c r="E18" t="n">
-        <v>1005.2</v>
+        <v>443.75</v>
       </c>
       <c r="F18" t="n">
-        <v>1060.6</v>
+        <v>425.25</v>
       </c>
       <c r="G18" t="n">
-        <v>3404797</v>
+        <v>47336484</v>
       </c>
       <c r="H18" t="n">
-        <v>1568233</v>
+        <v>50597809</v>
       </c>
       <c r="I18" t="n">
-        <v>1300</v>
+        <v>558</v>
       </c>
       <c r="J18" t="n">
-        <v>865</v>
+        <v>331</v>
       </c>
       <c r="K18" t="n">
-        <v>6000</v>
+        <v>-5716319</v>
       </c>
       <c r="L18" t="n">
-        <v>12000</v>
+        <v>-1491026</v>
       </c>
       <c r="M18" t="n">
-        <v>20000</v>
+        <v>13501619</v>
       </c>
       <c r="N18" t="n">
-        <v>30000</v>
+        <v>10633143</v>
       </c>
       <c r="O18" t="n">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>⚠️整理</t>
+          <t>🔥強勢</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -1796,290 +1796,294 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>站上5日線、空頭排列、超級爆量</t>
+          <t>站上5日線、多頭排列、量能未放大</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>籌碼轉強</t>
+          <t>5日法人明顯買超</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>短線偏強，站上5日線、空頭排列、超級爆量，可以列入觀察，但仍要注意是否追高。</t>
+          <t>強勢偏多：站上5日線、多頭排列、量能未放大、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>3105.TWO</t>
+          <t>2308.TW</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>穩懋</t>
+          <t>台達電</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>531</v>
+        <v>2290</v>
       </c>
       <c r="D19" t="n">
-        <v>473.5</v>
+        <v>2049</v>
       </c>
       <c r="E19" t="n">
-        <v>484.3</v>
+        <v>2085.5</v>
       </c>
       <c r="F19" t="n">
-        <v>499.57</v>
+        <v>2132.5</v>
       </c>
       <c r="G19" t="n">
-        <v>27582138</v>
+        <v>12049781</v>
       </c>
       <c r="H19" t="n">
-        <v>22972476</v>
+        <v>11885394</v>
       </c>
       <c r="I19" t="n">
-        <v>604</v>
+        <v>2370</v>
       </c>
       <c r="J19" t="n">
-        <v>436</v>
+        <v>1880</v>
       </c>
       <c r="K19" t="n">
-        <v>5000</v>
+        <v>4917556</v>
       </c>
       <c r="L19" t="n">
-        <v>10000</v>
+        <v>5273927</v>
       </c>
       <c r="M19" t="n">
-        <v>15000</v>
+        <v>1917848</v>
       </c>
       <c r="N19" t="n">
-        <v>20000</v>
+        <v>-4082627</v>
       </c>
       <c r="O19" t="n">
-        <v>35</v>
+        <v>65</v>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>⚠️整理</t>
+          <t>👀觀察</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>可追蹤</t>
+          <t>偏多觀察</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>站上5日線、空頭排列、成交量放大</t>
+          <t>站上5日線、空頭排列、量能溫和放大</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>籌碼轉強</t>
+          <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>目前有部分轉強訊號，站上5日線、空頭排列、成交量放大，可追蹤但不急著進場。</t>
+          <t>偏多觀察：站上5日線、空頭排列、量能溫和放大、法人連續偏買、5日法人明顯買超。條件不差，適合等待拉回或突破確認。</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>8046.TW</t>
+          <t>2374.TW</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>南電</t>
+          <t>佳能</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>934</v>
+        <v>83.7</v>
       </c>
       <c r="D20" t="n">
-        <v>844.8</v>
+        <v>81.23999999999999</v>
       </c>
       <c r="E20" t="n">
-        <v>854.5</v>
+        <v>81.34</v>
       </c>
       <c r="F20" t="n">
-        <v>895.45</v>
+        <v>79.59</v>
       </c>
       <c r="G20" t="n">
-        <v>16635783</v>
+        <v>11314147</v>
       </c>
       <c r="H20" t="n">
-        <v>13468721</v>
+        <v>10203164</v>
       </c>
       <c r="I20" t="n">
-        <v>1035</v>
+        <v>85.5</v>
       </c>
       <c r="J20" t="n">
-        <v>765</v>
+        <v>70.2</v>
       </c>
       <c r="K20" t="n">
-        <v>7000</v>
+        <v>-491799</v>
       </c>
       <c r="L20" t="n">
-        <v>15000</v>
+        <v>7106107</v>
       </c>
       <c r="M20" t="n">
-        <v>25000</v>
+        <v>4374099</v>
       </c>
       <c r="N20" t="n">
-        <v>35000</v>
+        <v>9626033</v>
       </c>
       <c r="O20" t="n">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>⚠️整理</t>
+          <t>👀觀察</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>可追蹤</t>
+          <t>偏多觀察</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>站上5日線、空頭排列、成交量放大</t>
+          <t>站上5日線、量能溫和放大</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>籌碼轉強</t>
+          <t>5日法人明顯買超</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>目前有部分轉強訊號，站上5日線、空頭排列、成交量放大，可追蹤但不急著進場。</t>
+          <t>偏多觀察：站上5日線、量能溫和放大、5日法人明顯買超。條件不差，適合等待拉回或突破確認。</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2408.TW</t>
+          <t>3105.TWO</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>南亞科</t>
+          <t>穩懋</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>310.5</v>
+        <v>543</v>
       </c>
       <c r="D21" t="n">
-        <v>291.6</v>
+        <v>492</v>
       </c>
       <c r="E21" t="n">
-        <v>305.35</v>
+        <v>486</v>
       </c>
       <c r="F21" t="n">
-        <v>275.52</v>
+        <v>499.38</v>
       </c>
       <c r="G21" t="n">
-        <v>154923679</v>
+        <v>42354000</v>
       </c>
       <c r="H21" t="n">
-        <v>131047919</v>
+        <v>28553600</v>
       </c>
       <c r="I21" t="n">
-        <v>353</v>
+        <v>566</v>
       </c>
       <c r="J21" t="n">
-        <v>199</v>
+        <v>436</v>
       </c>
       <c r="K21" t="n">
-        <v>-5000</v>
+        <v>-709786</v>
       </c>
       <c r="L21" t="n">
-        <v>-2000</v>
+        <v>7825302</v>
       </c>
       <c r="M21" t="n">
-        <v>3000</v>
+        <v>4382193</v>
       </c>
       <c r="N21" t="n">
-        <v>8000</v>
+        <v>-4637373</v>
       </c>
       <c r="O21" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>⚠️整理</t>
+          <t>👀觀察</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>可追蹤</t>
+          <t>偏多觀察</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>站上5日線、成交量放大</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr"/>
+          <t>站上5日線、量能溫和放大</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>5日法人明顯買超</t>
+        </is>
+      </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>目前有部分轉強訊號，站上5日線、成交量放大，可追蹤但不急著進場。</t>
+          <t>偏多觀察：站上5日線、量能溫和放大、5日法人明顯買超。條件不差，適合等待拉回或突破確認。</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>3481.TW</t>
+          <t>6669.TW</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>群創</t>
+          <t>緯穎</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>44.65</v>
+        <v>5610</v>
       </c>
       <c r="D22" t="n">
-        <v>39.67</v>
+        <v>5256</v>
       </c>
       <c r="E22" t="n">
-        <v>37.52</v>
+        <v>5329</v>
       </c>
       <c r="F22" t="n">
-        <v>31.72</v>
+        <v>5125.25</v>
       </c>
       <c r="G22" t="n">
-        <v>386510344</v>
+        <v>2115890</v>
       </c>
       <c r="H22" t="n">
-        <v>636475880</v>
+        <v>1971387</v>
       </c>
       <c r="I22" t="n">
-        <v>44.65</v>
+        <v>5880</v>
       </c>
       <c r="J22" t="n">
-        <v>22.95</v>
+        <v>4615</v>
       </c>
       <c r="K22" t="n">
-        <v>-71547</v>
+        <v>49559</v>
       </c>
       <c r="L22" t="n">
-        <v>-7378</v>
+        <v>97025</v>
       </c>
       <c r="M22" t="n">
-        <v>-219616</v>
+        <v>-160824</v>
       </c>
       <c r="N22" t="n">
-        <v>587508</v>
+        <v>-364679</v>
       </c>
       <c r="O22" t="n">
         <v>25</v>
@@ -2091,222 +2095,226 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>可追蹤</t>
+          <t>整理觀察</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>站上5日線、多頭排列、成交量未放大、突破20日高點</t>
+          <t>站上5日線、量能溫和放大</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>前期買超但短線轉弱、主力大賣</t>
+          <t>短線籌碼止穩、5日法人賣超</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>目前有部分轉強訊號，站上5日線、多頭排列、成交量未放大、突破20日高點，可追蹤但不急著進場。</t>
+          <t>整理觀察：站上5日線、量能溫和放大、短線籌碼止穩、5日法人賣超。多空訊號混合，建議降低追價衝動。</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>5289.TWO</t>
+          <t>2303.TW</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>宜鼎</t>
+          <t>聯電</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1725</v>
+        <v>125</v>
       </c>
       <c r="D23" t="n">
-        <v>1741</v>
+        <v>115.2</v>
       </c>
       <c r="E23" t="n">
-        <v>1765</v>
+        <v>110.79</v>
       </c>
       <c r="F23" t="n">
-        <v>1557.75</v>
+        <v>97.3</v>
       </c>
       <c r="G23" t="n">
-        <v>2948990</v>
+        <v>340935766</v>
       </c>
       <c r="H23" t="n">
-        <v>4147491</v>
+        <v>249027598</v>
       </c>
       <c r="I23" t="n">
-        <v>1935</v>
+        <v>125</v>
       </c>
       <c r="J23" t="n">
-        <v>1055</v>
+        <v>70.7</v>
       </c>
       <c r="K23" t="n">
-        <v>4000</v>
+        <v>32836623</v>
       </c>
       <c r="L23" t="n">
-        <v>8000</v>
+        <v>-1979065</v>
       </c>
       <c r="M23" t="n">
-        <v>12000</v>
+        <v>-21222223</v>
       </c>
       <c r="N23" t="n">
-        <v>18000</v>
+        <v>49323216</v>
       </c>
       <c r="O23" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>❌避開</t>
+          <t>⚠️整理</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>觀望</t>
+          <t>整理觀察</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>跌破5日線、成交量未放大</t>
+          <t>站上5日線、多頭排列、量能溫和放大、突破20日高點</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>籌碼轉強</t>
+          <t>中期買超轉短線賣壓、5日法人明顯賣超</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>訊號普通，跌破5日線、成交量未放大，目前方向不明，適合先觀察。</t>
+          <t>整理觀察：站上5日線、多頭排列、量能溫和放大、突破20日高點、中期買超轉短線賣壓、5日法人明顯賣超。多空訊號混合，建議降低追價衝動。</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>6488.TWO</t>
+          <t>2330.TW</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>環球晶</t>
+          <t>台積電</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>717</v>
+        <v>2310</v>
       </c>
       <c r="D24" t="n">
-        <v>683.8</v>
+        <v>2237</v>
       </c>
       <c r="E24" t="n">
-        <v>728.7</v>
+        <v>2243.5</v>
       </c>
       <c r="F24" t="n">
-        <v>688.65</v>
+        <v>2242</v>
       </c>
       <c r="G24" t="n">
-        <v>6305022</v>
+        <v>28250944</v>
       </c>
       <c r="H24" t="n">
-        <v>4509007</v>
+        <v>32784457</v>
       </c>
       <c r="I24" t="n">
-        <v>849</v>
+        <v>2345</v>
       </c>
       <c r="J24" t="n">
-        <v>534</v>
+        <v>2135</v>
       </c>
       <c r="K24" t="n">
-        <v>-3000</v>
+        <v>8271589</v>
       </c>
       <c r="L24" t="n">
-        <v>2000</v>
+        <v>10332214</v>
       </c>
       <c r="M24" t="n">
-        <v>12000</v>
+        <v>-12125572</v>
       </c>
       <c r="N24" t="n">
-        <v>30000</v>
+        <v>-16581218</v>
       </c>
       <c r="O24" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>❌避開</t>
+          <t>⚠️整理</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>觀望</t>
+          <t>整理觀察</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>站上5日線、死亡交叉、成交量放大</t>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr"/>
+          <t>站上5日線、量能未放大、接近20日高點</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>短線籌碼止穩、5日法人明顯賣超</t>
+        </is>
+      </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>訊號普通，站上5日線、死亡交叉、成交量放大，目前方向不明，適合先觀察。</t>
+          <t>整理觀察：站上5日線、量能未放大、接近20日高點、短線籌碼止穩、5日法人明顯賣超。多空訊號混合，建議降低追價衝動。</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2317.TW</t>
+          <t>6488.TWO</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>鴻海</t>
+          <t>環球晶</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>250</v>
+        <v>788</v>
       </c>
       <c r="D25" t="n">
-        <v>246.2</v>
+        <v>701.8</v>
       </c>
       <c r="E25" t="n">
-        <v>247.7</v>
+        <v>724</v>
       </c>
       <c r="F25" t="n">
-        <v>240.95</v>
+        <v>698.95</v>
       </c>
       <c r="G25" t="n">
-        <v>55061095</v>
+        <v>5700000</v>
       </c>
       <c r="H25" t="n">
-        <v>59202085</v>
+        <v>4980000</v>
       </c>
       <c r="I25" t="n">
-        <v>260</v>
+        <v>849</v>
       </c>
       <c r="J25" t="n">
-        <v>218</v>
+        <v>534</v>
       </c>
       <c r="K25" t="n">
-        <v>-3000</v>
+        <v>-261357</v>
       </c>
       <c r="L25" t="n">
-        <v>-8000</v>
+        <v>-3141303</v>
       </c>
       <c r="M25" t="n">
-        <v>-15000</v>
+        <v>-4610982</v>
       </c>
       <c r="N25" t="n">
-        <v>-20000</v>
+        <v>-4787133</v>
       </c>
       <c r="O25" t="n">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="P25" t="inlineStr">
         <is>
@@ -2315,74 +2323,74 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>避開</t>
+          <t>觀望</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>站上5日線、成交量未放大</t>
+          <t>站上5日線、黃金交叉、量能溫和放大</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>短線賣壓重</t>
+          <t>法人連續偏賣、5日法人明顯賣超</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>目前偏弱，站上5日線、成交量未放大，短線不建議急著進場。</t>
+          <t>風險偏高：站上5日線、黃金交叉、量能溫和放大、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1802.TW</t>
+          <t>6239.TW</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>台玻</t>
+          <t>力成</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>70.5</v>
+        <v>311</v>
       </c>
       <c r="D26" t="n">
-        <v>65.92</v>
+        <v>262.6</v>
       </c>
       <c r="E26" t="n">
-        <v>67.05</v>
+        <v>249.85</v>
       </c>
       <c r="F26" t="n">
-        <v>67.67</v>
+        <v>235.22</v>
       </c>
       <c r="G26" t="n">
-        <v>124473105</v>
+        <v>3433065</v>
       </c>
       <c r="H26" t="n">
-        <v>67843641</v>
+        <v>18105153</v>
       </c>
       <c r="I26" t="n">
-        <v>75.5</v>
+        <v>311</v>
       </c>
       <c r="J26" t="n">
-        <v>61.7</v>
+        <v>201</v>
       </c>
       <c r="K26" t="n">
-        <v>-3000</v>
+        <v>-1465366</v>
       </c>
       <c r="L26" t="n">
-        <v>-6000</v>
+        <v>-160620</v>
       </c>
       <c r="M26" t="n">
-        <v>-10000</v>
+        <v>-5984174</v>
       </c>
       <c r="N26" t="n">
-        <v>-15000</v>
+        <v>5074162</v>
       </c>
       <c r="O26" t="n">
-        <v>-15</v>
+        <v>-10</v>
       </c>
       <c r="P26" t="inlineStr">
         <is>
@@ -2391,98 +2399,554 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>避開</t>
+          <t>觀望</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>站上5日線、空頭排列、爆量</t>
+          <t>站上5日線、多頭排列、量能未放大、突破20日高點</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>短線賣壓重</t>
+          <t>法人連續偏賣、中期買超轉短線賣壓、5日法人明顯賣超</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>目前偏弱，站上5日線、空頭排列、爆量，短線不建議急著進場。</t>
+          <t>風險偏高：站上5日線、多頭排列、量能未放大、突破20日高點、法人連續偏賣、中期買超轉短線賣壓、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>3163.TWO</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>波若威</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1210</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1050.4</v>
+      </c>
+      <c r="E27" t="n">
+        <v>1022.2</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1063.35</v>
+      </c>
+      <c r="G27" t="n">
+        <v>7441000</v>
+      </c>
+      <c r="H27" t="n">
+        <v>2940200</v>
+      </c>
+      <c r="I27" t="n">
+        <v>1300</v>
+      </c>
+      <c r="J27" t="n">
+        <v>865</v>
+      </c>
+      <c r="K27" t="n">
+        <v>-1014980</v>
+      </c>
+      <c r="L27" t="n">
+        <v>-1037784</v>
+      </c>
+      <c r="M27" t="n">
+        <v>-1279466</v>
+      </c>
+      <c r="N27" t="n">
+        <v>-1723078</v>
+      </c>
+      <c r="O27" t="n">
+        <v>-15</v>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>❌避開</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>觀望</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>站上5日線、爆量</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>法人連續偏賣、5日法人明顯賣超</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>風險偏高：站上5日線、爆量、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>8046.TW</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>南電</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>884</v>
+      </c>
+      <c r="D28" t="n">
+        <v>863.4</v>
+      </c>
+      <c r="E28" t="n">
+        <v>852.1</v>
+      </c>
+      <c r="F28" t="n">
+        <v>895.95</v>
+      </c>
+      <c r="G28" t="n">
+        <v>30914905</v>
+      </c>
+      <c r="H28" t="n">
+        <v>17982182</v>
+      </c>
+      <c r="I28" t="n">
+        <v>1035</v>
+      </c>
+      <c r="J28" t="n">
+        <v>765</v>
+      </c>
+      <c r="K28" t="n">
+        <v>-8905954</v>
+      </c>
+      <c r="L28" t="n">
+        <v>-4812274</v>
+      </c>
+      <c r="M28" t="n">
+        <v>-4509560</v>
+      </c>
+      <c r="N28" t="n">
+        <v>-8787097</v>
+      </c>
+      <c r="O28" t="n">
+        <v>-20</v>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>❌避開</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>觀望</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>站上5日線、成交量放大</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>法人連續偏賣、5日法人明顯賣超</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>風險偏高：站上5日線、成交量放大、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2408.TW</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>南亞科</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>296</v>
+      </c>
+      <c r="D29" t="n">
+        <v>289.8</v>
+      </c>
+      <c r="E29" t="n">
+        <v>304.85</v>
+      </c>
+      <c r="F29" t="n">
+        <v>280.02</v>
+      </c>
+      <c r="G29" t="n">
+        <v>155862832</v>
+      </c>
+      <c r="H29" t="n">
+        <v>141256759</v>
+      </c>
+      <c r="I29" t="n">
+        <v>353</v>
+      </c>
+      <c r="J29" t="n">
+        <v>214.5</v>
+      </c>
+      <c r="K29" t="n">
+        <v>-13921163</v>
+      </c>
+      <c r="L29" t="n">
+        <v>-14185405</v>
+      </c>
+      <c r="M29" t="n">
+        <v>-47727411</v>
+      </c>
+      <c r="N29" t="n">
+        <v>-49157826</v>
+      </c>
+      <c r="O29" t="n">
+        <v>-25</v>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>❌避開</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>觀望</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>站上5日線、量能溫和放大</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>法人連續偏賣、5日法人明顯賣超</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>風險偏高：站上5日線、量能溫和放大、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>3481.TW</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>群創</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>23.95</v>
+      </c>
+      <c r="D30" t="n">
+        <v>23.99</v>
+      </c>
+      <c r="E30" t="n">
+        <v>24.77</v>
+      </c>
+      <c r="F30" t="n">
+        <v>25.45</v>
+      </c>
+      <c r="G30" t="n">
+        <v>103739940</v>
+      </c>
+      <c r="H30" t="n">
+        <v>172083654</v>
+      </c>
+      <c r="I30" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="J30" t="n">
+        <v>22.95</v>
+      </c>
+      <c r="K30" t="n">
+        <v>-2664727</v>
+      </c>
+      <c r="L30" t="n">
+        <v>121233278</v>
+      </c>
+      <c r="M30" t="n">
+        <v>74438491</v>
+      </c>
+      <c r="N30" t="n">
+        <v>153391454</v>
+      </c>
+      <c r="O30" t="n">
+        <v>-25</v>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>❌避開</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>觀望</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>跌破5日線、空頭排列、量能未放大、接近20日低點</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>5日法人明顯買超</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>風險偏高：跌破5日線、空頭排列、量能未放大、接近20日低點、5日法人明顯買超。目前不適合積極追蹤，等待結構改善。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>4960.TW</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>誠美材</t>
         </is>
       </c>
-      <c r="C27" t="n">
-        <v>35.8</v>
-      </c>
-      <c r="D27" t="n">
-        <v>34.69</v>
-      </c>
-      <c r="E27" t="n">
-        <v>35.36</v>
-      </c>
-      <c r="F27" t="n">
-        <v>37.68</v>
-      </c>
-      <c r="G27" t="n">
-        <v>25488550</v>
-      </c>
-      <c r="H27" t="n">
-        <v>17301029</v>
-      </c>
-      <c r="I27" t="n">
+      <c r="C31" t="n">
+        <v>36</v>
+      </c>
+      <c r="D31" t="n">
+        <v>35.19</v>
+      </c>
+      <c r="E31" t="n">
+        <v>34.98</v>
+      </c>
+      <c r="F31" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="G31" t="n">
+        <v>16699898</v>
+      </c>
+      <c r="H31" t="n">
+        <v>18191883</v>
+      </c>
+      <c r="I31" t="n">
         <v>44.05</v>
       </c>
-      <c r="J27" t="n">
+      <c r="J31" t="n">
         <v>31.1</v>
       </c>
-      <c r="K27" t="n">
-        <v>-5000</v>
-      </c>
-      <c r="L27" t="n">
-        <v>-10000</v>
-      </c>
-      <c r="M27" t="n">
-        <v>-15000</v>
-      </c>
-      <c r="N27" t="n">
-        <v>-25000</v>
-      </c>
-      <c r="O27" t="n">
-        <v>-20</v>
-      </c>
-      <c r="P27" t="inlineStr">
+      <c r="K31" t="n">
+        <v>-1669951</v>
+      </c>
+      <c r="L31" t="n">
+        <v>-4496950</v>
+      </c>
+      <c r="M31" t="n">
+        <v>-8242967</v>
+      </c>
+      <c r="N31" t="n">
+        <v>-5221995</v>
+      </c>
+      <c r="O31" t="n">
+        <v>-35</v>
+      </c>
+      <c r="P31" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="Q27" t="inlineStr">
-        <is>
-          <t>避開</t>
-        </is>
-      </c>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>站上5日線、空頭排列、成交量放大</t>
-        </is>
-      </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>短線賣壓重</t>
-        </is>
-      </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>目前偏弱，站上5日線、空頭排列、成交量放大，短線不建議急著進場。</t>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>觀望</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>站上5日線、量能未放大</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>法人連續偏賣、5日法人明顯賣超</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>風險偏高：站上5日線、量能未放大、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>6285.TW</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>啟碁</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>298</v>
+      </c>
+      <c r="D32" t="n">
+        <v>289.1</v>
+      </c>
+      <c r="E32" t="n">
+        <v>280.6</v>
+      </c>
+      <c r="F32" t="n">
+        <v>248.53</v>
+      </c>
+      <c r="G32" t="n">
+        <v>35285750</v>
+      </c>
+      <c r="H32" t="n">
+        <v>37916640</v>
+      </c>
+      <c r="I32" t="n">
+        <v>317</v>
+      </c>
+      <c r="J32" t="n">
+        <v>168</v>
+      </c>
+      <c r="K32" t="n">
+        <v>-5937776</v>
+      </c>
+      <c r="L32" t="n">
+        <v>-4853792</v>
+      </c>
+      <c r="M32" t="n">
+        <v>-11223101</v>
+      </c>
+      <c r="N32" t="n">
+        <v>1863302</v>
+      </c>
+      <c r="O32" t="n">
+        <v>-35</v>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>❌避開</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>觀望</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>站上5日線、多頭排列、量能未放大</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>法人連續偏賣、中期買超轉短線賣壓、5日法人明顯賣超</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>風險偏高：站上5日線、多頭排列、量能未放大、法人連續偏賣、中期買超轉短線賣壓、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>5289.TWO</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>宜鼎</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>1685</v>
+      </c>
+      <c r="D33" t="n">
+        <v>1705</v>
+      </c>
+      <c r="E33" t="n">
+        <v>1757.5</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1587.75</v>
+      </c>
+      <c r="G33" t="n">
+        <v>4686000</v>
+      </c>
+      <c r="H33" t="n">
+        <v>4122200</v>
+      </c>
+      <c r="I33" t="n">
+        <v>1935</v>
+      </c>
+      <c r="J33" t="n">
+        <v>1115</v>
+      </c>
+      <c r="K33" t="n">
+        <v>-352405</v>
+      </c>
+      <c r="L33" t="n">
+        <v>-707137</v>
+      </c>
+      <c r="M33" t="n">
+        <v>-868509</v>
+      </c>
+      <c r="N33" t="n">
+        <v>-2148559</v>
+      </c>
+      <c r="O33" t="n">
+        <v>-65</v>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>❌避開</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>觀望</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>跌破5日線、量能溫和放大</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>法人連續偏賣、5日法人明顯賣超</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>風險偏高：跌破5日線、量能溫和放大、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
add volume price anomaly signals
</commit_message>
<xml_diff>
--- a/output/stock_analysis_result.xlsx
+++ b/output/stock_analysis_result.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T33"/>
+  <dimension ref="A1:U33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,50 +469,55 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>量價異常</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>籌碼1日</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>籌碼3日</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>籌碼5日</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>籌碼10日</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>技術分數</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>狀態</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>綜合判斷</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>技術面</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>籌碼面</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>AI評語</t>
         </is>
@@ -521,456 +526,486 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2383.TW</t>
+          <t>2312.TW</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>台光電</t>
+          <t>金寶</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5505</v>
+        <v>40</v>
       </c>
       <c r="D2" t="n">
-        <v>4826</v>
+        <v>33.58</v>
       </c>
       <c r="E2" t="n">
-        <v>4804</v>
+        <v>30.93</v>
       </c>
       <c r="F2" t="n">
-        <v>4756.25</v>
+        <v>29.77</v>
       </c>
       <c r="G2" t="n">
-        <v>1801298</v>
+        <v>210267926</v>
       </c>
       <c r="H2" t="n">
-        <v>2244504</v>
+        <v>105612204</v>
       </c>
       <c r="I2" t="n">
-        <v>5505</v>
+        <v>40</v>
       </c>
       <c r="J2" t="n">
-        <v>4160</v>
-      </c>
-      <c r="K2" t="n">
-        <v>359818</v>
+        <v>26.65</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>帶量突破20日高點</t>
+        </is>
       </c>
       <c r="L2" t="n">
-        <v>1354542</v>
+        <v>10178504</v>
       </c>
       <c r="M2" t="n">
-        <v>1447903</v>
+        <v>70925202</v>
       </c>
       <c r="N2" t="n">
-        <v>2950399</v>
+        <v>76924762</v>
       </c>
       <c r="O2" t="n">
-        <v>155</v>
-      </c>
-      <c r="P2" t="inlineStr">
+        <v>66944449</v>
+      </c>
+      <c r="P2" t="n">
+        <v>170</v>
+      </c>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、黃金交叉、量能未放大、突破20日高點</t>
-        </is>
-      </c>
       <c r="S2" t="inlineStr">
         <is>
+          <t>站上5日線、多頭排列、成交量放大、突破20日高點、帶量突破20日高點</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
           <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、黃金交叉、量能未放大、突破20日高點、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、成交量放大、突破20日高點、帶量突破20日高點、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2317.TW</t>
+          <t>6116.TW</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>鴻海</t>
+          <t>彩晶</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>261</v>
+        <v>13.65</v>
       </c>
       <c r="D3" t="n">
-        <v>248.7</v>
+        <v>11.83</v>
       </c>
       <c r="E3" t="n">
-        <v>248.6</v>
+        <v>11.16</v>
       </c>
       <c r="F3" t="n">
-        <v>242.93</v>
+        <v>10.02</v>
       </c>
       <c r="G3" t="n">
-        <v>122990174</v>
+        <v>478320069</v>
       </c>
       <c r="H3" t="n">
-        <v>72731564</v>
+        <v>148294428</v>
       </c>
       <c r="I3" t="n">
-        <v>263.5</v>
+        <v>14.3</v>
       </c>
       <c r="J3" t="n">
-        <v>219.5</v>
-      </c>
-      <c r="K3" t="n">
-        <v>55787312</v>
+        <v>8.130000000000001</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>帶量突破20日高點</t>
+        </is>
       </c>
       <c r="L3" t="n">
-        <v>101690979</v>
+        <v>2108293</v>
       </c>
       <c r="M3" t="n">
-        <v>84630201</v>
+        <v>59515291</v>
       </c>
       <c r="N3" t="n">
-        <v>160089561</v>
+        <v>56282808</v>
       </c>
       <c r="O3" t="n">
-        <v>135</v>
-      </c>
-      <c r="P3" t="inlineStr">
+        <v>50628800</v>
+      </c>
+      <c r="P3" t="n">
+        <v>150</v>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、成交量放大、接近20日高點</t>
-        </is>
-      </c>
       <c r="S3" t="inlineStr">
         <is>
+          <t>站上5日線、多頭排列、爆量、帶量突破20日高點</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
           <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、成交量放大、接近20日高點、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、爆量、帶量突破20日高點、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>6116.TW</t>
+          <t>3189.TW</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>彩晶</t>
+          <t>景碩</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>13</v>
+        <v>696</v>
       </c>
       <c r="D4" t="n">
-        <v>11.13</v>
+        <v>606.4</v>
       </c>
       <c r="E4" t="n">
-        <v>10.86</v>
+        <v>555.55</v>
       </c>
       <c r="F4" t="n">
-        <v>9.75</v>
+        <v>529.38</v>
       </c>
       <c r="G4" t="n">
-        <v>43724582</v>
+        <v>50429815</v>
       </c>
       <c r="H4" t="n">
-        <v>60470183</v>
+        <v>29094105</v>
       </c>
       <c r="I4" t="n">
-        <v>13</v>
+        <v>719</v>
       </c>
       <c r="J4" t="n">
-        <v>8.119999999999999</v>
-      </c>
-      <c r="K4" t="n">
-        <v>2108293</v>
+        <v>445.5</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>帶量突破20日高點</t>
+        </is>
       </c>
       <c r="L4" t="n">
-        <v>59515291</v>
+        <v>964619</v>
       </c>
       <c r="M4" t="n">
-        <v>56282808</v>
+        <v>17496756</v>
       </c>
       <c r="N4" t="n">
-        <v>50628800</v>
+        <v>19603616</v>
       </c>
       <c r="O4" t="n">
-        <v>130</v>
-      </c>
-      <c r="P4" t="inlineStr">
+        <v>18095930</v>
+      </c>
+      <c r="P4" t="n">
+        <v>145</v>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、量能未放大、突破20日高點</t>
-        </is>
-      </c>
       <c r="S4" t="inlineStr">
         <is>
+          <t>站上5日線、多頭排列、成交量放大、帶量突破20日高點</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
           <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、量能未放大、突破20日高點、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、成交量放大、帶量突破20日高點、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2409.TW</t>
+          <t>3037.TW</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>友達</t>
+          <t>欣興</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>24.4</v>
+        <v>1085</v>
       </c>
       <c r="D5" t="n">
-        <v>20.94</v>
+        <v>954.6</v>
       </c>
       <c r="E5" t="n">
-        <v>20.35</v>
+        <v>900.1</v>
       </c>
       <c r="F5" t="n">
-        <v>19.02</v>
+        <v>881.7</v>
       </c>
       <c r="G5" t="n">
-        <v>82302936</v>
+        <v>34270461</v>
       </c>
       <c r="H5" t="n">
-        <v>230537458</v>
+        <v>30958709</v>
       </c>
       <c r="I5" t="n">
-        <v>24.4</v>
+        <v>1085</v>
       </c>
       <c r="J5" t="n">
-        <v>16.6</v>
-      </c>
-      <c r="K5" t="n">
-        <v>18947923</v>
+        <v>776</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>無明顯異常</t>
+        </is>
       </c>
       <c r="L5" t="n">
-        <v>211604454</v>
+        <v>1191293</v>
       </c>
       <c r="M5" t="n">
-        <v>192942642</v>
+        <v>14796086</v>
       </c>
       <c r="N5" t="n">
-        <v>353520387</v>
+        <v>14042095</v>
       </c>
       <c r="O5" t="n">
-        <v>130</v>
-      </c>
-      <c r="P5" t="inlineStr">
+        <v>12040296</v>
+      </c>
+      <c r="P5" t="n">
+        <v>140</v>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、量能未放大、突破20日高點</t>
-        </is>
-      </c>
       <c r="S5" t="inlineStr">
         <is>
+          <t>站上5日線、多頭排列、量能溫和放大、突破20日高點</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
           <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、量能未放大、突破20日高點、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、量能溫和放大、突破20日高點、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2312.TW</t>
+          <t>2317.TW</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>金寶</t>
+          <t>鴻海</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>36.4</v>
+        <v>259</v>
       </c>
       <c r="D6" t="n">
-        <v>31.13</v>
+        <v>251.5</v>
       </c>
       <c r="E6" t="n">
-        <v>29.88</v>
+        <v>249.5</v>
       </c>
       <c r="F6" t="n">
-        <v>29.14</v>
+        <v>244.47</v>
       </c>
       <c r="G6" t="n">
-        <v>66663284</v>
+        <v>55665305</v>
       </c>
       <c r="H6" t="n">
-        <v>67343380</v>
+        <v>69819957</v>
       </c>
       <c r="I6" t="n">
-        <v>36.4</v>
+        <v>263.5</v>
       </c>
       <c r="J6" t="n">
-        <v>25.45</v>
-      </c>
-      <c r="K6" t="n">
-        <v>10178504</v>
+        <v>219.5</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>無明顯異常</t>
+        </is>
       </c>
       <c r="L6" t="n">
-        <v>70925202</v>
+        <v>55787312</v>
       </c>
       <c r="M6" t="n">
-        <v>76924762</v>
+        <v>101690979</v>
       </c>
       <c r="N6" t="n">
-        <v>66944449</v>
+        <v>84630201</v>
       </c>
       <c r="O6" t="n">
-        <v>130</v>
-      </c>
-      <c r="P6" t="inlineStr">
+        <v>160089561</v>
+      </c>
+      <c r="P6" t="n">
+        <v>120</v>
+      </c>
+      <c r="Q6" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、量能未放大、突破20日高點</t>
-        </is>
-      </c>
       <c r="S6" t="inlineStr">
         <is>
+          <t>站上5日線、多頭排列、量能未放大、接近20日高點</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
           <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、量能未放大、突破20日高點、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、量能未放大、接近20日高點、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>3189.TW</t>
+          <t>2383.TW</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>景碩</t>
+          <t>台光電</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>669</v>
+        <v>5290</v>
       </c>
       <c r="D7" t="n">
-        <v>569.8</v>
+        <v>4977</v>
       </c>
       <c r="E7" t="n">
-        <v>535.35</v>
+        <v>4843</v>
       </c>
       <c r="F7" t="n">
-        <v>520.33</v>
+        <v>4784.25</v>
       </c>
       <c r="G7" t="n">
-        <v>8536899</v>
+        <v>2917258</v>
       </c>
       <c r="H7" t="n">
-        <v>26502334</v>
+        <v>2443800</v>
       </c>
       <c r="I7" t="n">
-        <v>669</v>
+        <v>5635</v>
       </c>
       <c r="J7" t="n">
-        <v>445.5</v>
-      </c>
-      <c r="K7" t="n">
-        <v>964619</v>
+        <v>4160</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>無明顯異常</t>
+        </is>
       </c>
       <c r="L7" t="n">
-        <v>17496756</v>
+        <v>359818</v>
       </c>
       <c r="M7" t="n">
-        <v>19603616</v>
+        <v>1354542</v>
       </c>
       <c r="N7" t="n">
-        <v>18095930</v>
+        <v>1447903</v>
       </c>
       <c r="O7" t="n">
-        <v>130</v>
-      </c>
-      <c r="P7" t="inlineStr">
+        <v>2950399</v>
+      </c>
+      <c r="P7" t="n">
+        <v>115</v>
+      </c>
+      <c r="Q7" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="R7" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、量能未放大、突破20日高點</t>
-        </is>
-      </c>
       <c r="S7" t="inlineStr">
         <is>
+          <t>站上5日線、多頭排列、量能溫和放大</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
           <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、量能未放大、突破20日高點、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、量能溫和放大、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
@@ -986,141 +1021,151 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>57.1</v>
+        <v>55.4</v>
       </c>
       <c r="D8" t="n">
-        <v>52.56</v>
+        <v>53.91</v>
       </c>
       <c r="E8" t="n">
-        <v>50.76</v>
+        <v>51.25</v>
       </c>
       <c r="F8" t="n">
-        <v>50.01</v>
+        <v>50.42</v>
       </c>
       <c r="G8" t="n">
-        <v>16550566</v>
+        <v>15723414</v>
       </c>
       <c r="H8" t="n">
-        <v>8831247</v>
+        <v>11255762</v>
       </c>
       <c r="I8" t="n">
-        <v>58.5</v>
+        <v>60.3</v>
       </c>
       <c r="J8" t="n">
         <v>45.45</v>
       </c>
-      <c r="K8" t="n">
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>無明顯異常</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
         <v>3454745</v>
       </c>
-      <c r="L8" t="n">
+      <c r="M8" t="n">
         <v>13009409</v>
       </c>
-      <c r="M8" t="n">
+      <c r="N8" t="n">
         <v>14246624</v>
       </c>
-      <c r="N8" t="n">
+      <c r="O8" t="n">
         <v>12266815</v>
       </c>
-      <c r="O8" t="n">
-        <v>120</v>
-      </c>
-      <c r="P8" t="inlineStr">
+      <c r="P8" t="n">
+        <v>115</v>
+      </c>
+      <c r="Q8" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr">
+      <c r="R8" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、成交量放大</t>
-        </is>
-      </c>
       <c r="S8" t="inlineStr">
         <is>
+          <t>站上5日線、多頭排列、量能溫和放大</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
           <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、成交量放大、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、量能溫和放大、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>6274.TWO</t>
+          <t>2344.TW</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>台燿</t>
+          <t>華邦電</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1600</v>
+        <v>141</v>
       </c>
       <c r="D9" t="n">
-        <v>1362</v>
+        <v>124.8</v>
       </c>
       <c r="E9" t="n">
-        <v>1372.5</v>
+        <v>125.75</v>
       </c>
       <c r="F9" t="n">
-        <v>1279.05</v>
+        <v>114.91</v>
       </c>
       <c r="G9" t="n">
-        <v>1486000</v>
+        <v>336105421</v>
       </c>
       <c r="H9" t="n">
-        <v>1401800</v>
+        <v>249474700</v>
       </c>
       <c r="I9" t="n">
-        <v>1600</v>
+        <v>141</v>
       </c>
       <c r="J9" t="n">
-        <v>941</v>
-      </c>
-      <c r="K9" t="n">
-        <v>282254</v>
+        <v>88.8</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>無明顯異常</t>
+        </is>
       </c>
       <c r="L9" t="n">
-        <v>969253</v>
+        <v>77651903</v>
       </c>
       <c r="M9" t="n">
-        <v>1221688</v>
+        <v>96687402</v>
       </c>
       <c r="N9" t="n">
-        <v>2123947</v>
+        <v>61728965</v>
       </c>
       <c r="O9" t="n">
+        <v>182119556</v>
+      </c>
+      <c r="P9" t="n">
         <v>115</v>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr">
+      <c r="R9" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="S9" t="inlineStr">
         <is>
           <t>站上5日線、量能溫和放大、突破20日高點</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>強勢偏多：站上5日線、量能溫和放大、突破20日高點、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
@@ -1129,74 +1174,79 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>3037.TW</t>
+          <t>8358.TWO</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>欣興</t>
+          <t>金居</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>990</v>
+        <v>533</v>
       </c>
       <c r="D10" t="n">
-        <v>901.2</v>
+        <v>511.6</v>
       </c>
       <c r="E10" t="n">
-        <v>879.1</v>
+        <v>468.75</v>
       </c>
       <c r="F10" t="n">
-        <v>869.4</v>
+        <v>448.2</v>
       </c>
       <c r="G10" t="n">
-        <v>24465071</v>
+        <v>2520000</v>
       </c>
       <c r="H10" t="n">
-        <v>28813042</v>
+        <v>4413800</v>
       </c>
       <c r="I10" t="n">
-        <v>1030</v>
+        <v>558</v>
       </c>
       <c r="J10" t="n">
-        <v>776</v>
-      </c>
-      <c r="K10" t="n">
-        <v>1191293</v>
+        <v>340</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>無明顯異常</t>
+        </is>
       </c>
       <c r="L10" t="n">
-        <v>14796086</v>
+        <v>434414</v>
       </c>
       <c r="M10" t="n">
-        <v>14042095</v>
+        <v>4299788</v>
       </c>
       <c r="N10" t="n">
-        <v>12040296</v>
+        <v>9649180</v>
       </c>
       <c r="O10" t="n">
+        <v>9535283</v>
+      </c>
+      <c r="P10" t="n">
         <v>105</v>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="Q10" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr">
+      <c r="R10" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="S10" t="inlineStr">
         <is>
           <t>站上5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>強勢偏多：站上5日線、多頭排列、量能未放大、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
@@ -1205,152 +1255,162 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>8358.TWO</t>
+          <t>6274.TWO</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>金居</t>
+          <t>台燿</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>545</v>
+        <v>1580</v>
       </c>
       <c r="D11" t="n">
-        <v>490.8</v>
+        <v>1433</v>
       </c>
       <c r="E11" t="n">
-        <v>463.15</v>
+        <v>1385.5</v>
       </c>
       <c r="F11" t="n">
-        <v>438.32</v>
+        <v>1308.55</v>
       </c>
       <c r="G11" t="n">
-        <v>2767000</v>
+        <v>9546000</v>
       </c>
       <c r="H11" t="n">
-        <v>4459600</v>
+        <v>3017800</v>
       </c>
       <c r="I11" t="n">
-        <v>558</v>
+        <v>1700</v>
       </c>
       <c r="J11" t="n">
-        <v>324.5</v>
-      </c>
-      <c r="K11" t="n">
-        <v>434414</v>
+        <v>941</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>爆量價未漲</t>
+        </is>
       </c>
       <c r="L11" t="n">
-        <v>4299788</v>
+        <v>282254</v>
       </c>
       <c r="M11" t="n">
-        <v>9649180</v>
+        <v>969253</v>
       </c>
       <c r="N11" t="n">
-        <v>9535283</v>
+        <v>1221688</v>
       </c>
       <c r="O11" t="n">
+        <v>2123947</v>
+      </c>
+      <c r="P11" t="n">
         <v>105</v>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="Q11" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr">
+      <c r="R11" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、量能未放大</t>
-        </is>
-      </c>
       <c r="S11" t="inlineStr">
         <is>
+          <t>站上5日線、多頭排列、爆量、爆量價未漲</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
           <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、量能未放大、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、爆量、爆量價未漲、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2344.TW</t>
+          <t>2327.TW</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>華邦電</t>
+          <t>國巨</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>128.5</v>
+        <v>661</v>
       </c>
       <c r="D12" t="n">
-        <v>120.1</v>
+        <v>614.6</v>
       </c>
       <c r="E12" t="n">
-        <v>123.8</v>
+        <v>540.85</v>
       </c>
       <c r="F12" t="n">
-        <v>117.83</v>
+        <v>448.73</v>
       </c>
       <c r="G12" t="n">
-        <v>357612926</v>
+        <v>29457930</v>
       </c>
       <c r="H12" t="n">
-        <v>219239775</v>
+        <v>56139070</v>
       </c>
       <c r="I12" t="n">
-        <v>136.5</v>
+        <v>691</v>
       </c>
       <c r="J12" t="n">
-        <v>91.09999999999999</v>
-      </c>
-      <c r="K12" t="n">
-        <v>77651903</v>
+        <v>307</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>無明顯異常</t>
+        </is>
       </c>
       <c r="L12" t="n">
-        <v>96687402</v>
+        <v>2231528</v>
       </c>
       <c r="M12" t="n">
-        <v>61728965</v>
+        <v>3889908</v>
       </c>
       <c r="N12" t="n">
-        <v>182119556</v>
+        <v>9359269</v>
       </c>
       <c r="O12" t="n">
-        <v>95</v>
-      </c>
-      <c r="P12" t="inlineStr">
+        <v>20009905</v>
+      </c>
+      <c r="P12" t="n">
+        <v>105</v>
+      </c>
+      <c r="Q12" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr">
+      <c r="R12" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>站上5日線、成交量放大</t>
-        </is>
-      </c>
       <c r="S12" t="inlineStr">
         <is>
+          <t>站上5日線、多頭排列、量能未放大</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
           <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、成交量放大、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、量能未放大、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
@@ -1366,903 +1426,963 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>73.90000000000001</v>
+        <v>72.2</v>
       </c>
       <c r="D13" t="n">
-        <v>67.73999999999999</v>
+        <v>69.12</v>
       </c>
       <c r="E13" t="n">
-        <v>67.45</v>
+        <v>67.56</v>
       </c>
       <c r="F13" t="n">
-        <v>68.11</v>
+        <v>68.52</v>
       </c>
       <c r="G13" t="n">
-        <v>185285181</v>
+        <v>337055872</v>
       </c>
       <c r="H13" t="n">
-        <v>96433207</v>
+        <v>147844553</v>
       </c>
       <c r="I13" t="n">
-        <v>76.8</v>
+        <v>81.2</v>
       </c>
       <c r="J13" t="n">
-        <v>61.7</v>
-      </c>
-      <c r="K13" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>爆量價未漲</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
         <v>44538498</v>
       </c>
-      <c r="L13" t="n">
+      <c r="M13" t="n">
         <v>88202486</v>
       </c>
-      <c r="M13" t="n">
+      <c r="N13" t="n">
         <v>75247740</v>
       </c>
-      <c r="N13" t="n">
+      <c r="O13" t="n">
         <v>32596649</v>
       </c>
-      <c r="O13" t="n">
-        <v>95</v>
-      </c>
-      <c r="P13" t="inlineStr">
+      <c r="P13" t="n">
+        <v>105</v>
+      </c>
+      <c r="Q13" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr">
+      <c r="R13" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>站上5日線、成交量放大</t>
-        </is>
-      </c>
       <c r="S13" t="inlineStr">
         <is>
+          <t>站上5日線、黃金交叉、爆量、爆量價未漲</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
           <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、成交量放大、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、黃金交叉、爆量、爆量價未漲、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>3711.TW</t>
+          <t>2409.TW</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>日月光投控</t>
+          <t>友達</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>617</v>
+        <v>22</v>
       </c>
       <c r="D14" t="n">
-        <v>527.2</v>
+        <v>21.51</v>
       </c>
       <c r="E14" t="n">
-        <v>534.4</v>
+        <v>20.48</v>
       </c>
       <c r="F14" t="n">
-        <v>523.17</v>
+        <v>19.25</v>
       </c>
       <c r="G14" t="n">
-        <v>26609382</v>
+        <v>818361725</v>
       </c>
       <c r="H14" t="n">
-        <v>28063686</v>
+        <v>356215638</v>
       </c>
       <c r="I14" t="n">
-        <v>617</v>
+        <v>25.8</v>
       </c>
       <c r="J14" t="n">
-        <v>465</v>
-      </c>
-      <c r="K14" t="n">
-        <v>-1946569</v>
+        <v>16.6</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>爆量價未漲</t>
+        </is>
       </c>
       <c r="L14" t="n">
-        <v>4398628</v>
+        <v>18947923</v>
       </c>
       <c r="M14" t="n">
-        <v>375095</v>
+        <v>211604454</v>
       </c>
       <c r="N14" t="n">
-        <v>-4267040</v>
+        <v>192942642</v>
       </c>
       <c r="O14" t="n">
-        <v>90</v>
-      </c>
-      <c r="P14" t="inlineStr">
+        <v>353520387</v>
+      </c>
+      <c r="P14" t="n">
+        <v>105</v>
+      </c>
+      <c r="Q14" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr">
+      <c r="R14" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>站上5日線、黃金交叉、量能未放大、突破20日高點</t>
-        </is>
-      </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>5日法人買超</t>
+          <t>站上5日線、多頭排列、爆量、爆量價未漲</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>強勢偏多：站上5日線、黃金交叉、量能未放大、突破20日高點、5日法人買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+          <t>法人連續偏買、5日法人明顯買超</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、爆量、爆量價未漲、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2609.TW</t>
+          <t>3105.TWO</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>陽明</t>
+          <t>穩懋</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>51.8</v>
+        <v>562</v>
       </c>
       <c r="D15" t="n">
-        <v>51.14</v>
+        <v>513.1</v>
       </c>
       <c r="E15" t="n">
-        <v>50.02</v>
+        <v>491</v>
       </c>
       <c r="F15" t="n">
-        <v>49.98</v>
+        <v>502.85</v>
       </c>
       <c r="G15" t="n">
-        <v>29869029</v>
+        <v>33746000</v>
       </c>
       <c r="H15" t="n">
-        <v>27481089</v>
+        <v>31597000</v>
       </c>
       <c r="I15" t="n">
-        <v>53.9</v>
+        <v>566</v>
       </c>
       <c r="J15" t="n">
-        <v>47.35</v>
-      </c>
-      <c r="K15" t="n">
-        <v>-7838235</v>
+        <v>436</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>無明顯異常</t>
+        </is>
       </c>
       <c r="L15" t="n">
-        <v>21017772</v>
+        <v>-709786</v>
       </c>
       <c r="M15" t="n">
-        <v>26241510</v>
+        <v>7825302</v>
       </c>
       <c r="N15" t="n">
-        <v>-434219</v>
+        <v>4382193</v>
       </c>
       <c r="O15" t="n">
-        <v>85</v>
-      </c>
-      <c r="P15" t="inlineStr">
+        <v>-4637373</v>
+      </c>
+      <c r="P15" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q15" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr">
+      <c r="R15" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、量能溫和放大</t>
-        </is>
-      </c>
       <c r="S15" t="inlineStr">
         <is>
+          <t>站上5日線、黃金交叉、量能溫和放大、接近20日高點</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
           <t>5日法人明顯買超</t>
         </is>
       </c>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、量能溫和放大、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、黃金交叉、量能溫和放大、接近20日高點、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>3035.TW</t>
+          <t>2308.TW</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>智原</t>
+          <t>台達電</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>218.5</v>
+        <v>2350</v>
       </c>
       <c r="D16" t="n">
-        <v>203.1</v>
+        <v>2136</v>
       </c>
       <c r="E16" t="n">
-        <v>199.95</v>
+        <v>2101</v>
       </c>
       <c r="F16" t="n">
-        <v>189.05</v>
+        <v>2149</v>
       </c>
       <c r="G16" t="n">
-        <v>30348381</v>
+        <v>12198582</v>
       </c>
       <c r="H16" t="n">
-        <v>20400910</v>
+        <v>11067330</v>
       </c>
       <c r="I16" t="n">
-        <v>231</v>
+        <v>2410</v>
       </c>
       <c r="J16" t="n">
-        <v>167</v>
-      </c>
-      <c r="K16" t="n">
-        <v>-1076740</v>
+        <v>1880</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>無明顯異常</t>
+        </is>
       </c>
       <c r="L16" t="n">
-        <v>6371419</v>
+        <v>4917556</v>
       </c>
       <c r="M16" t="n">
-        <v>6997630</v>
+        <v>5273927</v>
       </c>
       <c r="N16" t="n">
-        <v>194327</v>
+        <v>1917848</v>
       </c>
       <c r="O16" t="n">
-        <v>85</v>
-      </c>
-      <c r="P16" t="inlineStr">
+        <v>-4082627</v>
+      </c>
+      <c r="P16" t="n">
+        <v>90</v>
+      </c>
+      <c r="Q16" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr">
+      <c r="R16" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、量能溫和放大</t>
-        </is>
-      </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>5日法人明顯買超</t>
+          <t>站上5日線、量能溫和放大</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>強勢偏多：站上5日線、多頭排列、量能溫和放大、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+          <t>法人連續偏買、5日法人明顯買超</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、量能溫和放大、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2327.TW</t>
+          <t>2374.TW</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>國巨</t>
+          <t>佳能</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>317</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="D17" t="n">
-        <v>313.5</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="E17" t="n">
-        <v>313.7</v>
+        <v>81.34</v>
       </c>
       <c r="F17" t="n">
-        <v>299.55</v>
+        <v>80.16</v>
       </c>
       <c r="G17" t="n">
-        <v>35517666</v>
+        <v>12463968</v>
       </c>
       <c r="H17" t="n">
-        <v>36150847</v>
+        <v>10197116</v>
       </c>
       <c r="I17" t="n">
-        <v>336.5</v>
+        <v>85.8</v>
       </c>
       <c r="J17" t="n">
-        <v>245</v>
-      </c>
-      <c r="K17" t="n">
-        <v>2231528</v>
+        <v>70.2</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>無明顯異常</t>
+        </is>
       </c>
       <c r="L17" t="n">
-        <v>3889908</v>
+        <v>-491799</v>
       </c>
       <c r="M17" t="n">
-        <v>9359269</v>
+        <v>7106107</v>
       </c>
       <c r="N17" t="n">
-        <v>20009905</v>
+        <v>4374099</v>
       </c>
       <c r="O17" t="n">
-        <v>80</v>
-      </c>
-      <c r="P17" t="inlineStr">
+        <v>9626033</v>
+      </c>
+      <c r="P17" t="n">
+        <v>85</v>
+      </c>
+      <c r="Q17" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr">
+      <c r="R17" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>站上5日線、量能未放大</t>
-        </is>
-      </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>法人連續偏買、5日法人明顯買超</t>
+          <t>站上5日線、多頭排列、量能溫和放大</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>強勢偏多：站上5日線、量能未放大、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+          <t>5日法人明顯買超</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、量能溫和放大、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>4958.TW</t>
+          <t>3711.TW</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>臻鼎-KY</t>
+          <t>日月光投控</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>529</v>
+        <v>611</v>
       </c>
       <c r="D18" t="n">
-        <v>472.4</v>
+        <v>555</v>
       </c>
       <c r="E18" t="n">
-        <v>443.75</v>
+        <v>540</v>
       </c>
       <c r="F18" t="n">
-        <v>425.25</v>
+        <v>528.95</v>
       </c>
       <c r="G18" t="n">
-        <v>47336484</v>
+        <v>39627497</v>
       </c>
       <c r="H18" t="n">
-        <v>50597809</v>
+        <v>28597065</v>
       </c>
       <c r="I18" t="n">
-        <v>558</v>
+        <v>636</v>
       </c>
       <c r="J18" t="n">
-        <v>331</v>
-      </c>
-      <c r="K18" t="n">
-        <v>-5716319</v>
+        <v>465</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>無明顯異常</t>
+        </is>
       </c>
       <c r="L18" t="n">
-        <v>-1491026</v>
+        <v>-1946569</v>
       </c>
       <c r="M18" t="n">
-        <v>13501619</v>
+        <v>4398628</v>
       </c>
       <c r="N18" t="n">
-        <v>10633143</v>
+        <v>375095</v>
       </c>
       <c r="O18" t="n">
+        <v>-4267040</v>
+      </c>
+      <c r="P18" t="n">
         <v>75</v>
       </c>
-      <c r="P18" t="inlineStr">
+      <c r="Q18" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr">
+      <c r="R18" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、量能未放大</t>
-        </is>
-      </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>5日法人明顯買超</t>
+          <t>站上5日線、多頭排列、量能溫和放大</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>強勢偏多：站上5日線、多頭排列、量能未放大、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+          <t>5日法人買超</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、量能溫和放大、5日法人買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2308.TW</t>
+          <t>3481.TW</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>台達電</t>
+          <t>群創</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2290</v>
+        <v>45.7</v>
       </c>
       <c r="D19" t="n">
-        <v>2049</v>
+        <v>43.4</v>
       </c>
       <c r="E19" t="n">
-        <v>2085.5</v>
+        <v>40.22</v>
       </c>
       <c r="F19" t="n">
-        <v>2132.5</v>
+        <v>34.08</v>
       </c>
       <c r="G19" t="n">
-        <v>12049781</v>
+        <v>1463227218</v>
       </c>
       <c r="H19" t="n">
-        <v>11885394</v>
+        <v>613882104</v>
       </c>
       <c r="I19" t="n">
-        <v>2370</v>
+        <v>52.2</v>
       </c>
       <c r="J19" t="n">
-        <v>1880</v>
-      </c>
-      <c r="K19" t="n">
-        <v>4917556</v>
+        <v>23.65</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>爆量價未漲</t>
+        </is>
       </c>
       <c r="L19" t="n">
-        <v>5273927</v>
+        <v>-2664727</v>
       </c>
       <c r="M19" t="n">
-        <v>1917848</v>
+        <v>121233278</v>
       </c>
       <c r="N19" t="n">
-        <v>-4082627</v>
+        <v>74438491</v>
       </c>
       <c r="O19" t="n">
-        <v>65</v>
-      </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>👀觀察</t>
-        </is>
+        <v>153391454</v>
+      </c>
+      <c r="P19" t="n">
+        <v>75</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>偏多觀察</t>
+          <t>🔥強勢</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>站上5日線、空頭排列、量能溫和放大</t>
+          <t>強勢觀察</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>法人連續偏買、5日法人明顯買超</t>
+          <t>站上5日線、多頭排列、爆量、爆量價未漲</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>偏多觀察：站上5日線、空頭排列、量能溫和放大、法人連續偏買、5日法人明顯買超。條件不差，適合等待拉回或突破確認。</t>
+          <t>5日法人明顯買超</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、爆量、爆量價未漲、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2374.TW</t>
+          <t>4958.TW</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>佳能</t>
+          <t>臻鼎-KY</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>83.7</v>
+        <v>540</v>
       </c>
       <c r="D20" t="n">
-        <v>81.23999999999999</v>
+        <v>498.7</v>
       </c>
       <c r="E20" t="n">
-        <v>81.34</v>
+        <v>457.05</v>
       </c>
       <c r="F20" t="n">
-        <v>79.59</v>
+        <v>434.32</v>
       </c>
       <c r="G20" t="n">
-        <v>11314147</v>
+        <v>41904053</v>
       </c>
       <c r="H20" t="n">
-        <v>10203164</v>
+        <v>51443369</v>
       </c>
       <c r="I20" t="n">
-        <v>85.5</v>
+        <v>558</v>
       </c>
       <c r="J20" t="n">
-        <v>70.2</v>
-      </c>
-      <c r="K20" t="n">
-        <v>-491799</v>
+        <v>354</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>無明顯異常</t>
+        </is>
       </c>
       <c r="L20" t="n">
-        <v>7106107</v>
+        <v>-5716319</v>
       </c>
       <c r="M20" t="n">
-        <v>4374099</v>
+        <v>-1491026</v>
       </c>
       <c r="N20" t="n">
-        <v>9626033</v>
+        <v>13501619</v>
       </c>
       <c r="O20" t="n">
-        <v>60</v>
-      </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>👀觀察</t>
-        </is>
+        <v>10633143</v>
+      </c>
+      <c r="P20" t="n">
+        <v>75</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>偏多觀察</t>
+          <t>🔥強勢</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>站上5日線、量能溫和放大</t>
+          <t>強勢觀察</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
+          <t>站上5日線、多頭排列、量能未放大</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
           <t>5日法人明顯買超</t>
         </is>
       </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>偏多觀察：站上5日線、量能溫和放大、5日法人明顯買超。條件不差，適合等待拉回或突破確認。</t>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、量能未放大、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>3105.TWO</t>
+          <t>2609.TW</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>穩懋</t>
+          <t>陽明</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>543</v>
+        <v>52</v>
       </c>
       <c r="D21" t="n">
-        <v>492</v>
+        <v>51.64</v>
       </c>
       <c r="E21" t="n">
-        <v>486</v>
+        <v>50.21</v>
       </c>
       <c r="F21" t="n">
-        <v>499.38</v>
+        <v>50.11</v>
       </c>
       <c r="G21" t="n">
-        <v>42354000</v>
+        <v>14910096</v>
       </c>
       <c r="H21" t="n">
-        <v>28553600</v>
+        <v>26622786</v>
       </c>
       <c r="I21" t="n">
-        <v>566</v>
+        <v>53.9</v>
       </c>
       <c r="J21" t="n">
-        <v>436</v>
-      </c>
-      <c r="K21" t="n">
-        <v>-709786</v>
+        <v>47.35</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>無明顯異常</t>
+        </is>
       </c>
       <c r="L21" t="n">
-        <v>7825302</v>
+        <v>-7838235</v>
       </c>
       <c r="M21" t="n">
-        <v>4382193</v>
+        <v>21017772</v>
       </c>
       <c r="N21" t="n">
-        <v>-4637373</v>
+        <v>26241510</v>
       </c>
       <c r="O21" t="n">
-        <v>60</v>
-      </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>👀觀察</t>
-        </is>
+        <v>-434219</v>
+      </c>
+      <c r="P21" t="n">
+        <v>75</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>偏多觀察</t>
+          <t>🔥強勢</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>站上5日線、量能溫和放大</t>
+          <t>強勢觀察</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
+          <t>站上5日線、多頭排列、量能未放大</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
           <t>5日法人明顯買超</t>
         </is>
       </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>偏多觀察：站上5日線、量能溫和放大、5日法人明顯買超。條件不差，適合等待拉回或突破確認。</t>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、量能未放大、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>6669.TW</t>
+          <t>3035.TW</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>緯穎</t>
+          <t>智原</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>5610</v>
+        <v>208</v>
       </c>
       <c r="D22" t="n">
-        <v>5256</v>
+        <v>207</v>
       </c>
       <c r="E22" t="n">
-        <v>5329</v>
+        <v>199.9</v>
       </c>
       <c r="F22" t="n">
-        <v>5125.25</v>
+        <v>190.12</v>
       </c>
       <c r="G22" t="n">
-        <v>2115890</v>
+        <v>20600438</v>
       </c>
       <c r="H22" t="n">
-        <v>1971387</v>
+        <v>22454689</v>
       </c>
       <c r="I22" t="n">
-        <v>5880</v>
+        <v>231</v>
       </c>
       <c r="J22" t="n">
-        <v>4615</v>
-      </c>
-      <c r="K22" t="n">
-        <v>49559</v>
+        <v>167</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>無明顯異常</t>
+        </is>
       </c>
       <c r="L22" t="n">
-        <v>97025</v>
+        <v>-1076740</v>
       </c>
       <c r="M22" t="n">
-        <v>-160824</v>
+        <v>6371419</v>
       </c>
       <c r="N22" t="n">
-        <v>-364679</v>
+        <v>6997630</v>
       </c>
       <c r="O22" t="n">
-        <v>25</v>
-      </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>⚠️整理</t>
-        </is>
+        <v>194327</v>
+      </c>
+      <c r="P22" t="n">
+        <v>75</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>整理觀察</t>
+          <t>🔥強勢</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>站上5日線、量能溫和放大</t>
+          <t>強勢觀察</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>短線籌碼止穩、5日法人賣超</t>
+          <t>站上5日線、多頭排列、量能未放大</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>整理觀察：站上5日線、量能溫和放大、短線籌碼止穩、5日法人賣超。多空訊號混合，建議降低追價衝動。</t>
+          <t>5日法人明顯買超</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、量能未放大、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2303.TW</t>
+          <t>2330.TW</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>聯電</t>
+          <t>台積電</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>125</v>
+        <v>2270</v>
       </c>
       <c r="D23" t="n">
-        <v>115.2</v>
+        <v>2250</v>
       </c>
       <c r="E23" t="n">
-        <v>110.79</v>
+        <v>2245</v>
       </c>
       <c r="F23" t="n">
-        <v>97.3</v>
+        <v>2242.25</v>
       </c>
       <c r="G23" t="n">
-        <v>340935766</v>
+        <v>32781470</v>
       </c>
       <c r="H23" t="n">
-        <v>249027598</v>
+        <v>30223565</v>
       </c>
       <c r="I23" t="n">
-        <v>125</v>
+        <v>2345</v>
       </c>
       <c r="J23" t="n">
-        <v>70.7</v>
-      </c>
-      <c r="K23" t="n">
-        <v>32836623</v>
+        <v>2135</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>無明顯異常</t>
+        </is>
       </c>
       <c r="L23" t="n">
-        <v>-1979065</v>
+        <v>8271589</v>
       </c>
       <c r="M23" t="n">
-        <v>-21222223</v>
+        <v>10332214</v>
       </c>
       <c r="N23" t="n">
-        <v>49323216</v>
+        <v>-12125572</v>
       </c>
       <c r="O23" t="n">
-        <v>25</v>
-      </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>⚠️整理</t>
-        </is>
+        <v>-16581218</v>
+      </c>
+      <c r="P23" t="n">
+        <v>65</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>整理觀察</t>
+          <t>👀觀察</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>站上5日線、多頭排列、量能溫和放大、突破20日高點</t>
+          <t>偏多觀察</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>中期買超轉短線賣壓、5日法人明顯賣超</t>
+          <t>站上5日線、多頭排列、黃金交叉、量能溫和放大</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>整理觀察：站上5日線、多頭排列、量能溫和放大、突破20日高點、中期買超轉短線賣壓、5日法人明顯賣超。多空訊號混合，建議降低追價衝動。</t>
+          <t>短線籌碼止穩、5日法人明顯賣超</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>偏多觀察：站上5日線、多頭排列、黃金交叉、量能溫和放大、短線籌碼止穩、5日法人明顯賣超。條件不差，適合等待拉回或突破確認。</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2330.TW</t>
+          <t>6239.TW</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>台積電</t>
+          <t>力成</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2310</v>
+        <v>342</v>
       </c>
       <c r="D24" t="n">
-        <v>2237</v>
+        <v>285.6</v>
       </c>
       <c r="E24" t="n">
-        <v>2243.5</v>
+        <v>261.4</v>
       </c>
       <c r="F24" t="n">
-        <v>2242</v>
+        <v>241.47</v>
       </c>
       <c r="G24" t="n">
-        <v>28250944</v>
+        <v>57938700</v>
       </c>
       <c r="H24" t="n">
-        <v>32784457</v>
+        <v>22861322</v>
       </c>
       <c r="I24" t="n">
-        <v>2345</v>
+        <v>342</v>
       </c>
       <c r="J24" t="n">
-        <v>2135</v>
-      </c>
-      <c r="K24" t="n">
-        <v>8271589</v>
+        <v>201</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>帶量突破20日高點</t>
+        </is>
       </c>
       <c r="L24" t="n">
-        <v>10332214</v>
+        <v>-1465366</v>
       </c>
       <c r="M24" t="n">
-        <v>-12125572</v>
+        <v>-160620</v>
       </c>
       <c r="N24" t="n">
-        <v>-16581218</v>
+        <v>-5984174</v>
       </c>
       <c r="O24" t="n">
-        <v>20</v>
-      </c>
-      <c r="P24" t="inlineStr">
+        <v>5074162</v>
+      </c>
+      <c r="P24" t="n">
+        <v>35</v>
+      </c>
+      <c r="Q24" t="inlineStr">
         <is>
           <t>⚠️整理</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr">
+      <c r="R24" t="inlineStr">
         <is>
           <t>整理觀察</t>
         </is>
       </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>站上5日線、量能未放大、接近20日高點</t>
-        </is>
-      </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>短線籌碼止穩、5日法人明顯賣超</t>
+          <t>站上5日線、多頭排列、爆量、突破20日高點、帶量突破20日高點</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>整理觀察：站上5日線、量能未放大、接近20日高點、短線籌碼止穩、5日法人明顯賣超。多空訊號混合，建議降低追價衝動。</t>
+          <t>法人連續偏賣、中期買超轉短線賣壓、5日法人明顯賣超</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>整理觀察：站上5日線、多頭排列、爆量、突破20日高點、帶量突破20日高點、法人連續偏賣、中期買超轉短線賣壓、5日法人明顯賣超。多空訊號混合，建議降低追價衝動。</t>
         </is>
       </c>
     </row>
@@ -2278,143 +2398,153 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>788</v>
+        <v>866</v>
       </c>
       <c r="D25" t="n">
-        <v>701.8</v>
+        <v>742</v>
       </c>
       <c r="E25" t="n">
-        <v>724</v>
+        <v>732.1</v>
       </c>
       <c r="F25" t="n">
-        <v>698.95</v>
+        <v>711.25</v>
       </c>
       <c r="G25" t="n">
-        <v>5700000</v>
+        <v>2958000</v>
       </c>
       <c r="H25" t="n">
-        <v>4980000</v>
+        <v>4678000</v>
       </c>
       <c r="I25" t="n">
-        <v>849</v>
+        <v>866</v>
       </c>
       <c r="J25" t="n">
         <v>534</v>
       </c>
-      <c r="K25" t="n">
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>無明顯異常</t>
+        </is>
+      </c>
+      <c r="L25" t="n">
         <v>-261357</v>
       </c>
-      <c r="L25" t="n">
+      <c r="M25" t="n">
         <v>-3141303</v>
       </c>
-      <c r="M25" t="n">
+      <c r="N25" t="n">
         <v>-4610982</v>
       </c>
-      <c r="N25" t="n">
+      <c r="O25" t="n">
         <v>-4787133</v>
       </c>
-      <c r="O25" t="n">
-        <v>0</v>
-      </c>
-      <c r="P25" t="inlineStr">
+      <c r="P25" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q25" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="Q25" t="inlineStr">
+      <c r="R25" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>站上5日線、黃金交叉、量能溫和放大</t>
-        </is>
-      </c>
       <c r="S25" t="inlineStr">
         <is>
+          <t>站上5日線、多頭排列、量能未放大、突破20日高點</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
           <t>法人連續偏賣、5日法人明顯賣超</t>
         </is>
       </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t>風險偏高：站上5日線、黃金交叉、量能溫和放大、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>風險偏高：站上5日線、多頭排列、量能未放大、突破20日高點、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>6239.TW</t>
+          <t>6669.TW</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>力成</t>
+          <t>緯穎</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>311</v>
+        <v>5280</v>
       </c>
       <c r="D26" t="n">
-        <v>262.6</v>
+        <v>5334</v>
       </c>
       <c r="E26" t="n">
-        <v>249.85</v>
+        <v>5278</v>
       </c>
       <c r="F26" t="n">
-        <v>235.22</v>
+        <v>5144.75</v>
       </c>
       <c r="G26" t="n">
-        <v>3433065</v>
+        <v>2655826</v>
       </c>
       <c r="H26" t="n">
-        <v>18105153</v>
+        <v>2172103</v>
       </c>
       <c r="I26" t="n">
-        <v>311</v>
+        <v>5880</v>
       </c>
       <c r="J26" t="n">
-        <v>201</v>
-      </c>
-      <c r="K26" t="n">
-        <v>-1465366</v>
+        <v>4615</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>無明顯異常</t>
+        </is>
       </c>
       <c r="L26" t="n">
-        <v>-160620</v>
+        <v>49559</v>
       </c>
       <c r="M26" t="n">
-        <v>-5984174</v>
+        <v>97025</v>
       </c>
       <c r="N26" t="n">
-        <v>5074162</v>
+        <v>-160824</v>
       </c>
       <c r="O26" t="n">
-        <v>-10</v>
-      </c>
-      <c r="P26" t="inlineStr">
+        <v>-364679</v>
+      </c>
+      <c r="P26" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q26" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="Q26" t="inlineStr">
+      <c r="R26" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、量能未放大、突破20日高點</t>
-        </is>
-      </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>法人連續偏賣、中期買超轉短線賣壓、5日法人明顯賣超</t>
+          <t>跌破5日線、多頭排列、量能溫和放大</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>風險偏高：站上5日線、多頭排列、量能未放大、突破20日高點、法人連續偏賣、中期買超轉短線賣壓、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
+          <t>短線籌碼止穩、5日法人賣超</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>風險偏高：跌破5日線、多頭排列、量能溫和放大、短線籌碼止穩、5日法人賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
@@ -2430,22 +2560,22 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1210</v>
+        <v>1220</v>
       </c>
       <c r="D27" t="n">
-        <v>1050.4</v>
+        <v>1114.4</v>
       </c>
       <c r="E27" t="n">
-        <v>1022.2</v>
+        <v>1037.7</v>
       </c>
       <c r="F27" t="n">
-        <v>1063.35</v>
+        <v>1072.35</v>
       </c>
       <c r="G27" t="n">
-        <v>7441000</v>
+        <v>4415000</v>
       </c>
       <c r="H27" t="n">
-        <v>2940200</v>
+        <v>3736800</v>
       </c>
       <c r="I27" t="n">
         <v>1300</v>
@@ -2453,120 +2583,130 @@
       <c r="J27" t="n">
         <v>865</v>
       </c>
-      <c r="K27" t="n">
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>無明顯異常</t>
+        </is>
+      </c>
+      <c r="L27" t="n">
         <v>-1014980</v>
       </c>
-      <c r="L27" t="n">
+      <c r="M27" t="n">
         <v>-1037784</v>
       </c>
-      <c r="M27" t="n">
+      <c r="N27" t="n">
         <v>-1279466</v>
       </c>
-      <c r="N27" t="n">
+      <c r="O27" t="n">
         <v>-1723078</v>
       </c>
-      <c r="O27" t="n">
-        <v>-15</v>
-      </c>
-      <c r="P27" t="inlineStr">
+      <c r="P27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="Q27" t="inlineStr">
+      <c r="R27" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>站上5日線、爆量</t>
-        </is>
-      </c>
       <c r="S27" t="inlineStr">
         <is>
+          <t>站上5日線、黃金交叉、量能溫和放大</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
           <t>法人連續偏賣、5日法人明顯賣超</t>
         </is>
       </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>風險偏高：站上5日線、爆量、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>風險偏高：站上5日線、黃金交叉、量能溫和放大、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>8046.TW</t>
+          <t>2303.TW</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>南電</t>
+          <t>聯電</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>884</v>
+        <v>130.5</v>
       </c>
       <c r="D28" t="n">
-        <v>863.4</v>
+        <v>118.7</v>
       </c>
       <c r="E28" t="n">
-        <v>852.1</v>
+        <v>113.39</v>
       </c>
       <c r="F28" t="n">
-        <v>895.95</v>
+        <v>100.19</v>
       </c>
       <c r="G28" t="n">
-        <v>30914905</v>
+        <v>291896012</v>
       </c>
       <c r="H28" t="n">
-        <v>17982182</v>
+        <v>252641517</v>
       </c>
       <c r="I28" t="n">
-        <v>1035</v>
+        <v>133.5</v>
       </c>
       <c r="J28" t="n">
-        <v>765</v>
-      </c>
-      <c r="K28" t="n">
-        <v>-8905954</v>
+        <v>71.3</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>無明顯異常</t>
+        </is>
       </c>
       <c r="L28" t="n">
-        <v>-4812274</v>
+        <v>32836623</v>
       </c>
       <c r="M28" t="n">
-        <v>-4509560</v>
+        <v>-1979065</v>
       </c>
       <c r="N28" t="n">
-        <v>-8787097</v>
+        <v>-21222223</v>
       </c>
       <c r="O28" t="n">
-        <v>-20</v>
-      </c>
-      <c r="P28" t="inlineStr">
+        <v>49323216</v>
+      </c>
+      <c r="P28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="Q28" t="inlineStr">
+      <c r="R28" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>站上5日線、成交量放大</t>
-        </is>
-      </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>法人連續偏賣、5日法人明顯賣超</t>
+          <t>站上5日線、多頭排列、量能溫和放大</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>風險偏高：站上5日線、成交量放大、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
+          <t>中期買超轉短線賣壓、5日法人明顯賣超</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>風險偏高：站上5日線、多頭排列、量能溫和放大、中期買超轉短線賣壓、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
@@ -2582,22 +2722,22 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>296</v>
+        <v>303.5</v>
       </c>
       <c r="D29" t="n">
-        <v>289.8</v>
+        <v>295.6</v>
       </c>
       <c r="E29" t="n">
-        <v>304.85</v>
+        <v>303.1</v>
       </c>
       <c r="F29" t="n">
-        <v>280.02</v>
+        <v>283.88</v>
       </c>
       <c r="G29" t="n">
-        <v>155862832</v>
+        <v>152949355</v>
       </c>
       <c r="H29" t="n">
-        <v>141256759</v>
+        <v>148065232</v>
       </c>
       <c r="I29" t="n">
         <v>353</v>
@@ -2605,42 +2745,47 @@
       <c r="J29" t="n">
         <v>214.5</v>
       </c>
-      <c r="K29" t="n">
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>無明顯異常</t>
+        </is>
+      </c>
+      <c r="L29" t="n">
         <v>-13921163</v>
       </c>
-      <c r="L29" t="n">
+      <c r="M29" t="n">
         <v>-14185405</v>
       </c>
-      <c r="M29" t="n">
+      <c r="N29" t="n">
         <v>-47727411</v>
       </c>
-      <c r="N29" t="n">
+      <c r="O29" t="n">
         <v>-49157826</v>
       </c>
-      <c r="O29" t="n">
+      <c r="P29" t="n">
         <v>-25</v>
       </c>
-      <c r="P29" t="inlineStr">
+      <c r="Q29" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="Q29" t="inlineStr">
+      <c r="R29" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="R29" t="inlineStr">
+      <c r="S29" t="inlineStr">
         <is>
           <t>站上5日線、量能溫和放大</t>
         </is>
       </c>
-      <c r="S29" t="inlineStr">
+      <c r="T29" t="inlineStr">
         <is>
           <t>法人連續偏賣、5日法人明顯賣超</t>
         </is>
       </c>
-      <c r="T29" t="inlineStr">
+      <c r="U29" t="inlineStr">
         <is>
           <t>風險偏高：站上5日線、量能溫和放大、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -2649,228 +2794,243 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>3481.TW</t>
+          <t>8046.TW</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>群創</t>
+          <t>南電</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>23.95</v>
+        <v>922</v>
       </c>
       <c r="D30" t="n">
-        <v>23.99</v>
+        <v>888.2</v>
       </c>
       <c r="E30" t="n">
-        <v>24.77</v>
+        <v>854.3</v>
       </c>
       <c r="F30" t="n">
-        <v>25.45</v>
+        <v>896.4</v>
       </c>
       <c r="G30" t="n">
-        <v>103739940</v>
+        <v>24438087</v>
       </c>
       <c r="H30" t="n">
-        <v>172083654</v>
+        <v>20893593</v>
       </c>
       <c r="I30" t="n">
-        <v>28.9</v>
+        <v>1035</v>
       </c>
       <c r="J30" t="n">
-        <v>22.95</v>
-      </c>
-      <c r="K30" t="n">
-        <v>-2664727</v>
+        <v>765</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>無明顯異常</t>
+        </is>
       </c>
       <c r="L30" t="n">
-        <v>121233278</v>
+        <v>-8905954</v>
       </c>
       <c r="M30" t="n">
-        <v>74438491</v>
+        <v>-4812274</v>
       </c>
       <c r="N30" t="n">
-        <v>153391454</v>
+        <v>-4509560</v>
       </c>
       <c r="O30" t="n">
+        <v>-8787097</v>
+      </c>
+      <c r="P30" t="n">
         <v>-25</v>
       </c>
-      <c r="P30" t="inlineStr">
+      <c r="Q30" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="Q30" t="inlineStr">
+      <c r="R30" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>跌破5日線、空頭排列、量能未放大、接近20日低點</t>
-        </is>
-      </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>5日法人明顯買超</t>
+          <t>站上5日線、量能溫和放大</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>風險偏高：跌破5日線、空頭排列、量能未放大、接近20日低點、5日法人明顯買超。目前不適合積極追蹤，等待結構改善。</t>
+          <t>法人連續偏賣、5日法人明顯賣超</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>風險偏高：站上5日線、量能溫和放大、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>4960.TW</t>
+          <t>6285.TW</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>誠美材</t>
+          <t>啟碁</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>36</v>
+        <v>304.5</v>
       </c>
       <c r="D31" t="n">
-        <v>35.19</v>
+        <v>291.6</v>
       </c>
       <c r="E31" t="n">
-        <v>34.98</v>
+        <v>282.85</v>
       </c>
       <c r="F31" t="n">
-        <v>37.5</v>
+        <v>260.6</v>
       </c>
       <c r="G31" t="n">
-        <v>16699898</v>
+        <v>21738108</v>
       </c>
       <c r="H31" t="n">
-        <v>18191883</v>
+        <v>31212343</v>
       </c>
       <c r="I31" t="n">
-        <v>44.05</v>
+        <v>317</v>
       </c>
       <c r="J31" t="n">
-        <v>31.1</v>
-      </c>
-      <c r="K31" t="n">
-        <v>-1669951</v>
+        <v>208.5</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>無明顯異常</t>
+        </is>
       </c>
       <c r="L31" t="n">
-        <v>-4496950</v>
+        <v>-5937776</v>
       </c>
       <c r="M31" t="n">
-        <v>-8242967</v>
+        <v>-4853792</v>
       </c>
       <c r="N31" t="n">
-        <v>-5221995</v>
+        <v>-11223101</v>
       </c>
       <c r="O31" t="n">
+        <v>1863302</v>
+      </c>
+      <c r="P31" t="n">
         <v>-35</v>
       </c>
-      <c r="P31" t="inlineStr">
+      <c r="Q31" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="Q31" t="inlineStr">
+      <c r="R31" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="R31" t="inlineStr">
-        <is>
-          <t>站上5日線、量能未放大</t>
-        </is>
-      </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>法人連續偏賣、5日法人明顯賣超</t>
+          <t>站上5日線、多頭排列、量能未放大</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>風險偏高：站上5日線、量能未放大、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
+          <t>法人連續偏賣、中期買超轉短線賣壓、5日法人明顯賣超</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>風險偏高：站上5日線、多頭排列、量能未放大、法人連續偏賣、中期買超轉短線賣壓、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>6285.TW</t>
+          <t>4960.TW</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>啟碁</t>
+          <t>誠美材</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>298</v>
+        <v>34.25</v>
       </c>
       <c r="D32" t="n">
-        <v>289.1</v>
+        <v>35.13</v>
       </c>
       <c r="E32" t="n">
-        <v>280.6</v>
+        <v>34.6</v>
       </c>
       <c r="F32" t="n">
-        <v>248.53</v>
+        <v>37.35</v>
       </c>
       <c r="G32" t="n">
-        <v>35285750</v>
+        <v>11138430</v>
       </c>
       <c r="H32" t="n">
-        <v>37916640</v>
+        <v>16177150</v>
       </c>
       <c r="I32" t="n">
-        <v>317</v>
+        <v>44.05</v>
       </c>
       <c r="J32" t="n">
-        <v>168</v>
-      </c>
-      <c r="K32" t="n">
-        <v>-5937776</v>
+        <v>31.1</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>無明顯異常</t>
+        </is>
       </c>
       <c r="L32" t="n">
-        <v>-4853792</v>
+        <v>-1669951</v>
       </c>
       <c r="M32" t="n">
-        <v>-11223101</v>
+        <v>-4496950</v>
       </c>
       <c r="N32" t="n">
-        <v>1863302</v>
+        <v>-8242967</v>
       </c>
       <c r="O32" t="n">
-        <v>-35</v>
-      </c>
-      <c r="P32" t="inlineStr">
+        <v>-5221995</v>
+      </c>
+      <c r="P32" t="n">
+        <v>-75</v>
+      </c>
+      <c r="Q32" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="Q32" t="inlineStr">
+      <c r="R32" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、量能未放大</t>
-        </is>
-      </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>法人連續偏賣、中期買超轉短線賣壓、5日法人明顯賣超</t>
+          <t>跌破5日線、量能未放大</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>風險偏高：站上5日線、多頭排列、量能未放大、法人連續偏賣、中期買超轉短線賣壓、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
+          <t>法人連續偏賣、5日法人明顯賣超</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>風險偏高：跌破5日線、量能未放大、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
@@ -2886,67 +3046,72 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1685</v>
+        <v>1690</v>
       </c>
       <c r="D33" t="n">
-        <v>1705</v>
+        <v>1697</v>
       </c>
       <c r="E33" t="n">
-        <v>1757.5</v>
+        <v>1747</v>
       </c>
       <c r="F33" t="n">
-        <v>1587.75</v>
+        <v>1612.75</v>
       </c>
       <c r="G33" t="n">
-        <v>4686000</v>
+        <v>3178000</v>
       </c>
       <c r="H33" t="n">
-        <v>4122200</v>
+        <v>3603600</v>
       </c>
       <c r="I33" t="n">
         <v>1935</v>
       </c>
       <c r="J33" t="n">
-        <v>1115</v>
-      </c>
-      <c r="K33" t="n">
+        <v>1190</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>無明顯異常</t>
+        </is>
+      </c>
+      <c r="L33" t="n">
         <v>-352405</v>
       </c>
-      <c r="L33" t="n">
+      <c r="M33" t="n">
         <v>-707137</v>
       </c>
-      <c r="M33" t="n">
+      <c r="N33" t="n">
         <v>-868509</v>
       </c>
-      <c r="N33" t="n">
+      <c r="O33" t="n">
         <v>-2148559</v>
       </c>
-      <c r="O33" t="n">
-        <v>-65</v>
-      </c>
-      <c r="P33" t="inlineStr">
+      <c r="P33" t="n">
+        <v>-75</v>
+      </c>
+      <c r="Q33" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="Q33" t="inlineStr">
+      <c r="R33" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>跌破5日線、量能溫和放大</t>
-        </is>
-      </c>
       <c r="S33" t="inlineStr">
         <is>
+          <t>跌破5日線、量能未放大</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
           <t>法人連續偏賣、5日法人明顯賣超</t>
         </is>
       </c>
-      <c r="T33" t="inlineStr">
-        <is>
-          <t>風險偏高：跌破5日線、量能溫和放大、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>風險偏高：跌破5日線、量能未放大、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
split institutional chip signals
</commit_message>
<xml_diff>
--- a/output/stock_analysis_result.xlsx
+++ b/output/stock_analysis_result.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U33"/>
+  <dimension ref="A1:AG33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -494,30 +494,90 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>外資1日</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>外資3日</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>外資5日</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>外資10日</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>投信1日</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>投信3日</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>投信5日</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>投信10日</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>自營商1日</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>自營商3日</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>自營商5日</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>自營商10日</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
           <t>技術分數</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>狀態</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>綜合判斷</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>技術面</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>籌碼面</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>AI評語</t>
         </is>
@@ -564,80 +624,116 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>10178504</v>
+        <v>3713763</v>
       </c>
       <c r="M2" t="n">
-        <v>70925202</v>
+        <v>19615583</v>
       </c>
       <c r="N2" t="n">
-        <v>76924762</v>
+        <v>68174224</v>
       </c>
       <c r="O2" t="n">
-        <v>66944449</v>
+        <v>70505841</v>
       </c>
       <c r="P2" t="n">
+        <v>3559089</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>22504498</v>
+      </c>
+      <c r="R2" t="n">
+        <v>72623387</v>
+      </c>
+      <c r="S2" t="n">
+        <v>76471865</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" t="n">
+        <v>-4063000</v>
+      </c>
+      <c r="V2" t="n">
+        <v>-7036000</v>
+      </c>
+      <c r="W2" t="n">
+        <v>-7676000</v>
+      </c>
+      <c r="X2" t="n">
+        <v>154674</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>1174085</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>2586837</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>1709976</v>
+      </c>
+      <c r="AB2" t="n">
         <v>170</v>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="AE2" t="inlineStr">
         <is>
           <t>站上5日線、多頭排列、成交量放大、突破20日高點、帶量突破20日高點</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>法人連續偏買、5日法人明顯買超</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、成交量放大、突破20日高點、帶量突破20日高點、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>法人連續偏買、5日法人明顯買超、外資買投信賣</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、成交量放大、突破20日高點、帶量突破20日高點、法人連續偏買、5日法人明顯買超、外資買投信賣。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>6116.TW</t>
+          <t>3189.TW</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>彩晶</t>
+          <t>景碩</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>13.65</v>
+        <v>696</v>
       </c>
       <c r="D3" t="n">
-        <v>11.83</v>
+        <v>606.4</v>
       </c>
       <c r="E3" t="n">
-        <v>11.16</v>
+        <v>555.55</v>
       </c>
       <c r="F3" t="n">
-        <v>10.02</v>
+        <v>529.38</v>
       </c>
       <c r="G3" t="n">
-        <v>478320069</v>
+        <v>50429815</v>
       </c>
       <c r="H3" t="n">
-        <v>148294428</v>
+        <v>29094105</v>
       </c>
       <c r="I3" t="n">
-        <v>14.3</v>
+        <v>719</v>
       </c>
       <c r="J3" t="n">
-        <v>8.130000000000001</v>
+        <v>445.5</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -645,161 +741,233 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>2108293</v>
+        <v>1039882</v>
       </c>
       <c r="M3" t="n">
-        <v>59515291</v>
+        <v>2873236</v>
       </c>
       <c r="N3" t="n">
-        <v>56282808</v>
+        <v>18611901</v>
       </c>
       <c r="O3" t="n">
-        <v>50628800</v>
+        <v>20676322</v>
       </c>
       <c r="P3" t="n">
-        <v>150</v>
-      </c>
-      <c r="Q3" t="inlineStr">
+        <v>17922</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>1412705</v>
+      </c>
+      <c r="R3" t="n">
+        <v>13349743</v>
+      </c>
+      <c r="S3" t="n">
+        <v>13948306</v>
+      </c>
+      <c r="T3" t="n">
+        <v>613000</v>
+      </c>
+      <c r="U3" t="n">
+        <v>1197000</v>
+      </c>
+      <c r="V3" t="n">
+        <v>3587000</v>
+      </c>
+      <c r="W3" t="n">
+        <v>3764897</v>
+      </c>
+      <c r="X3" t="n">
+        <v>408960</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>263531</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>1675158</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>2963119</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>165</v>
+      </c>
+      <c r="AC3" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="AD3" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、爆量、帶量突破20日高點</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>法人連續偏買、5日法人明顯買超</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、爆量、帶量突破20日高點、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>站上5日線、多頭排列、成交量放大、帶量突破20日高點</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>法人連續偏買、5日法人明顯買超、外資投信同步買超</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、成交量放大、帶量突破20日高點、法人連續偏買、5日法人明顯買超、外資投信同步買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>3189.TW</t>
+          <t>3037.TW</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>景碩</t>
+          <t>欣興</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>696</v>
+        <v>1085</v>
       </c>
       <c r="D4" t="n">
-        <v>606.4</v>
+        <v>954.6</v>
       </c>
       <c r="E4" t="n">
-        <v>555.55</v>
+        <v>900.1</v>
       </c>
       <c r="F4" t="n">
-        <v>529.38</v>
+        <v>881.7</v>
       </c>
       <c r="G4" t="n">
-        <v>50429815</v>
+        <v>34270461</v>
       </c>
       <c r="H4" t="n">
-        <v>29094105</v>
+        <v>30958709</v>
       </c>
       <c r="I4" t="n">
-        <v>719</v>
+        <v>1085</v>
       </c>
       <c r="J4" t="n">
-        <v>445.5</v>
+        <v>776</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>帶量突破20日高點</t>
+          <t>無明顯異常</t>
         </is>
       </c>
       <c r="L4" t="n">
-        <v>964619</v>
+        <v>290189</v>
       </c>
       <c r="M4" t="n">
-        <v>17496756</v>
+        <v>5536520</v>
       </c>
       <c r="N4" t="n">
-        <v>19603616</v>
+        <v>14185171</v>
       </c>
       <c r="O4" t="n">
-        <v>18095930</v>
+        <v>9049490</v>
       </c>
       <c r="P4" t="n">
-        <v>145</v>
-      </c>
-      <c r="Q4" t="inlineStr">
+        <v>226631</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>4886174</v>
+      </c>
+      <c r="R4" t="n">
+        <v>11932486</v>
+      </c>
+      <c r="S4" t="n">
+        <v>4161497</v>
+      </c>
+      <c r="T4" t="n">
+        <v>212000</v>
+      </c>
+      <c r="U4" t="n">
+        <v>983843</v>
+      </c>
+      <c r="V4" t="n">
+        <v>1605943</v>
+      </c>
+      <c r="W4" t="n">
+        <v>5737686</v>
+      </c>
+      <c r="X4" t="n">
+        <v>-148442</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>-333497</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>646742</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>-849693</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>160</v>
+      </c>
+      <c r="AC4" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="AD4" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、成交量放大、帶量突破20日高點</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>法人連續偏買、5日法人明顯買超</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、成交量放大、帶量突破20日高點、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>站上5日線、多頭排列、量能溫和放大、突破20日高點</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>法人連續偏買、5日法人明顯買超、外資投信同步買超</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、量能溫和放大、突破20日高點、法人連續偏買、5日法人明顯買超、外資投信同步買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3037.TW</t>
+          <t>3105.TWO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>欣興</t>
+          <t>穩懋</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1085</v>
+        <v>562</v>
       </c>
       <c r="D5" t="n">
-        <v>954.6</v>
+        <v>513.1</v>
       </c>
       <c r="E5" t="n">
-        <v>900.1</v>
+        <v>491</v>
       </c>
       <c r="F5" t="n">
-        <v>881.7</v>
+        <v>502.85</v>
       </c>
       <c r="G5" t="n">
-        <v>34270461</v>
+        <v>33746000</v>
       </c>
       <c r="H5" t="n">
-        <v>30958709</v>
+        <v>31597000</v>
       </c>
       <c r="I5" t="n">
-        <v>1085</v>
+        <v>566</v>
       </c>
       <c r="J5" t="n">
-        <v>776</v>
+        <v>436</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -807,80 +975,116 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>1191293</v>
+        <v>4244062</v>
       </c>
       <c r="M5" t="n">
-        <v>14796086</v>
+        <v>8968342</v>
       </c>
       <c r="N5" t="n">
-        <v>14042095</v>
+        <v>9409867</v>
       </c>
       <c r="O5" t="n">
-        <v>12040296</v>
+        <v>5771807</v>
       </c>
       <c r="P5" t="n">
-        <v>140</v>
-      </c>
-      <c r="Q5" t="inlineStr">
+        <v>3267388</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>4671266</v>
+      </c>
+      <c r="R5" t="n">
+        <v>2987230</v>
+      </c>
+      <c r="S5" t="n">
+        <v>2361844</v>
+      </c>
+      <c r="T5" t="n">
+        <v>169999</v>
+      </c>
+      <c r="U5" t="n">
+        <v>1483999</v>
+      </c>
+      <c r="V5" t="n">
+        <v>3688999</v>
+      </c>
+      <c r="W5" t="n">
+        <v>2820262</v>
+      </c>
+      <c r="X5" t="n">
+        <v>806675</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>2813077</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>2733638</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>589701</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>150</v>
+      </c>
+      <c r="AC5" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="AD5" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、量能溫和放大、突破20日高點</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>法人連續偏買、5日法人明顯買超</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、量能溫和放大、突破20日高點、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>站上5日線、黃金交叉、量能溫和放大、接近20日高點</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>法人連續偏買、5日法人明顯買超、外資投信同步買超</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、黃金交叉、量能溫和放大、接近20日高點、法人連續偏買、5日法人明顯買超、外資投信同步買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2317.TW</t>
+          <t>2383.TW</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>鴻海</t>
+          <t>台光電</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>259</v>
+        <v>5290</v>
       </c>
       <c r="D6" t="n">
-        <v>251.5</v>
+        <v>4977</v>
       </c>
       <c r="E6" t="n">
-        <v>249.5</v>
+        <v>4843</v>
       </c>
       <c r="F6" t="n">
-        <v>244.47</v>
+        <v>4784.25</v>
       </c>
       <c r="G6" t="n">
-        <v>55665305</v>
+        <v>2917258</v>
       </c>
       <c r="H6" t="n">
-        <v>69819957</v>
+        <v>2443800</v>
       </c>
       <c r="I6" t="n">
-        <v>263.5</v>
+        <v>5635</v>
       </c>
       <c r="J6" t="n">
-        <v>219.5</v>
+        <v>4160</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -888,161 +1092,233 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>55787312</v>
+        <v>358474</v>
       </c>
       <c r="M6" t="n">
-        <v>101690979</v>
+        <v>862813</v>
       </c>
       <c r="N6" t="n">
-        <v>84630201</v>
+        <v>1711672</v>
       </c>
       <c r="O6" t="n">
-        <v>160089561</v>
+        <v>2931478</v>
       </c>
       <c r="P6" t="n">
-        <v>120</v>
-      </c>
-      <c r="Q6" t="inlineStr">
+        <v>279663</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>550985</v>
+      </c>
+      <c r="R6" t="n">
+        <v>1390729</v>
+      </c>
+      <c r="S6" t="n">
+        <v>2316469</v>
+      </c>
+      <c r="T6" t="n">
+        <v>16000</v>
+      </c>
+      <c r="U6" t="n">
+        <v>246834</v>
+      </c>
+      <c r="V6" t="n">
+        <v>147674</v>
+      </c>
+      <c r="W6" t="n">
+        <v>424908</v>
+      </c>
+      <c r="X6" t="n">
+        <v>62811</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>64994</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>173269</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>190101</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>135</v>
+      </c>
+      <c r="AC6" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="AD6" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、量能未放大、接近20日高點</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>法人連續偏買、5日法人明顯買超</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、量能未放大、接近20日高點、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>站上5日線、多頭排列、量能溫和放大</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>法人連續偏買、5日法人明顯買超、外資投信同步買超</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、量能溫和放大、法人連續偏買、5日法人明顯買超、外資投信同步買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2383.TW</t>
+          <t>2409.TW</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>台光電</t>
+          <t>友達</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>5290</v>
+        <v>22</v>
       </c>
       <c r="D7" t="n">
-        <v>4977</v>
+        <v>21.51</v>
       </c>
       <c r="E7" t="n">
-        <v>4843</v>
+        <v>20.48</v>
       </c>
       <c r="F7" t="n">
-        <v>4784.25</v>
+        <v>19.25</v>
       </c>
       <c r="G7" t="n">
-        <v>2917258</v>
+        <v>818361725</v>
       </c>
       <c r="H7" t="n">
-        <v>2443800</v>
+        <v>356215638</v>
       </c>
       <c r="I7" t="n">
-        <v>5635</v>
+        <v>25.8</v>
       </c>
       <c r="J7" t="n">
-        <v>4160</v>
+        <v>16.6</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>無明顯異常</t>
+          <t>爆量價未漲</t>
         </is>
       </c>
       <c r="L7" t="n">
-        <v>359818</v>
+        <v>7043839</v>
       </c>
       <c r="M7" t="n">
-        <v>1354542</v>
+        <v>40455605</v>
       </c>
       <c r="N7" t="n">
-        <v>1447903</v>
+        <v>206744209</v>
       </c>
       <c r="O7" t="n">
-        <v>2950399</v>
+        <v>255008076</v>
       </c>
       <c r="P7" t="n">
-        <v>115</v>
-      </c>
-      <c r="Q7" t="inlineStr">
+        <v>6297953</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>34550487</v>
+      </c>
+      <c r="R7" t="n">
+        <v>197817998</v>
+      </c>
+      <c r="S7" t="n">
+        <v>252197139</v>
+      </c>
+      <c r="T7" t="n">
+        <v>7000</v>
+      </c>
+      <c r="U7" t="n">
+        <v>-14237</v>
+      </c>
+      <c r="V7" t="n">
+        <v>38763</v>
+      </c>
+      <c r="W7" t="n">
+        <v>20162</v>
+      </c>
+      <c r="X7" t="n">
+        <v>738886</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>5919355</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>8887448</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>2790775</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>125</v>
+      </c>
+      <c r="AC7" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="AD7" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、量能溫和放大</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>法人連續偏買、5日法人明顯買超</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、量能溫和放大、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>站上5日線、多頭排列、爆量、爆量價未漲</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>法人連續偏買、5日法人明顯買超、外資投信同步買超</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、爆量、爆量價未漲、法人連續偏買、5日法人明顯買超、外資投信同步買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2338.TW</t>
+          <t>8358.TWO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>光罩</t>
+          <t>金居</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>55.4</v>
+        <v>533</v>
       </c>
       <c r="D8" t="n">
-        <v>53.91</v>
+        <v>511.6</v>
       </c>
       <c r="E8" t="n">
-        <v>51.25</v>
+        <v>468.75</v>
       </c>
       <c r="F8" t="n">
-        <v>50.42</v>
+        <v>448.2</v>
       </c>
       <c r="G8" t="n">
-        <v>15723414</v>
+        <v>2520000</v>
       </c>
       <c r="H8" t="n">
-        <v>11255762</v>
+        <v>4413800</v>
       </c>
       <c r="I8" t="n">
-        <v>60.3</v>
+        <v>558</v>
       </c>
       <c r="J8" t="n">
-        <v>45.45</v>
+        <v>340</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -1050,80 +1326,116 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>3454745</v>
+        <v>755377</v>
       </c>
       <c r="M8" t="n">
-        <v>13009409</v>
+        <v>2856804</v>
       </c>
       <c r="N8" t="n">
-        <v>14246624</v>
+        <v>9398836</v>
       </c>
       <c r="O8" t="n">
-        <v>12266815</v>
+        <v>7366124</v>
       </c>
       <c r="P8" t="n">
-        <v>115</v>
-      </c>
-      <c r="Q8" t="inlineStr">
+        <v>737962</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>2860498</v>
+      </c>
+      <c r="R8" t="n">
+        <v>8822301</v>
+      </c>
+      <c r="S8" t="n">
+        <v>10989591</v>
+      </c>
+      <c r="T8" t="n">
+        <v>-1200</v>
+      </c>
+      <c r="U8" t="n">
+        <v>35400</v>
+      </c>
+      <c r="V8" t="n">
+        <v>89400</v>
+      </c>
+      <c r="W8" t="n">
+        <v>-1897400</v>
+      </c>
+      <c r="X8" t="n">
+        <v>18615</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>-39094</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>487135</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>-1726067</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>125</v>
+      </c>
+      <c r="AC8" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="AD8" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、量能溫和放大</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>法人連續偏買、5日法人明顯買超</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、量能溫和放大、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>站上5日線、多頭排列、量能未放大</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>法人連續偏買、5日法人明顯買超、外資投信同步買超</t>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、量能未放大、法人連續偏買、5日法人明顯買超、外資投信同步買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2344.TW</t>
+          <t>2317.TW</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>華邦電</t>
+          <t>鴻海</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>141</v>
+        <v>259</v>
       </c>
       <c r="D9" t="n">
-        <v>124.8</v>
+        <v>251.5</v>
       </c>
       <c r="E9" t="n">
-        <v>125.75</v>
+        <v>249.5</v>
       </c>
       <c r="F9" t="n">
-        <v>114.91</v>
+        <v>244.47</v>
       </c>
       <c r="G9" t="n">
-        <v>336105421</v>
+        <v>55665305</v>
       </c>
       <c r="H9" t="n">
-        <v>249474700</v>
+        <v>69819957</v>
       </c>
       <c r="I9" t="n">
-        <v>141</v>
+        <v>263.5</v>
       </c>
       <c r="J9" t="n">
-        <v>88.8</v>
+        <v>219.5</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -1131,242 +1443,350 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>77651903</v>
+        <v>1176560</v>
       </c>
       <c r="M9" t="n">
-        <v>96687402</v>
+        <v>22207913</v>
       </c>
       <c r="N9" t="n">
-        <v>61728965</v>
+        <v>48256787</v>
       </c>
       <c r="O9" t="n">
-        <v>182119556</v>
+        <v>103877303</v>
       </c>
       <c r="P9" t="n">
-        <v>115</v>
-      </c>
-      <c r="Q9" t="inlineStr">
+        <v>1667042</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>22481766</v>
+      </c>
+      <c r="R9" t="n">
+        <v>48192094</v>
+      </c>
+      <c r="S9" t="n">
+        <v>110732127</v>
+      </c>
+      <c r="T9" t="n">
+        <v>-12810</v>
+      </c>
+      <c r="U9" t="n">
+        <v>-97437</v>
+      </c>
+      <c r="V9" t="n">
+        <v>-273247</v>
+      </c>
+      <c r="W9" t="n">
+        <v>-4762535</v>
+      </c>
+      <c r="X9" t="n">
+        <v>-477672</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>-176416</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>337940</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>-2092289</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC9" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="AD9" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>站上5日線、量能溫和放大、突破20日高點</t>
-        </is>
-      </c>
-      <c r="T9" t="inlineStr">
-        <is>
-          <t>法人連續偏買、5日法人明顯買超</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、量能溫和放大、突破20日高點、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>站上5日線、多頭排列、量能未放大、接近20日高點</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>法人連續偏買、5日法人明顯買超、外資買投信賣</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、量能未放大、接近20日高點、法人連續偏買、5日法人明顯買超、外資買投信賣。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>8358.TWO</t>
+          <t>6116.TW</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>金居</t>
+          <t>彩晶</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>533</v>
+        <v>13.65</v>
       </c>
       <c r="D10" t="n">
-        <v>511.6</v>
+        <v>11.83</v>
       </c>
       <c r="E10" t="n">
-        <v>468.75</v>
+        <v>11.16</v>
       </c>
       <c r="F10" t="n">
-        <v>448.2</v>
+        <v>10.02</v>
       </c>
       <c r="G10" t="n">
-        <v>2520000</v>
+        <v>478320069</v>
       </c>
       <c r="H10" t="n">
-        <v>4413800</v>
+        <v>148294428</v>
       </c>
       <c r="I10" t="n">
-        <v>558</v>
+        <v>14.3</v>
       </c>
       <c r="J10" t="n">
-        <v>340</v>
+        <v>8.130000000000001</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>無明顯異常</t>
+          <t>帶量突破20日高點</t>
         </is>
       </c>
       <c r="L10" t="n">
-        <v>434414</v>
+        <v>-3262412</v>
       </c>
       <c r="M10" t="n">
-        <v>4299788</v>
+        <v>22044344</v>
       </c>
       <c r="N10" t="n">
-        <v>9649180</v>
+        <v>50882174</v>
       </c>
       <c r="O10" t="n">
-        <v>9535283</v>
+        <v>25324386</v>
       </c>
       <c r="P10" t="n">
-        <v>105</v>
-      </c>
-      <c r="Q10" t="inlineStr">
+        <v>-4232242</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>20328525</v>
+      </c>
+      <c r="R10" t="n">
+        <v>47907283</v>
+      </c>
+      <c r="S10" t="n">
+        <v>21954098</v>
+      </c>
+      <c r="T10" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" t="n">
+        <v>0</v>
+      </c>
+      <c r="V10" t="n">
+        <v>0</v>
+      </c>
+      <c r="W10" t="n">
+        <v>0</v>
+      </c>
+      <c r="X10" t="n">
+        <v>969830</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>1715819</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>2974891</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>3370288</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC10" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="AD10" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、量能未放大</t>
-        </is>
-      </c>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>法人連續偏買、5日法人明顯買超</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、量能未放大、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>站上5日線、多頭排列、爆量、帶量突破20日高點</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>5日法人明顯買超</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、爆量、帶量突破20日高點、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>6274.TWO</t>
+          <t>2338.TW</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>台燿</t>
+          <t>光罩</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1580</v>
+        <v>55.4</v>
       </c>
       <c r="D11" t="n">
-        <v>1433</v>
+        <v>53.91</v>
       </c>
       <c r="E11" t="n">
-        <v>1385.5</v>
+        <v>51.25</v>
       </c>
       <c r="F11" t="n">
-        <v>1308.55</v>
+        <v>50.42</v>
       </c>
       <c r="G11" t="n">
-        <v>9546000</v>
+        <v>15723414</v>
       </c>
       <c r="H11" t="n">
-        <v>3017800</v>
+        <v>11255762</v>
       </c>
       <c r="I11" t="n">
-        <v>1700</v>
+        <v>60.3</v>
       </c>
       <c r="J11" t="n">
-        <v>941</v>
+        <v>45.45</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>爆量價未漲</t>
+          <t>無明顯異常</t>
         </is>
       </c>
       <c r="L11" t="n">
-        <v>282254</v>
+        <v>198200</v>
       </c>
       <c r="M11" t="n">
-        <v>969253</v>
+        <v>4087251</v>
       </c>
       <c r="N11" t="n">
-        <v>1221688</v>
+        <v>9951064</v>
       </c>
       <c r="O11" t="n">
-        <v>2123947</v>
+        <v>7954561</v>
       </c>
       <c r="P11" t="n">
-        <v>105</v>
-      </c>
-      <c r="Q11" t="inlineStr">
+        <v>177415</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>3934844</v>
+      </c>
+      <c r="R11" t="n">
+        <v>9678259</v>
+      </c>
+      <c r="S11" t="n">
+        <v>7765339</v>
+      </c>
+      <c r="T11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X11" t="n">
+        <v>20785</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>152407</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>272805</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>189222</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>115</v>
+      </c>
+      <c r="AC11" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
+      <c r="AD11" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、爆量、爆量價未漲</t>
-        </is>
-      </c>
-      <c r="T11" t="inlineStr">
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>站上5日線、多頭排列、量能溫和放大</t>
+        </is>
+      </c>
+      <c r="AF11" t="inlineStr">
         <is>
           <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、爆量、爆量價未漲、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、量能溫和放大、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2327.TW</t>
+          <t>6285.TW</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>國巨</t>
+          <t>啟碁</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>661</v>
+        <v>304.5</v>
       </c>
       <c r="D12" t="n">
-        <v>614.6</v>
+        <v>291.6</v>
       </c>
       <c r="E12" t="n">
-        <v>540.85</v>
+        <v>282.85</v>
       </c>
       <c r="F12" t="n">
-        <v>448.73</v>
+        <v>260.6</v>
       </c>
       <c r="G12" t="n">
-        <v>29457930</v>
+        <v>21738108</v>
       </c>
       <c r="H12" t="n">
-        <v>56139070</v>
+        <v>31212343</v>
       </c>
       <c r="I12" t="n">
-        <v>691</v>
+        <v>317</v>
       </c>
       <c r="J12" t="n">
-        <v>307</v>
+        <v>208.5</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -1374,404 +1794,584 @@
         </is>
       </c>
       <c r="L12" t="n">
-        <v>2231528</v>
+        <v>4745353</v>
       </c>
       <c r="M12" t="n">
-        <v>3889908</v>
+        <v>9834017</v>
       </c>
       <c r="N12" t="n">
-        <v>9359269</v>
+        <v>10574690</v>
       </c>
       <c r="O12" t="n">
-        <v>20009905</v>
+        <v>20883168</v>
       </c>
       <c r="P12" t="n">
+        <v>4763785</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>10787025</v>
+      </c>
+      <c r="R12" t="n">
+        <v>13381377</v>
+      </c>
+      <c r="S12" t="n">
+        <v>26096411</v>
+      </c>
+      <c r="T12" t="n">
+        <v>-101000</v>
+      </c>
+      <c r="U12" t="n">
+        <v>-1724000</v>
+      </c>
+      <c r="V12" t="n">
+        <v>-3525000</v>
+      </c>
+      <c r="W12" t="n">
+        <v>-4431464</v>
+      </c>
+      <c r="X12" t="n">
+        <v>82568</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>770992</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>718313</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>-781779</v>
+      </c>
+      <c r="AB12" t="n">
         <v>105</v>
       </c>
-      <c r="Q12" t="inlineStr">
+      <c r="AC12" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
+      <c r="AD12" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr">
+      <c r="AE12" t="inlineStr">
         <is>
           <t>站上5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr">
-        <is>
-          <t>法人連續偏買、5日法人明顯買超</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、量能未放大、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>法人連續偏買、5日法人明顯買超、外資買投信賣</t>
+        </is>
+      </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、量能未放大、法人連續偏買、5日法人明顯買超、外資買投信賣。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1802.TW</t>
+          <t>2609.TW</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>台玻</t>
+          <t>陽明</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>72.2</v>
+        <v>52</v>
       </c>
       <c r="D13" t="n">
-        <v>69.12</v>
+        <v>51.64</v>
       </c>
       <c r="E13" t="n">
-        <v>67.56</v>
+        <v>50.21</v>
       </c>
       <c r="F13" t="n">
-        <v>68.52</v>
+        <v>50.11</v>
       </c>
       <c r="G13" t="n">
-        <v>337055872</v>
+        <v>14910096</v>
       </c>
       <c r="H13" t="n">
-        <v>147844553</v>
+        <v>26622786</v>
       </c>
       <c r="I13" t="n">
-        <v>81.2</v>
+        <v>53.9</v>
       </c>
       <c r="J13" t="n">
-        <v>61.8</v>
+        <v>47.35</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>爆量價未漲</t>
+          <t>無明顯異常</t>
         </is>
       </c>
       <c r="L13" t="n">
-        <v>44538498</v>
+        <v>1599308</v>
       </c>
       <c r="M13" t="n">
-        <v>88202486</v>
+        <v>19287277</v>
       </c>
       <c r="N13" t="n">
-        <v>75247740</v>
+        <v>32054623</v>
       </c>
       <c r="O13" t="n">
-        <v>32596649</v>
+        <v>9933706</v>
       </c>
       <c r="P13" t="n">
+        <v>1194273</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>18166886</v>
+      </c>
+      <c r="R13" t="n">
+        <v>30323339</v>
+      </c>
+      <c r="S13" t="n">
+        <v>8970452</v>
+      </c>
+      <c r="T13" t="n">
+        <v>900</v>
+      </c>
+      <c r="U13" t="n">
+        <v>-26066</v>
+      </c>
+      <c r="V13" t="n">
+        <v>-64166</v>
+      </c>
+      <c r="W13" t="n">
+        <v>-341744</v>
+      </c>
+      <c r="X13" t="n">
+        <v>404135</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>1146457</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>1795450</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>1304998</v>
+      </c>
+      <c r="AB13" t="n">
         <v>105</v>
       </c>
-      <c r="Q13" t="inlineStr">
+      <c r="AC13" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="R13" t="inlineStr">
+      <c r="AD13" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>站上5日線、黃金交叉、爆量、爆量價未漲</t>
-        </is>
-      </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>法人連續偏買、5日法人明顯買超</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、黃金交叉、爆量、爆量價未漲、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>站上5日線、多頭排列、量能未放大</t>
+        </is>
+      </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>法人連續偏買、5日法人明顯買超、外資買投信賣</t>
+        </is>
+      </c>
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、量能未放大、法人連續偏買、5日法人明顯買超、外資買投信賣。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2409.TW</t>
+          <t>2327.TW</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>友達</t>
+          <t>國巨</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>22</v>
+        <v>661</v>
       </c>
       <c r="D14" t="n">
-        <v>21.51</v>
+        <v>614.6</v>
       </c>
       <c r="E14" t="n">
-        <v>20.48</v>
+        <v>540.85</v>
       </c>
       <c r="F14" t="n">
-        <v>19.25</v>
+        <v>448.73</v>
       </c>
       <c r="G14" t="n">
-        <v>818361725</v>
+        <v>29457930</v>
       </c>
       <c r="H14" t="n">
-        <v>356215638</v>
+        <v>56139070</v>
       </c>
       <c r="I14" t="n">
-        <v>25.8</v>
+        <v>691</v>
       </c>
       <c r="J14" t="n">
-        <v>16.6</v>
+        <v>307</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>爆量價未漲</t>
+          <t>無明顯異常</t>
         </is>
       </c>
       <c r="L14" t="n">
-        <v>18947923</v>
+        <v>1102045</v>
       </c>
       <c r="M14" t="n">
-        <v>211604454</v>
+        <v>4327355</v>
       </c>
       <c r="N14" t="n">
-        <v>192942642</v>
+        <v>3862470</v>
       </c>
       <c r="O14" t="n">
-        <v>353520387</v>
+        <v>14290677</v>
       </c>
       <c r="P14" t="n">
+        <v>-4617135</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>-4685625</v>
+      </c>
+      <c r="R14" t="n">
+        <v>-12048132</v>
+      </c>
+      <c r="S14" t="n">
+        <v>-24677774</v>
+      </c>
+      <c r="T14" t="n">
+        <v>6849000</v>
+      </c>
+      <c r="U14" t="n">
+        <v>8963449</v>
+      </c>
+      <c r="V14" t="n">
+        <v>16117449</v>
+      </c>
+      <c r="W14" t="n">
+        <v>41742069</v>
+      </c>
+      <c r="X14" t="n">
+        <v>-1129820</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>49531</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>-206847</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>-2773618</v>
+      </c>
+      <c r="AB14" t="n">
         <v>105</v>
       </c>
-      <c r="Q14" t="inlineStr">
+      <c r="AC14" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr">
+      <c r="AD14" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、爆量、爆量價未漲</t>
-        </is>
-      </c>
-      <c r="T14" t="inlineStr">
-        <is>
-          <t>法人連續偏買、5日法人明顯買超</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、爆量、爆量價未漲、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>站上5日線、多頭排列、量能未放大</t>
+        </is>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>法人連續偏買、5日法人明顯買超、投信買外資賣</t>
+        </is>
+      </c>
+      <c r="AG14" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、量能未放大、法人連續偏買、5日法人明顯買超、投信買外資賣。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>3105.TWO</t>
+          <t>1802.TW</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>穩懋</t>
+          <t>台玻</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>562</v>
+        <v>72.2</v>
       </c>
       <c r="D15" t="n">
-        <v>513.1</v>
+        <v>69.12</v>
       </c>
       <c r="E15" t="n">
-        <v>491</v>
+        <v>67.56</v>
       </c>
       <c r="F15" t="n">
-        <v>502.85</v>
+        <v>68.52</v>
       </c>
       <c r="G15" t="n">
-        <v>33746000</v>
+        <v>337055872</v>
       </c>
       <c r="H15" t="n">
-        <v>31597000</v>
+        <v>147844553</v>
       </c>
       <c r="I15" t="n">
-        <v>566</v>
+        <v>81.2</v>
       </c>
       <c r="J15" t="n">
-        <v>436</v>
+        <v>61.8</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>無明顯異常</t>
+          <t>爆量價未漲</t>
         </is>
       </c>
       <c r="L15" t="n">
-        <v>-709786</v>
+        <v>-8515087</v>
       </c>
       <c r="M15" t="n">
-        <v>7825302</v>
+        <v>28946585</v>
       </c>
       <c r="N15" t="n">
-        <v>4382193</v>
+        <v>26633814</v>
       </c>
       <c r="O15" t="n">
-        <v>-4637373</v>
+        <v>-37000661</v>
       </c>
       <c r="P15" t="n">
-        <v>100</v>
-      </c>
-      <c r="Q15" t="inlineStr">
+        <v>-9231376</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>26801156</v>
+      </c>
+      <c r="R15" t="n">
+        <v>23647845</v>
+      </c>
+      <c r="S15" t="n">
+        <v>-36842695</v>
+      </c>
+      <c r="T15" t="n">
+        <v>0</v>
+      </c>
+      <c r="U15" t="n">
+        <v>11000</v>
+      </c>
+      <c r="V15" t="n">
+        <v>33000</v>
+      </c>
+      <c r="W15" t="n">
+        <v>26000</v>
+      </c>
+      <c r="X15" t="n">
+        <v>716289</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>2134429</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>2952969</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>-183966</v>
+      </c>
+      <c r="AB15" t="n">
+        <v>95</v>
+      </c>
+      <c r="AC15" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr">
+      <c r="AD15" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>站上5日線、黃金交叉、量能溫和放大、接近20日高點</t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t>5日法人明顯買超</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、黃金交叉、量能溫和放大、接近20日高點、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>站上5日線、黃金交叉、爆量、爆量價未漲</t>
+        </is>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>5日法人明顯買超、外資投信同步買超</t>
+        </is>
+      </c>
+      <c r="AG15" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、黃金交叉、爆量、爆量價未漲、5日法人明顯買超、外資投信同步買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2308.TW</t>
+          <t>3481.TW</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>台達電</t>
+          <t>群創</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2350</v>
+        <v>45.7</v>
       </c>
       <c r="D16" t="n">
-        <v>2136</v>
+        <v>43.4</v>
       </c>
       <c r="E16" t="n">
-        <v>2101</v>
+        <v>40.22</v>
       </c>
       <c r="F16" t="n">
-        <v>2149</v>
+        <v>34.08</v>
       </c>
       <c r="G16" t="n">
-        <v>12198582</v>
+        <v>1463227218</v>
       </c>
       <c r="H16" t="n">
-        <v>11067330</v>
+        <v>613882104</v>
       </c>
       <c r="I16" t="n">
-        <v>2410</v>
+        <v>52.2</v>
       </c>
       <c r="J16" t="n">
-        <v>1880</v>
+        <v>23.65</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>無明顯異常</t>
+          <t>爆量價未漲</t>
         </is>
       </c>
       <c r="L16" t="n">
-        <v>4917556</v>
+        <v>-20234462</v>
       </c>
       <c r="M16" t="n">
-        <v>5273927</v>
+        <v>-5521196</v>
       </c>
       <c r="N16" t="n">
-        <v>1917848</v>
+        <v>83429081</v>
       </c>
       <c r="O16" t="n">
-        <v>-4082627</v>
+        <v>59378294</v>
       </c>
       <c r="P16" t="n">
-        <v>90</v>
-      </c>
-      <c r="Q16" t="inlineStr">
+        <v>-26508116</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>-14599220</v>
+      </c>
+      <c r="R16" t="n">
+        <v>56981613</v>
+      </c>
+      <c r="S16" t="n">
+        <v>16527987</v>
+      </c>
+      <c r="T16" t="n">
+        <v>43100</v>
+      </c>
+      <c r="U16" t="n">
+        <v>13211</v>
+      </c>
+      <c r="V16" t="n">
+        <v>17311</v>
+      </c>
+      <c r="W16" t="n">
+        <v>453089</v>
+      </c>
+      <c r="X16" t="n">
+        <v>6230554</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>9064813</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>26430157</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>42397218</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>95</v>
+      </c>
+      <c r="AC16" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="R16" t="inlineStr">
+      <c r="AD16" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>站上5日線、量能溫和放大</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>法人連續偏買、5日法人明顯買超</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、量能溫和放大、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>站上5日線、多頭排列、爆量、爆量價未漲</t>
+        </is>
+      </c>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t>5日法人明顯買超、外資投信同步買超</t>
+        </is>
+      </c>
+      <c r="AG16" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、爆量、爆量價未漲、5日法人明顯買超、外資投信同步買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2374.TW</t>
+          <t>8046.TW</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>佳能</t>
+          <t>南電</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>82.40000000000001</v>
+        <v>922</v>
       </c>
       <c r="D17" t="n">
-        <v>81.73999999999999</v>
+        <v>888.2</v>
       </c>
       <c r="E17" t="n">
-        <v>81.34</v>
+        <v>854.3</v>
       </c>
       <c r="F17" t="n">
-        <v>80.16</v>
+        <v>896.4</v>
       </c>
       <c r="G17" t="n">
-        <v>12463968</v>
+        <v>24438087</v>
       </c>
       <c r="H17" t="n">
-        <v>10197116</v>
+        <v>20893593</v>
       </c>
       <c r="I17" t="n">
-        <v>85.8</v>
+        <v>1035</v>
       </c>
       <c r="J17" t="n">
-        <v>70.2</v>
+        <v>765</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -1779,80 +2379,116 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>-491799</v>
+        <v>-208181</v>
       </c>
       <c r="M17" t="n">
-        <v>7106107</v>
+        <v>3582994</v>
       </c>
       <c r="N17" t="n">
-        <v>4374099</v>
+        <v>3677318</v>
       </c>
       <c r="O17" t="n">
-        <v>9626033</v>
+        <v>-1724114</v>
       </c>
       <c r="P17" t="n">
-        <v>85</v>
-      </c>
-      <c r="Q17" t="inlineStr">
+        <v>39735</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>1895312</v>
+      </c>
+      <c r="R17" t="n">
+        <v>1121613</v>
+      </c>
+      <c r="S17" t="n">
+        <v>-12620</v>
+      </c>
+      <c r="T17" t="n">
+        <v>-165000</v>
+      </c>
+      <c r="U17" t="n">
+        <v>1591000</v>
+      </c>
+      <c r="V17" t="n">
+        <v>2486000</v>
+      </c>
+      <c r="W17" t="n">
+        <v>-1244694</v>
+      </c>
+      <c r="X17" t="n">
+        <v>-82916</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>96682</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>69705</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>-466800</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>80</v>
+      </c>
+      <c r="AC17" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr">
+      <c r="AD17" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、量能溫和放大</t>
-        </is>
-      </c>
-      <c r="T17" t="inlineStr">
-        <is>
-          <t>5日法人明顯買超</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、量能溫和放大、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>站上5日線、量能溫和放大</t>
+        </is>
+      </c>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t>5日法人明顯買超、外資投信同步買超</t>
+        </is>
+      </c>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、量能溫和放大、5日法人明顯買超、外資投信同步買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>3711.TW</t>
+          <t>4958.TW</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>日月光投控</t>
+          <t>臻鼎-KY</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>611</v>
+        <v>540</v>
       </c>
       <c r="D18" t="n">
-        <v>555</v>
+        <v>498.7</v>
       </c>
       <c r="E18" t="n">
-        <v>540</v>
+        <v>457.05</v>
       </c>
       <c r="F18" t="n">
-        <v>528.95</v>
+        <v>434.32</v>
       </c>
       <c r="G18" t="n">
-        <v>39627497</v>
+        <v>41904053</v>
       </c>
       <c r="H18" t="n">
-        <v>28597065</v>
+        <v>51443369</v>
       </c>
       <c r="I18" t="n">
-        <v>636</v>
+        <v>558</v>
       </c>
       <c r="J18" t="n">
-        <v>465</v>
+        <v>354</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -1860,80 +2496,116 @@
         </is>
       </c>
       <c r="L18" t="n">
-        <v>-1946569</v>
+        <v>-967994</v>
       </c>
       <c r="M18" t="n">
-        <v>4398628</v>
+        <v>-1212400</v>
       </c>
       <c r="N18" t="n">
-        <v>375095</v>
+        <v>2289305</v>
       </c>
       <c r="O18" t="n">
-        <v>-4267040</v>
+        <v>1887707</v>
       </c>
       <c r="P18" t="n">
+        <v>1375340</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>-2831559</v>
+      </c>
+      <c r="R18" t="n">
+        <v>-676473</v>
+      </c>
+      <c r="S18" t="n">
+        <v>4958845</v>
+      </c>
+      <c r="T18" t="n">
+        <v>-2688000</v>
+      </c>
+      <c r="U18" t="n">
+        <v>848563</v>
+      </c>
+      <c r="V18" t="n">
+        <v>1580563</v>
+      </c>
+      <c r="W18" t="n">
+        <v>-4914501</v>
+      </c>
+      <c r="X18" t="n">
+        <v>344666</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>770596</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>1385215</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>1843363</v>
+      </c>
+      <c r="AB18" t="n">
         <v>75</v>
       </c>
-      <c r="Q18" t="inlineStr">
+      <c r="AC18" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="R18" t="inlineStr">
+      <c r="AD18" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、量能溫和放大</t>
-        </is>
-      </c>
-      <c r="T18" t="inlineStr">
-        <is>
-          <t>5日法人買超</t>
-        </is>
-      </c>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、量能溫和放大、5日法人買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>站上5日線、多頭排列、量能未放大</t>
+        </is>
+      </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>5日法人明顯買超、投信買外資賣</t>
+        </is>
+      </c>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、量能未放大、5日法人明顯買超、投信買外資賣。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>3481.TW</t>
+          <t>6274.TWO</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>群創</t>
+          <t>台燿</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>45.7</v>
+        <v>1580</v>
       </c>
       <c r="D19" t="n">
-        <v>43.4</v>
+        <v>1433</v>
       </c>
       <c r="E19" t="n">
-        <v>40.22</v>
+        <v>1385.5</v>
       </c>
       <c r="F19" t="n">
-        <v>34.08</v>
+        <v>1308.55</v>
       </c>
       <c r="G19" t="n">
-        <v>1463227218</v>
+        <v>9546000</v>
       </c>
       <c r="H19" t="n">
-        <v>613882104</v>
+        <v>3017800</v>
       </c>
       <c r="I19" t="n">
-        <v>52.2</v>
+        <v>1700</v>
       </c>
       <c r="J19" t="n">
-        <v>23.65</v>
+        <v>941</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -1941,80 +2613,116 @@
         </is>
       </c>
       <c r="L19" t="n">
-        <v>-2664727</v>
+        <v>-83545</v>
       </c>
       <c r="M19" t="n">
-        <v>121233278</v>
+        <v>660709</v>
       </c>
       <c r="N19" t="n">
-        <v>74438491</v>
+        <v>848398</v>
       </c>
       <c r="O19" t="n">
-        <v>153391454</v>
+        <v>2026953</v>
       </c>
       <c r="P19" t="n">
+        <v>-1100380</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>-461658</v>
+      </c>
+      <c r="R19" t="n">
+        <v>-27799</v>
+      </c>
+      <c r="S19" t="n">
+        <v>1154682</v>
+      </c>
+      <c r="T19" t="n">
+        <v>1406000</v>
+      </c>
+      <c r="U19" t="n">
+        <v>1457700</v>
+      </c>
+      <c r="V19" t="n">
+        <v>1445700</v>
+      </c>
+      <c r="W19" t="n">
+        <v>427100</v>
+      </c>
+      <c r="X19" t="n">
+        <v>-389165</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>-335333</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>-569503</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>445171</v>
+      </c>
+      <c r="AB19" t="n">
         <v>75</v>
       </c>
-      <c r="Q19" t="inlineStr">
+      <c r="AC19" t="inlineStr">
         <is>
           <t>🔥強勢</t>
         </is>
       </c>
-      <c r="R19" t="inlineStr">
+      <c r="AD19" t="inlineStr">
         <is>
           <t>強勢觀察</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr">
+      <c r="AE19" t="inlineStr">
         <is>
           <t>站上5日線、多頭排列、爆量、爆量價未漲</t>
         </is>
       </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>5日法人明顯買超</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、爆量、爆量價未漲、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>5日法人明顯買超、投信買外資賣</t>
+        </is>
+      </c>
+      <c r="AG19" t="inlineStr">
+        <is>
+          <t>強勢偏多：站上5日線、多頭排列、爆量、爆量價未漲、5日法人明顯買超、投信買外資賣。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>4958.TW</t>
+          <t>6669.TW</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>臻鼎-KY</t>
+          <t>緯穎</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>540</v>
+        <v>5280</v>
       </c>
       <c r="D20" t="n">
-        <v>498.7</v>
+        <v>5334</v>
       </c>
       <c r="E20" t="n">
-        <v>457.05</v>
+        <v>5278</v>
       </c>
       <c r="F20" t="n">
-        <v>434.32</v>
+        <v>5144.75</v>
       </c>
       <c r="G20" t="n">
-        <v>41904053</v>
+        <v>2655826</v>
       </c>
       <c r="H20" t="n">
-        <v>51443369</v>
+        <v>2172103</v>
       </c>
       <c r="I20" t="n">
-        <v>558</v>
+        <v>5880</v>
       </c>
       <c r="J20" t="n">
-        <v>354</v>
+        <v>4615</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -2022,80 +2730,116 @@
         </is>
       </c>
       <c r="L20" t="n">
-        <v>-5716319</v>
+        <v>15106</v>
       </c>
       <c r="M20" t="n">
-        <v>-1491026</v>
+        <v>117253</v>
       </c>
       <c r="N20" t="n">
-        <v>13501619</v>
+        <v>77678</v>
       </c>
       <c r="O20" t="n">
-        <v>10633143</v>
+        <v>198915</v>
       </c>
       <c r="P20" t="n">
-        <v>75</v>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>🔥強勢</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>強勢觀察</t>
-        </is>
-      </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、量能未放大</t>
-        </is>
-      </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>5日法人明顯買超</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、量能未放大、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+        <v>-44712</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>91809</v>
+      </c>
+      <c r="R20" t="n">
+        <v>-160303</v>
+      </c>
+      <c r="S20" t="n">
+        <v>-526781</v>
+      </c>
+      <c r="T20" t="n">
+        <v>36000</v>
+      </c>
+      <c r="U20" t="n">
+        <v>-29006</v>
+      </c>
+      <c r="V20" t="n">
+        <v>78994</v>
+      </c>
+      <c r="W20" t="n">
+        <v>635413</v>
+      </c>
+      <c r="X20" t="n">
+        <v>23818</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>54450</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>158987</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>90283</v>
+      </c>
+      <c r="AB20" t="n">
+        <v>55</v>
+      </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>👀觀察</t>
+        </is>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>偏多觀察</t>
+        </is>
+      </c>
+      <c r="AE20" t="inlineStr">
+        <is>
+          <t>跌破5日線、多頭排列、量能溫和放大</t>
+        </is>
+      </c>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>法人連續偏買、5日法人小幅買超、投信買外資賣</t>
+        </is>
+      </c>
+      <c r="AG20" t="inlineStr">
+        <is>
+          <t>偏多觀察：跌破5日線、多頭排列、量能溫和放大、法人連續偏買、5日法人小幅買超、投信買外資賣。條件不差，適合等待拉回或突破確認。</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2609.TW</t>
+          <t>3035.TW</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>陽明</t>
+          <t>智原</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>52</v>
+        <v>168</v>
       </c>
       <c r="D21" t="n">
-        <v>51.64</v>
+        <v>176.9</v>
       </c>
       <c r="E21" t="n">
-        <v>50.21</v>
+        <v>174.55</v>
       </c>
       <c r="F21" t="n">
-        <v>50.11</v>
+        <v>161.45</v>
       </c>
       <c r="G21" t="n">
-        <v>14910096</v>
+        <v>9878768</v>
       </c>
       <c r="H21" t="n">
-        <v>26622786</v>
+        <v>26306205</v>
       </c>
       <c r="I21" t="n">
-        <v>53.9</v>
+        <v>198.5</v>
       </c>
       <c r="J21" t="n">
-        <v>47.35</v>
+        <v>139</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -2103,80 +2847,116 @@
         </is>
       </c>
       <c r="L21" t="n">
-        <v>-7838235</v>
+        <v>836799</v>
       </c>
       <c r="M21" t="n">
-        <v>21017772</v>
+        <v>-413419</v>
       </c>
       <c r="N21" t="n">
-        <v>26241510</v>
+        <v>9121757</v>
       </c>
       <c r="O21" t="n">
-        <v>-434219</v>
+        <v>4176141</v>
       </c>
       <c r="P21" t="n">
-        <v>75</v>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>🔥強勢</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>強勢觀察</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、量能未放大</t>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>5日法人明顯買超</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、量能未放大、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+        <v>449302</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>-565158</v>
+      </c>
+      <c r="R21" t="n">
+        <v>7723967</v>
+      </c>
+      <c r="S21" t="n">
+        <v>3221282</v>
+      </c>
+      <c r="T21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U21" t="n">
+        <v>0</v>
+      </c>
+      <c r="V21" t="n">
+        <v>5000</v>
+      </c>
+      <c r="W21" t="n">
+        <v>6393</v>
+      </c>
+      <c r="X21" t="n">
+        <v>387497</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>151739</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>1392790</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>948466</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>55</v>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>👀觀察</t>
+        </is>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>偏多觀察</t>
+        </is>
+      </c>
+      <c r="AE21" t="inlineStr">
+        <is>
+          <t>跌破5日線、多頭排列、量能未放大</t>
+        </is>
+      </c>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>5日法人明顯買超、外資投信同步買超</t>
+        </is>
+      </c>
+      <c r="AG21" t="inlineStr">
+        <is>
+          <t>偏多觀察：跌破5日線、多頭排列、量能未放大、5日法人明顯買超、外資投信同步買超。條件不差，適合等待拉回或突破確認。</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>3035.TW</t>
+          <t>2374.TW</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>智原</t>
+          <t>佳能</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>208</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="D22" t="n">
-        <v>207</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="E22" t="n">
-        <v>199.9</v>
+        <v>81.34</v>
       </c>
       <c r="F22" t="n">
-        <v>190.12</v>
+        <v>80.16</v>
       </c>
       <c r="G22" t="n">
-        <v>20600438</v>
+        <v>12463968</v>
       </c>
       <c r="H22" t="n">
-        <v>22454689</v>
+        <v>10197116</v>
       </c>
       <c r="I22" t="n">
-        <v>231</v>
+        <v>85.8</v>
       </c>
       <c r="J22" t="n">
-        <v>167</v>
+        <v>70.2</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -2184,80 +2964,116 @@
         </is>
       </c>
       <c r="L22" t="n">
-        <v>-1076740</v>
+        <v>-4199015</v>
       </c>
       <c r="M22" t="n">
-        <v>6371419</v>
+        <v>2506502</v>
       </c>
       <c r="N22" t="n">
-        <v>6997630</v>
+        <v>-800124</v>
       </c>
       <c r="O22" t="n">
-        <v>194327</v>
+        <v>-4198886</v>
       </c>
       <c r="P22" t="n">
-        <v>75</v>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>🔥強勢</t>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>強勢觀察</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、量能未放大</t>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t>5日法人明顯買超</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、量能未放大、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+        <v>-4105690</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>2163760</v>
+      </c>
+      <c r="R22" t="n">
+        <v>-1000255</v>
+      </c>
+      <c r="S22" t="n">
+        <v>-4318549</v>
+      </c>
+      <c r="T22" t="n">
+        <v>0</v>
+      </c>
+      <c r="U22" t="n">
+        <v>0</v>
+      </c>
+      <c r="V22" t="n">
+        <v>0</v>
+      </c>
+      <c r="W22" t="n">
+        <v>-8000</v>
+      </c>
+      <c r="X22" t="n">
+        <v>-93325</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>342742</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>200131</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>127663</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>40</v>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>⚠️整理</t>
+        </is>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>整理觀察</t>
+        </is>
+      </c>
+      <c r="AE22" t="inlineStr">
+        <is>
+          <t>站上5日線、多頭排列、量能溫和放大</t>
+        </is>
+      </c>
+      <c r="AF22" t="inlineStr">
+        <is>
+          <t>短線籌碼止穩、5日法人明顯賣超</t>
+        </is>
+      </c>
+      <c r="AG22" t="inlineStr">
+        <is>
+          <t>整理觀察：站上5日線、多頭排列、量能溫和放大、短線籌碼止穩、5日法人明顯賣超。多空訊號混合，建議降低追價衝動。</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2330.TW</t>
+          <t>2308.TW</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>台積電</t>
+          <t>台達電</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2270</v>
+        <v>2350</v>
       </c>
       <c r="D23" t="n">
-        <v>2250</v>
+        <v>2136</v>
       </c>
       <c r="E23" t="n">
-        <v>2245</v>
+        <v>2101</v>
       </c>
       <c r="F23" t="n">
-        <v>2242.25</v>
+        <v>2149</v>
       </c>
       <c r="G23" t="n">
-        <v>32781470</v>
+        <v>12198582</v>
       </c>
       <c r="H23" t="n">
-        <v>30223565</v>
+        <v>11067330</v>
       </c>
       <c r="I23" t="n">
-        <v>2345</v>
+        <v>2410</v>
       </c>
       <c r="J23" t="n">
-        <v>2135</v>
+        <v>1880</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -2265,161 +3081,233 @@
         </is>
       </c>
       <c r="L23" t="n">
-        <v>8271589</v>
+        <v>-65912</v>
       </c>
       <c r="M23" t="n">
-        <v>10332214</v>
+        <v>-250347</v>
       </c>
       <c r="N23" t="n">
-        <v>-12125572</v>
+        <v>290459</v>
       </c>
       <c r="O23" t="n">
-        <v>-16581218</v>
+        <v>-1481438</v>
       </c>
       <c r="P23" t="n">
-        <v>65</v>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>👀觀察</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>偏多觀察</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、黃金交叉、量能溫和放大</t>
-        </is>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>短線籌碼止穩、5日法人明顯賣超</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>偏多觀察：站上5日線、多頭排列、黃金交叉、量能溫和放大、短線籌碼止穩、5日法人明顯賣超。條件不差，適合等待拉回或突破確認。</t>
+        <v>121443</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>-295</v>
+      </c>
+      <c r="R23" t="n">
+        <v>-145909</v>
+      </c>
+      <c r="S23" t="n">
+        <v>33483</v>
+      </c>
+      <c r="T23" t="n">
+        <v>-120500</v>
+      </c>
+      <c r="U23" t="n">
+        <v>-231968</v>
+      </c>
+      <c r="V23" t="n">
+        <v>-485259</v>
+      </c>
+      <c r="W23" t="n">
+        <v>-1333854</v>
+      </c>
+      <c r="X23" t="n">
+        <v>-66855</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>-18084</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>921627</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>-181067</v>
+      </c>
+      <c r="AB23" t="n">
+        <v>30</v>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>⚠️整理</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>整理觀察</t>
+        </is>
+      </c>
+      <c r="AE23" t="inlineStr">
+        <is>
+          <t>站上5日線、量能溫和放大</t>
+        </is>
+      </c>
+      <c r="AF23" t="inlineStr">
+        <is>
+          <t>5日法人買超、外資投信同步賣超</t>
+        </is>
+      </c>
+      <c r="AG23" t="inlineStr">
+        <is>
+          <t>整理觀察：站上5日線、量能溫和放大、5日法人買超、外資投信同步賣超。多空訊號混合，建議降低追價衝動。</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>6239.TW</t>
+          <t>2330.TW</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>力成</t>
+          <t>台積電</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>342</v>
+        <v>2270</v>
       </c>
       <c r="D24" t="n">
-        <v>285.6</v>
+        <v>2250</v>
       </c>
       <c r="E24" t="n">
-        <v>261.4</v>
+        <v>2245</v>
       </c>
       <c r="F24" t="n">
-        <v>241.47</v>
+        <v>2242.25</v>
       </c>
       <c r="G24" t="n">
-        <v>57938700</v>
+        <v>32781470</v>
       </c>
       <c r="H24" t="n">
-        <v>22861322</v>
+        <v>30223565</v>
       </c>
       <c r="I24" t="n">
-        <v>342</v>
+        <v>2345</v>
       </c>
       <c r="J24" t="n">
-        <v>201</v>
+        <v>2135</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>帶量突破20日高點</t>
+          <t>無明顯異常</t>
         </is>
       </c>
       <c r="L24" t="n">
-        <v>-1465366</v>
+        <v>-2572029</v>
       </c>
       <c r="M24" t="n">
-        <v>-160620</v>
+        <v>-2116239</v>
       </c>
       <c r="N24" t="n">
-        <v>-5984174</v>
+        <v>-3083433</v>
       </c>
       <c r="O24" t="n">
-        <v>5074162</v>
+        <v>-10178055</v>
       </c>
       <c r="P24" t="n">
-        <v>35</v>
-      </c>
-      <c r="Q24" t="inlineStr">
+        <v>-9521827</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>-8788853</v>
+      </c>
+      <c r="R24" t="n">
+        <v>-17296342</v>
+      </c>
+      <c r="S24" t="n">
+        <v>-51109009</v>
+      </c>
+      <c r="T24" t="n">
+        <v>6429500</v>
+      </c>
+      <c r="U24" t="n">
+        <v>5964652</v>
+      </c>
+      <c r="V24" t="n">
+        <v>12561152</v>
+      </c>
+      <c r="W24" t="n">
+        <v>40136470</v>
+      </c>
+      <c r="X24" t="n">
+        <v>520298</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>707962</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>1651757</v>
+      </c>
+      <c r="AA24" t="n">
+        <v>794484</v>
+      </c>
+      <c r="AB24" t="n">
+        <v>25</v>
+      </c>
+      <c r="AC24" t="inlineStr">
         <is>
           <t>⚠️整理</t>
         </is>
       </c>
-      <c r="R24" t="inlineStr">
+      <c r="AD24" t="inlineStr">
         <is>
           <t>整理觀察</t>
         </is>
       </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、爆量、突破20日高點、帶量突破20日高點</t>
-        </is>
-      </c>
-      <c r="T24" t="inlineStr">
-        <is>
-          <t>法人連續偏賣、中期買超轉短線賣壓、5日法人明顯賣超</t>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>整理觀察：站上5日線、多頭排列、爆量、突破20日高點、帶量突破20日高點、法人連續偏賣、中期買超轉短線賣壓、5日法人明顯賣超。多空訊號混合，建議降低追價衝動。</t>
+      <c r="AE24" t="inlineStr">
+        <is>
+          <t>站上5日線、多頭排列、黃金交叉、量能溫和放大</t>
+        </is>
+      </c>
+      <c r="AF24" t="inlineStr">
+        <is>
+          <t>法人連續偏賣、5日法人明顯賣超、投信買外資賣</t>
+        </is>
+      </c>
+      <c r="AG24" t="inlineStr">
+        <is>
+          <t>整理觀察：站上5日線、多頭排列、黃金交叉、量能溫和放大、法人連續偏賣、5日法人明顯賣超、投信買外資賣。多空訊號混合，建議降低追價衝動。</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>6488.TWO</t>
+          <t>2344.TW</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>環球晶</t>
+          <t>華邦電</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>866</v>
+        <v>141</v>
       </c>
       <c r="D25" t="n">
-        <v>742</v>
+        <v>124.8</v>
       </c>
       <c r="E25" t="n">
-        <v>732.1</v>
+        <v>125.75</v>
       </c>
       <c r="F25" t="n">
-        <v>711.25</v>
+        <v>114.91</v>
       </c>
       <c r="G25" t="n">
-        <v>2958000</v>
+        <v>336105421</v>
       </c>
       <c r="H25" t="n">
-        <v>4678000</v>
+        <v>249474700</v>
       </c>
       <c r="I25" t="n">
-        <v>866</v>
+        <v>141</v>
       </c>
       <c r="J25" t="n">
-        <v>534</v>
+        <v>88.8</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -2427,80 +3315,116 @@
         </is>
       </c>
       <c r="L25" t="n">
-        <v>-261357</v>
+        <v>-11962552</v>
       </c>
       <c r="M25" t="n">
-        <v>-3141303</v>
+        <v>40167238</v>
       </c>
       <c r="N25" t="n">
-        <v>-4610982</v>
+        <v>-4889605</v>
       </c>
       <c r="O25" t="n">
-        <v>-4787133</v>
+        <v>68676281</v>
       </c>
       <c r="P25" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>❌避開</t>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>觀望</t>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、量能未放大、突破20日高點</t>
-        </is>
-      </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t>法人連續偏賣、5日法人明顯賣超</t>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr">
-        <is>
-          <t>風險偏高：站上5日線、多頭排列、量能未放大、突破20日高點、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
+        <v>-19138371</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>32303633</v>
+      </c>
+      <c r="R25" t="n">
+        <v>-18031163</v>
+      </c>
+      <c r="S25" t="n">
+        <v>-12020795</v>
+      </c>
+      <c r="T25" t="n">
+        <v>7462000</v>
+      </c>
+      <c r="U25" t="n">
+        <v>6270969</v>
+      </c>
+      <c r="V25" t="n">
+        <v>10656969</v>
+      </c>
+      <c r="W25" t="n">
+        <v>76451043</v>
+      </c>
+      <c r="X25" t="n">
+        <v>-286181</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>1592636</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>2484589</v>
+      </c>
+      <c r="AA25" t="n">
+        <v>4246033</v>
+      </c>
+      <c r="AB25" t="n">
+        <v>25</v>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>⚠️整理</t>
+        </is>
+      </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>整理觀察</t>
+        </is>
+      </c>
+      <c r="AE25" t="inlineStr">
+        <is>
+          <t>站上5日線、量能溫和放大、突破20日高點</t>
+        </is>
+      </c>
+      <c r="AF25" t="inlineStr">
+        <is>
+          <t>5日法人明顯賣超、投信買外資賣</t>
+        </is>
+      </c>
+      <c r="AG25" t="inlineStr">
+        <is>
+          <t>整理觀察：站上5日線、量能溫和放大、突破20日高點、5日法人明顯賣超、投信買外資賣。多空訊號混合，建議降低追價衝動。</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>6669.TW</t>
+          <t>3163.TWO</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>緯穎</t>
+          <t>波若威</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>5280</v>
+        <v>1220</v>
       </c>
       <c r="D26" t="n">
-        <v>5334</v>
+        <v>1114.4</v>
       </c>
       <c r="E26" t="n">
-        <v>5278</v>
+        <v>1037.7</v>
       </c>
       <c r="F26" t="n">
-        <v>5144.75</v>
+        <v>1072.35</v>
       </c>
       <c r="G26" t="n">
-        <v>2655826</v>
+        <v>4415000</v>
       </c>
       <c r="H26" t="n">
-        <v>2172103</v>
+        <v>3736800</v>
       </c>
       <c r="I26" t="n">
-        <v>5880</v>
+        <v>1300</v>
       </c>
       <c r="J26" t="n">
-        <v>4615</v>
+        <v>865</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -2508,161 +3432,233 @@
         </is>
       </c>
       <c r="L26" t="n">
-        <v>49559</v>
+        <v>78870</v>
       </c>
       <c r="M26" t="n">
-        <v>97025</v>
+        <v>-1139380</v>
       </c>
       <c r="N26" t="n">
-        <v>-160824</v>
+        <v>-1176252</v>
       </c>
       <c r="O26" t="n">
-        <v>-364679</v>
+        <v>-1740259</v>
       </c>
       <c r="P26" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>❌避開</t>
-        </is>
-      </c>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>觀望</t>
-        </is>
-      </c>
-      <c r="S26" t="inlineStr">
-        <is>
-          <t>跌破5日線、多頭排列、量能溫和放大</t>
-        </is>
-      </c>
-      <c r="T26" t="inlineStr">
-        <is>
-          <t>短線籌碼止穩、5日法人賣超</t>
-        </is>
-      </c>
-      <c r="U26" t="inlineStr">
-        <is>
-          <t>風險偏高：跌破5日線、多頭排列、量能溫和放大、短線籌碼止穩、5日法人賣超。目前不適合積極追蹤，等待結構改善。</t>
+        <v>-73248</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>-1970174</v>
+      </c>
+      <c r="R26" t="n">
+        <v>-2217164</v>
+      </c>
+      <c r="S26" t="n">
+        <v>-2350595</v>
+      </c>
+      <c r="T26" t="n">
+        <v>210000</v>
+      </c>
+      <c r="U26" t="n">
+        <v>871000</v>
+      </c>
+      <c r="V26" t="n">
+        <v>1046000</v>
+      </c>
+      <c r="W26" t="n">
+        <v>567000</v>
+      </c>
+      <c r="X26" t="n">
+        <v>-57882</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>-40206</v>
+      </c>
+      <c r="Z26" t="n">
+        <v>-5088</v>
+      </c>
+      <c r="AA26" t="n">
+        <v>43336</v>
+      </c>
+      <c r="AB26" t="n">
+        <v>25</v>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>⚠️整理</t>
+        </is>
+      </c>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>整理觀察</t>
+        </is>
+      </c>
+      <c r="AE26" t="inlineStr">
+        <is>
+          <t>站上5日線、黃金交叉、量能溫和放大</t>
+        </is>
+      </c>
+      <c r="AF26" t="inlineStr">
+        <is>
+          <t>5日法人明顯賣超、投信買外資賣</t>
+        </is>
+      </c>
+      <c r="AG26" t="inlineStr">
+        <is>
+          <t>整理觀察：站上5日線、黃金交叉、量能溫和放大、5日法人明顯賣超、投信買外資賣。多空訊號混合，建議降低追價衝動。</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>3163.TWO</t>
+          <t>6239.TW</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>波若威</t>
+          <t>力成</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1220</v>
+        <v>342</v>
       </c>
       <c r="D27" t="n">
-        <v>1114.4</v>
+        <v>285.6</v>
       </c>
       <c r="E27" t="n">
-        <v>1037.7</v>
+        <v>261.4</v>
       </c>
       <c r="F27" t="n">
-        <v>1072.35</v>
+        <v>241.47</v>
       </c>
       <c r="G27" t="n">
-        <v>4415000</v>
+        <v>57938700</v>
       </c>
       <c r="H27" t="n">
-        <v>3736800</v>
+        <v>22861322</v>
       </c>
       <c r="I27" t="n">
-        <v>1300</v>
+        <v>342</v>
       </c>
       <c r="J27" t="n">
-        <v>865</v>
+        <v>201</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>無明顯異常</t>
+          <t>帶量突破20日高點</t>
         </is>
       </c>
       <c r="L27" t="n">
-        <v>-1014980</v>
+        <v>-1834154</v>
       </c>
       <c r="M27" t="n">
-        <v>-1037784</v>
+        <v>-4443864</v>
       </c>
       <c r="N27" t="n">
-        <v>-1279466</v>
+        <v>-2363562</v>
       </c>
       <c r="O27" t="n">
-        <v>-1723078</v>
+        <v>8629303</v>
       </c>
       <c r="P27" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q27" t="inlineStr">
+        <v>-2734302</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>-3531935</v>
+      </c>
+      <c r="R27" t="n">
+        <v>-4279508</v>
+      </c>
+      <c r="S27" t="n">
+        <v>4990232</v>
+      </c>
+      <c r="T27" t="n">
+        <v>94000</v>
+      </c>
+      <c r="U27" t="n">
+        <v>-1715000</v>
+      </c>
+      <c r="V27" t="n">
+        <v>-408000</v>
+      </c>
+      <c r="W27" t="n">
+        <v>-455184</v>
+      </c>
+      <c r="X27" t="n">
+        <v>806148</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>803071</v>
+      </c>
+      <c r="Z27" t="n">
+        <v>2323946</v>
+      </c>
+      <c r="AA27" t="n">
+        <v>4094255</v>
+      </c>
+      <c r="AB27" t="n">
+        <v>15</v>
+      </c>
+      <c r="AC27" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="R27" t="inlineStr">
+      <c r="AD27" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>站上5日線、黃金交叉、量能溫和放大</t>
-        </is>
-      </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>法人連續偏賣、5日法人明顯賣超</t>
-        </is>
-      </c>
-      <c r="U27" t="inlineStr">
-        <is>
-          <t>風險偏高：站上5日線、黃金交叉、量能溫和放大、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
+      <c r="AE27" t="inlineStr">
+        <is>
+          <t>站上5日線、多頭排列、爆量、突破20日高點、帶量突破20日高點</t>
+        </is>
+      </c>
+      <c r="AF27" t="inlineStr">
+        <is>
+          <t>法人連續偏賣、中期買超轉短線賣壓、5日法人明顯賣超、外資投信同步賣超</t>
+        </is>
+      </c>
+      <c r="AG27" t="inlineStr">
+        <is>
+          <t>風險偏高：站上5日線、多頭排列、爆量、突破20日高點、帶量突破20日高點、法人連續偏賣、中期買超轉短線賣壓、5日法人明顯賣超、外資投信同步賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2303.TW</t>
+          <t>4960.TW</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>聯電</t>
+          <t>誠美材</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>130.5</v>
+        <v>34.25</v>
       </c>
       <c r="D28" t="n">
-        <v>118.7</v>
+        <v>35.13</v>
       </c>
       <c r="E28" t="n">
-        <v>113.39</v>
+        <v>34.6</v>
       </c>
       <c r="F28" t="n">
-        <v>100.19</v>
+        <v>37.35</v>
       </c>
       <c r="G28" t="n">
-        <v>291896012</v>
+        <v>11138430</v>
       </c>
       <c r="H28" t="n">
-        <v>252641517</v>
+        <v>16177150</v>
       </c>
       <c r="I28" t="n">
-        <v>133.5</v>
+        <v>44.05</v>
       </c>
       <c r="J28" t="n">
-        <v>71.3</v>
+        <v>31.1</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
@@ -2670,80 +3666,116 @@
         </is>
       </c>
       <c r="L28" t="n">
-        <v>32836623</v>
+        <v>2800000</v>
       </c>
       <c r="M28" t="n">
-        <v>-1979065</v>
+        <v>-2768167</v>
       </c>
       <c r="N28" t="n">
-        <v>-21222223</v>
+        <v>2773001</v>
       </c>
       <c r="O28" t="n">
-        <v>49323216</v>
+        <v>11403137</v>
       </c>
       <c r="P28" t="n">
+        <v>2798000</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>-2599000</v>
+      </c>
+      <c r="R28" t="n">
+        <v>2771000</v>
+      </c>
+      <c r="S28" t="n">
+        <v>11617136</v>
+      </c>
+      <c r="T28" t="n">
         <v>0</v>
       </c>
-      <c r="Q28" t="inlineStr">
+      <c r="U28" t="n">
+        <v>0</v>
+      </c>
+      <c r="V28" t="n">
+        <v>0</v>
+      </c>
+      <c r="W28" t="n">
+        <v>0</v>
+      </c>
+      <c r="X28" t="n">
+        <v>2000</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>-169167</v>
+      </c>
+      <c r="Z28" t="n">
+        <v>2001</v>
+      </c>
+      <c r="AA28" t="n">
+        <v>-213999</v>
+      </c>
+      <c r="AB28" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC28" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="R28" t="inlineStr">
+      <c r="AD28" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="S28" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、量能溫和放大</t>
-        </is>
-      </c>
-      <c r="T28" t="inlineStr">
-        <is>
-          <t>中期買超轉短線賣壓、5日法人明顯賣超</t>
-        </is>
-      </c>
-      <c r="U28" t="inlineStr">
-        <is>
-          <t>風險偏高：站上5日線、多頭排列、量能溫和放大、中期買超轉短線賣壓、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
+      <c r="AE28" t="inlineStr">
+        <is>
+          <t>跌破5日線、量能未放大</t>
+        </is>
+      </c>
+      <c r="AF28" t="inlineStr">
+        <is>
+          <t>5日法人明顯買超</t>
+        </is>
+      </c>
+      <c r="AG28" t="inlineStr">
+        <is>
+          <t>風險偏高：跌破5日線、量能未放大、5日法人明顯買超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2408.TW</t>
+          <t>6488.TWO</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>南亞科</t>
+          <t>環球晶</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>303.5</v>
+        <v>866</v>
       </c>
       <c r="D29" t="n">
-        <v>295.6</v>
+        <v>742</v>
       </c>
       <c r="E29" t="n">
-        <v>303.1</v>
+        <v>732.1</v>
       </c>
       <c r="F29" t="n">
-        <v>283.88</v>
+        <v>711.25</v>
       </c>
       <c r="G29" t="n">
-        <v>152949355</v>
+        <v>2958000</v>
       </c>
       <c r="H29" t="n">
-        <v>148065232</v>
+        <v>4678000</v>
       </c>
       <c r="I29" t="n">
-        <v>353</v>
+        <v>866</v>
       </c>
       <c r="J29" t="n">
-        <v>214.5</v>
+        <v>534</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
@@ -2751,80 +3783,116 @@
         </is>
       </c>
       <c r="L29" t="n">
-        <v>-13921163</v>
+        <v>-541871</v>
       </c>
       <c r="M29" t="n">
-        <v>-14185405</v>
+        <v>-2561156</v>
       </c>
       <c r="N29" t="n">
-        <v>-47727411</v>
+        <v>-4480928</v>
       </c>
       <c r="O29" t="n">
-        <v>-49157826</v>
+        <v>-5069064</v>
       </c>
       <c r="P29" t="n">
-        <v>-25</v>
-      </c>
-      <c r="Q29" t="inlineStr">
+        <v>-566747</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>-3254183</v>
+      </c>
+      <c r="R29" t="n">
+        <v>-4533384</v>
+      </c>
+      <c r="S29" t="n">
+        <v>-6369986</v>
+      </c>
+      <c r="T29" t="n">
+        <v>-84038</v>
+      </c>
+      <c r="U29" t="n">
+        <v>-295650</v>
+      </c>
+      <c r="V29" t="n">
+        <v>-946650</v>
+      </c>
+      <c r="W29" t="n">
+        <v>-269880</v>
+      </c>
+      <c r="X29" t="n">
+        <v>108914</v>
+      </c>
+      <c r="Y29" t="n">
+        <v>988677</v>
+      </c>
+      <c r="Z29" t="n">
+        <v>999106</v>
+      </c>
+      <c r="AA29" t="n">
+        <v>1570802</v>
+      </c>
+      <c r="AB29" t="n">
+        <v>-5</v>
+      </c>
+      <c r="AC29" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="R29" t="inlineStr">
+      <c r="AD29" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="S29" t="inlineStr">
-        <is>
-          <t>站上5日線、量能溫和放大</t>
-        </is>
-      </c>
-      <c r="T29" t="inlineStr">
-        <is>
-          <t>法人連續偏賣、5日法人明顯賣超</t>
-        </is>
-      </c>
-      <c r="U29" t="inlineStr">
-        <is>
-          <t>風險偏高：站上5日線、量能溫和放大、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
+      <c r="AE29" t="inlineStr">
+        <is>
+          <t>站上5日線、多頭排列、量能未放大、突破20日高點</t>
+        </is>
+      </c>
+      <c r="AF29" t="inlineStr">
+        <is>
+          <t>法人連續偏賣、5日法人明顯賣超、外資投信同步賣超</t>
+        </is>
+      </c>
+      <c r="AG29" t="inlineStr">
+        <is>
+          <t>風險偏高：站上5日線、多頭排列、量能未放大、突破20日高點、法人連續偏賣、5日法人明顯賣超、外資投信同步賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>8046.TW</t>
+          <t>2303.TW</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>南電</t>
+          <t>聯電</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>922</v>
+        <v>130.5</v>
       </c>
       <c r="D30" t="n">
-        <v>888.2</v>
+        <v>118.7</v>
       </c>
       <c r="E30" t="n">
-        <v>854.3</v>
+        <v>113.39</v>
       </c>
       <c r="F30" t="n">
-        <v>896.4</v>
+        <v>100.19</v>
       </c>
       <c r="G30" t="n">
-        <v>24438087</v>
+        <v>291896012</v>
       </c>
       <c r="H30" t="n">
-        <v>20893593</v>
+        <v>252641517</v>
       </c>
       <c r="I30" t="n">
-        <v>1035</v>
+        <v>133.5</v>
       </c>
       <c r="J30" t="n">
-        <v>765</v>
+        <v>71.3</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
@@ -2832,80 +3900,116 @@
         </is>
       </c>
       <c r="L30" t="n">
-        <v>-8905954</v>
+        <v>-24732790</v>
       </c>
       <c r="M30" t="n">
-        <v>-4812274</v>
+        <v>-79198141</v>
       </c>
       <c r="N30" t="n">
-        <v>-4509560</v>
+        <v>-84281268</v>
       </c>
       <c r="O30" t="n">
-        <v>-8787097</v>
+        <v>-88381049</v>
       </c>
       <c r="P30" t="n">
-        <v>-25</v>
-      </c>
-      <c r="Q30" t="inlineStr">
+        <v>-45921195</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>-76267503</v>
+      </c>
+      <c r="R30" t="n">
+        <v>-78400331</v>
+      </c>
+      <c r="S30" t="n">
+        <v>-182437864</v>
+      </c>
+      <c r="T30" t="n">
+        <v>20707132</v>
+      </c>
+      <c r="U30" t="n">
+        <v>-4178019</v>
+      </c>
+      <c r="V30" t="n">
+        <v>-9430887</v>
+      </c>
+      <c r="W30" t="n">
+        <v>94794673</v>
+      </c>
+      <c r="X30" t="n">
+        <v>481273</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>1247381</v>
+      </c>
+      <c r="Z30" t="n">
+        <v>3549950</v>
+      </c>
+      <c r="AA30" t="n">
+        <v>-737858</v>
+      </c>
+      <c r="AB30" t="n">
+        <v>-20</v>
+      </c>
+      <c r="AC30" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="R30" t="inlineStr">
+      <c r="AD30" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="S30" t="inlineStr">
-        <is>
-          <t>站上5日線、量能溫和放大</t>
-        </is>
-      </c>
-      <c r="T30" t="inlineStr">
-        <is>
-          <t>法人連續偏賣、5日法人明顯賣超</t>
-        </is>
-      </c>
-      <c r="U30" t="inlineStr">
-        <is>
-          <t>風險偏高：站上5日線、量能溫和放大、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
+      <c r="AE30" t="inlineStr">
+        <is>
+          <t>站上5日線、多頭排列、量能溫和放大</t>
+        </is>
+      </c>
+      <c r="AF30" t="inlineStr">
+        <is>
+          <t>法人連續偏賣、5日法人明顯賣超、外資投信同步賣超</t>
+        </is>
+      </c>
+      <c r="AG30" t="inlineStr">
+        <is>
+          <t>風險偏高：站上5日線、多頭排列、量能溫和放大、法人連續偏賣、5日法人明顯賣超、外資投信同步賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>6285.TW</t>
+          <t>2408.TW</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>啟碁</t>
+          <t>南亞科</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>304.5</v>
+        <v>303.5</v>
       </c>
       <c r="D31" t="n">
-        <v>291.6</v>
+        <v>295.6</v>
       </c>
       <c r="E31" t="n">
-        <v>282.85</v>
+        <v>303.1</v>
       </c>
       <c r="F31" t="n">
-        <v>260.6</v>
+        <v>281.4</v>
       </c>
       <c r="G31" t="n">
-        <v>21738108</v>
+        <v>152949355</v>
       </c>
       <c r="H31" t="n">
-        <v>31212343</v>
+        <v>148065232</v>
       </c>
       <c r="I31" t="n">
-        <v>317</v>
+        <v>353</v>
       </c>
       <c r="J31" t="n">
-        <v>208.5</v>
+        <v>198.5</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
@@ -2913,80 +4017,116 @@
         </is>
       </c>
       <c r="L31" t="n">
-        <v>-5937776</v>
+        <v>-7167551</v>
       </c>
       <c r="M31" t="n">
-        <v>-4853792</v>
+        <v>-6915479</v>
       </c>
       <c r="N31" t="n">
-        <v>-11223101</v>
+        <v>-14599344</v>
       </c>
       <c r="O31" t="n">
-        <v>1863302</v>
+        <v>-52051868</v>
       </c>
       <c r="P31" t="n">
-        <v>-35</v>
-      </c>
-      <c r="Q31" t="inlineStr">
+        <v>2181497</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>1871943</v>
+      </c>
+      <c r="R31" t="n">
+        <v>2834419</v>
+      </c>
+      <c r="S31" t="n">
+        <v>-21992353</v>
+      </c>
+      <c r="T31" t="n">
+        <v>-8258000</v>
+      </c>
+      <c r="U31" t="n">
+        <v>-8507165</v>
+      </c>
+      <c r="V31" t="n">
+        <v>-16981165</v>
+      </c>
+      <c r="W31" t="n">
+        <v>-26831509</v>
+      </c>
+      <c r="X31" t="n">
+        <v>-1091048</v>
+      </c>
+      <c r="Y31" t="n">
+        <v>-280257</v>
+      </c>
+      <c r="Z31" t="n">
+        <v>-452598</v>
+      </c>
+      <c r="AA31" t="n">
+        <v>-3228006</v>
+      </c>
+      <c r="AB31" t="n">
+        <v>-25</v>
+      </c>
+      <c r="AC31" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="R31" t="inlineStr">
+      <c r="AD31" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="S31" t="inlineStr">
-        <is>
-          <t>站上5日線、多頭排列、量能未放大</t>
-        </is>
-      </c>
-      <c r="T31" t="inlineStr">
-        <is>
-          <t>法人連續偏賣、中期買超轉短線賣壓、5日法人明顯賣超</t>
-        </is>
-      </c>
-      <c r="U31" t="inlineStr">
-        <is>
-          <t>風險偏高：站上5日線、多頭排列、量能未放大、法人連續偏賣、中期買超轉短線賣壓、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
+      <c r="AE31" t="inlineStr">
+        <is>
+          <t>站上5日線、量能溫和放大</t>
+        </is>
+      </c>
+      <c r="AF31" t="inlineStr">
+        <is>
+          <t>法人連續偏賣、5日法人明顯賣超、外資買投信賣</t>
+        </is>
+      </c>
+      <c r="AG31" t="inlineStr">
+        <is>
+          <t>風險偏高：站上5日線、量能溫和放大、法人連續偏賣、5日法人明顯賣超、外資買投信賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>4960.TW</t>
+          <t>3711.TW</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>誠美材</t>
+          <t>日月光投控</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>34.25</v>
+        <v>478</v>
       </c>
       <c r="D32" t="n">
-        <v>35.13</v>
+        <v>490.7</v>
       </c>
       <c r="E32" t="n">
-        <v>34.6</v>
+        <v>475.85</v>
       </c>
       <c r="F32" t="n">
-        <v>37.35</v>
+        <v>436.95</v>
       </c>
       <c r="G32" t="n">
-        <v>11138430</v>
+        <v>36584546</v>
       </c>
       <c r="H32" t="n">
-        <v>16177150</v>
+        <v>27861072</v>
       </c>
       <c r="I32" t="n">
-        <v>44.05</v>
+        <v>523</v>
       </c>
       <c r="J32" t="n">
-        <v>31.1</v>
+        <v>344.5</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
@@ -2994,43 +4134,79 @@
         </is>
       </c>
       <c r="L32" t="n">
-        <v>-1669951</v>
+        <v>-5830786</v>
       </c>
       <c r="M32" t="n">
-        <v>-4496950</v>
+        <v>-1856284</v>
       </c>
       <c r="N32" t="n">
-        <v>-8242967</v>
+        <v>-5316375</v>
       </c>
       <c r="O32" t="n">
-        <v>-5221995</v>
+        <v>-18584918</v>
       </c>
       <c r="P32" t="n">
-        <v>-75</v>
-      </c>
-      <c r="Q32" t="inlineStr">
+        <v>-5948511</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>-2968809</v>
+      </c>
+      <c r="R32" t="n">
+        <v>-6389494</v>
+      </c>
+      <c r="S32" t="n">
+        <v>-22409660</v>
+      </c>
+      <c r="T32" t="n">
+        <v>262000</v>
+      </c>
+      <c r="U32" t="n">
+        <v>1510683</v>
+      </c>
+      <c r="V32" t="n">
+        <v>1749683</v>
+      </c>
+      <c r="W32" t="n">
+        <v>4998304</v>
+      </c>
+      <c r="X32" t="n">
+        <v>-144275</v>
+      </c>
+      <c r="Y32" t="n">
+        <v>-398158</v>
+      </c>
+      <c r="Z32" t="n">
+        <v>-676564</v>
+      </c>
+      <c r="AA32" t="n">
+        <v>-1173562</v>
+      </c>
+      <c r="AB32" t="n">
+        <v>-40</v>
+      </c>
+      <c r="AC32" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="R32" t="inlineStr">
+      <c r="AD32" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t>跌破5日線、量能未放大</t>
-        </is>
-      </c>
-      <c r="T32" t="inlineStr">
-        <is>
-          <t>法人連續偏賣、5日法人明顯賣超</t>
-        </is>
-      </c>
-      <c r="U32" t="inlineStr">
-        <is>
-          <t>風險偏高：跌破5日線、量能未放大、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
+      <c r="AE32" t="inlineStr">
+        <is>
+          <t>跌破5日線、多頭排列、量能溫和放大</t>
+        </is>
+      </c>
+      <c r="AF32" t="inlineStr">
+        <is>
+          <t>法人連續偏賣、5日法人明顯賣超、投信買外資賣</t>
+        </is>
+      </c>
+      <c r="AG32" t="inlineStr">
+        <is>
+          <t>風險偏高：跌破5日線、多頭排列、量能溫和放大、法人連續偏賣、5日法人明顯賣超、投信買外資賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
@@ -3075,43 +4251,79 @@
         </is>
       </c>
       <c r="L33" t="n">
-        <v>-352405</v>
+        <v>-467151</v>
       </c>
       <c r="M33" t="n">
-        <v>-707137</v>
+        <v>-779449</v>
       </c>
       <c r="N33" t="n">
-        <v>-868509</v>
+        <v>-1431458</v>
       </c>
       <c r="O33" t="n">
-        <v>-2148559</v>
+        <v>-2655109</v>
       </c>
       <c r="P33" t="n">
-        <v>-75</v>
-      </c>
-      <c r="Q33" t="inlineStr">
+        <v>-190195</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>-247868</v>
+      </c>
+      <c r="R33" t="n">
+        <v>-528542</v>
+      </c>
+      <c r="S33" t="n">
+        <v>-1615246</v>
+      </c>
+      <c r="T33" t="n">
+        <v>-264617</v>
+      </c>
+      <c r="U33" t="n">
+        <v>-524617</v>
+      </c>
+      <c r="V33" t="n">
+        <v>-879117</v>
+      </c>
+      <c r="W33" t="n">
+        <v>-828848</v>
+      </c>
+      <c r="X33" t="n">
+        <v>-12339</v>
+      </c>
+      <c r="Y33" t="n">
+        <v>-6964</v>
+      </c>
+      <c r="Z33" t="n">
+        <v>-23799</v>
+      </c>
+      <c r="AA33" t="n">
+        <v>-211015</v>
+      </c>
+      <c r="AB33" t="n">
+        <v>-95</v>
+      </c>
+      <c r="AC33" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="R33" t="inlineStr">
+      <c r="AD33" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="S33" t="inlineStr">
+      <c r="AE33" t="inlineStr">
         <is>
           <t>跌破5日線、量能未放大</t>
         </is>
       </c>
-      <c r="T33" t="inlineStr">
-        <is>
-          <t>法人連續偏賣、5日法人明顯賣超</t>
-        </is>
-      </c>
-      <c r="U33" t="inlineStr">
-        <is>
-          <t>風險偏高：跌破5日線、量能未放大、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
+      <c r="AF33" t="inlineStr">
+        <is>
+          <t>法人連續偏賣、5日法人明顯賣超、外資投信同步賣超</t>
+        </is>
+      </c>
+      <c r="AG33" t="inlineStr">
+        <is>
+          <t>風險偏高：跌破5日線、量能未放大、法人連續偏賣、5日法人明顯賣超、外資投信同步賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
reweight deeptrend score and add score change
</commit_message>
<xml_diff>
--- a/output/stock_analysis_result.xlsx
+++ b/output/stock_analysis_result.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG69"/>
+  <dimension ref="A1:AN69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -559,25 +559,60 @@
       </c>
       <c r="AC1" t="inlineStr">
         <is>
+          <t>DeepTrend分數</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>技術面分數</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>籌碼分數</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>量價分數</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>前次分數</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>分數變化</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>分數變化率</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
           <t>狀態</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>綜合判斷</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>技術面</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>籌碼面</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>AI評語</t>
         </is>
@@ -672,31 +707,46 @@
         <v>13852</v>
       </c>
       <c r="AB2" t="n">
-        <v>130</v>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>🔥強勢</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>強勢觀察</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr">
+        <v>52</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>52</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>70</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>60</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>👀觀察</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>偏多觀察</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
         <is>
           <t>站上5日線、多頭排列、量能溫和放大、接近20日高點</t>
         </is>
       </c>
-      <c r="AF2" t="inlineStr">
+      <c r="AM2" t="inlineStr">
         <is>
           <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
-      <c r="AG2" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、量能溫和放大、接近20日高點、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>偏多觀察：站上5日線、多頭排列、量能溫和放大、接近20日高點、法人連續偏買、5日法人明顯買超。條件不差，適合等待拉回或突破確認。</t>
         </is>
       </c>
     </row>
@@ -789,31 +839,46 @@
         <v>1307747</v>
       </c>
       <c r="AB3" t="n">
-        <v>115</v>
-      </c>
-      <c r="AC3" t="inlineStr">
-        <is>
-          <t>🔥強勢</t>
-        </is>
-      </c>
-      <c r="AD3" t="inlineStr">
-        <is>
-          <t>強勢觀察</t>
-        </is>
-      </c>
-      <c r="AE3" t="inlineStr">
+        <v>46</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>46</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>55</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>60</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>⚠️整理</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>整理觀察</t>
+        </is>
+      </c>
+      <c r="AL3" t="inlineStr">
         <is>
           <t>站上5日線、多頭排列、量能溫和放大</t>
         </is>
       </c>
-      <c r="AF3" t="inlineStr">
+      <c r="AM3" t="inlineStr">
         <is>
           <t>法人連續偏買、5日法人明顯買超、外資買投信賣</t>
         </is>
       </c>
-      <c r="AG3" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、量能溫和放大、法人連續偏買、5日法人明顯買超、外資買投信賣。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t>整理觀察：站上5日線、多頭排列、量能溫和放大、法人連續偏買、5日法人明顯買超、外資買投信賣。多空訊號混合，建議降低追價衝動。</t>
         </is>
       </c>
     </row>
@@ -906,31 +971,46 @@
         <v>2399716</v>
       </c>
       <c r="AB4" t="n">
-        <v>105</v>
-      </c>
-      <c r="AC4" t="inlineStr">
-        <is>
-          <t>🔥強勢</t>
-        </is>
-      </c>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>強勢觀察</t>
-        </is>
-      </c>
-      <c r="AE4" t="inlineStr">
+        <v>42</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>42</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>45</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>60</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG4" t="inlineStr"/>
+      <c r="AH4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr"/>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>⚠️整理</t>
+        </is>
+      </c>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>整理觀察</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
         <is>
           <t>站上5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF4" t="inlineStr">
+      <c r="AM4" t="inlineStr">
         <is>
           <t>法人連續偏買、5日法人明顯買超、外資買投信賣</t>
         </is>
       </c>
-      <c r="AG4" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、量能未放大、法人連續偏買、5日法人明顯買超、外資買投信賣。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>整理觀察：站上5日線、多頭排列、量能未放大、法人連續偏買、5日法人明顯買超、外資買投信賣。多空訊號混合，建議降低追價衝動。</t>
         </is>
       </c>
     </row>
@@ -1023,31 +1103,46 @@
         <v>59816079</v>
       </c>
       <c r="AB5" t="n">
-        <v>95</v>
-      </c>
-      <c r="AC5" t="inlineStr">
-        <is>
-          <t>🔥強勢</t>
-        </is>
-      </c>
-      <c r="AD5" t="inlineStr">
-        <is>
-          <t>強勢觀察</t>
-        </is>
-      </c>
-      <c r="AE5" t="inlineStr">
+        <v>38</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>38</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>15</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>80</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>⚠️整理</t>
+        </is>
+      </c>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>整理觀察</t>
+        </is>
+      </c>
+      <c r="AL5" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能溫和放大</t>
         </is>
       </c>
-      <c r="AF5" t="inlineStr">
+      <c r="AM5" t="inlineStr">
         <is>
           <t>法人連續偏買、5日法人明顯買超、外資投信同步買超</t>
         </is>
       </c>
-      <c r="AG5" t="inlineStr">
-        <is>
-          <t>強勢偏多：跌破5日線、多頭排列、量能溫和放大、法人連續偏買、5日法人明顯買超、外資投信同步買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t>整理觀察：跌破5日線、多頭排列、量能溫和放大、法人連續偏買、5日法人明顯買超、外資投信同步買超。多空訊號混合，建議降低追價衝動。</t>
         </is>
       </c>
     </row>
@@ -1140,31 +1235,46 @@
         <v>3273117</v>
       </c>
       <c r="AB6" t="n">
-        <v>90</v>
-      </c>
-      <c r="AC6" t="inlineStr">
-        <is>
-          <t>🔥強勢</t>
-        </is>
-      </c>
-      <c r="AD6" t="inlineStr">
-        <is>
-          <t>強勢觀察</t>
-        </is>
-      </c>
-      <c r="AE6" t="inlineStr">
+        <v>36</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>36</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>60</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>30</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr"/>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>⚠️整理</t>
+        </is>
+      </c>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>整理觀察</t>
+        </is>
+      </c>
+      <c r="AL6" t="inlineStr">
         <is>
           <t>站上5日線、多頭排列、量能未放大、接近20日高點</t>
         </is>
       </c>
-      <c r="AF6" t="inlineStr">
+      <c r="AM6" t="inlineStr">
         <is>
           <t>5日法人明顯買超、投信買外資賣</t>
         </is>
       </c>
-      <c r="AG6" t="inlineStr">
-        <is>
-          <t>強勢偏多：站上5日線、多頭排列、量能未放大、接近20日高點、5日法人明顯買超、投信買外資賣。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>整理觀察：站上5日線、多頭排列、量能未放大、接近20日高點、5日法人明顯買超、投信買外資賣。多空訊號混合，建議降低追價衝動。</t>
         </is>
       </c>
     </row>
@@ -1257,31 +1367,46 @@
         <v>1352749</v>
       </c>
       <c r="AB7" t="n">
-        <v>85</v>
-      </c>
-      <c r="AC7" t="inlineStr">
-        <is>
-          <t>🔥強勢</t>
-        </is>
-      </c>
-      <c r="AD7" t="inlineStr">
-        <is>
-          <t>強勢觀察</t>
-        </is>
-      </c>
-      <c r="AE7" t="inlineStr">
+        <v>34</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>34</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>80</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>⚠️整理</t>
+        </is>
+      </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t>整理觀察</t>
+        </is>
+      </c>
+      <c r="AL7" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF7" t="inlineStr">
+      <c r="AM7" t="inlineStr">
         <is>
           <t>法人連續偏買、5日法人明顯買超、外資投信同步買超</t>
         </is>
       </c>
-      <c r="AG7" t="inlineStr">
-        <is>
-          <t>強勢偏多：跌破5日線、多頭排列、量能未放大、法人連續偏買、5日法人明顯買超、外資投信同步買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t>整理觀察：跌破5日線、多頭排列、量能未放大、法人連續偏買、5日法人明顯買超、外資投信同步買超。多空訊號混合，建議降低追價衝動。</t>
         </is>
       </c>
     </row>
@@ -1374,31 +1499,46 @@
         <v>208358546</v>
       </c>
       <c r="AB8" t="n">
-        <v>75</v>
-      </c>
-      <c r="AC8" t="inlineStr">
-        <is>
-          <t>🔥強勢</t>
-        </is>
-      </c>
-      <c r="AD8" t="inlineStr">
-        <is>
-          <t>強勢觀察</t>
-        </is>
-      </c>
-      <c r="AE8" t="inlineStr">
+        <v>30</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>30</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>15</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>60</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr"/>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>⚠️整理</t>
+        </is>
+      </c>
+      <c r="AK8" t="inlineStr">
+        <is>
+          <t>整理觀察</t>
+        </is>
+      </c>
+      <c r="AL8" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能溫和放大</t>
         </is>
       </c>
-      <c r="AF8" t="inlineStr">
+      <c r="AM8" t="inlineStr">
         <is>
           <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
-      <c r="AG8" t="inlineStr">
-        <is>
-          <t>強勢偏多：跌破5日線、多頭排列、量能溫和放大、法人連續偏買、5日法人明顯買超。可列入優先觀察，但仍需留意乖離與量能是否過熱。</t>
+      <c r="AN8" t="inlineStr">
+        <is>
+          <t>整理觀察：跌破5日線、多頭排列、量能溫和放大、法人連續偏買、5日法人明顯買超。多空訊號混合，建議降低追價衝動。</t>
         </is>
       </c>
     </row>
@@ -1491,31 +1631,46 @@
         <v>478457</v>
       </c>
       <c r="AB9" t="n">
-        <v>65</v>
-      </c>
-      <c r="AC9" t="inlineStr">
-        <is>
-          <t>👀觀察</t>
-        </is>
-      </c>
-      <c r="AD9" t="inlineStr">
-        <is>
-          <t>偏多觀察</t>
-        </is>
-      </c>
-      <c r="AE9" t="inlineStr">
+        <v>26</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>26</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>60</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG9" t="inlineStr"/>
+      <c r="AH9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr"/>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>⚠️整理</t>
+        </is>
+      </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t>整理觀察</t>
+        </is>
+      </c>
+      <c r="AL9" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF9" t="inlineStr">
+      <c r="AM9" t="inlineStr">
         <is>
           <t>法人連續偏買、5日法人明顯買超、投信買外資賣</t>
         </is>
       </c>
-      <c r="AG9" t="inlineStr">
-        <is>
-          <t>偏多觀察：跌破5日線、多頭排列、量能未放大、法人連續偏買、5日法人明顯買超、投信買外資賣。條件不差，適合等待拉回或突破確認。</t>
+      <c r="AN9" t="inlineStr">
+        <is>
+          <t>整理觀察：跌破5日線、多頭排列、量能未放大、法人連續偏買、5日法人明顯買超、投信買外資賣。多空訊號混合，建議降低追價衝動。</t>
         </is>
       </c>
     </row>
@@ -1608,31 +1763,46 @@
         <v>177977</v>
       </c>
       <c r="AB10" t="n">
-        <v>55</v>
-      </c>
-      <c r="AC10" t="inlineStr">
-        <is>
-          <t>👀觀察</t>
-        </is>
-      </c>
-      <c r="AD10" t="inlineStr">
-        <is>
-          <t>偏多觀察</t>
-        </is>
-      </c>
-      <c r="AE10" t="inlineStr">
+        <v>22</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>22</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>50</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG10" t="inlineStr"/>
+      <c r="AH10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr"/>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>⚠️整理</t>
+        </is>
+      </c>
+      <c r="AK10" t="inlineStr">
+        <is>
+          <t>整理觀察</t>
+        </is>
+      </c>
+      <c r="AL10" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF10" t="inlineStr">
+      <c r="AM10" t="inlineStr">
         <is>
           <t>5日法人明顯買超、外資投信同步買超</t>
         </is>
       </c>
-      <c r="AG10" t="inlineStr">
-        <is>
-          <t>偏多觀察：跌破5日線、多頭排列、量能未放大、5日法人明顯買超、外資投信同步買超。條件不差，適合等待拉回或突破確認。</t>
+      <c r="AN10" t="inlineStr">
+        <is>
+          <t>整理觀察：跌破5日線、多頭排列、量能未放大、5日法人明顯買超、外資投信同步買超。多空訊號混合，建議降低追價衝動。</t>
         </is>
       </c>
     </row>
@@ -1725,31 +1895,46 @@
         <v>409195</v>
       </c>
       <c r="AB11" t="n">
-        <v>55</v>
-      </c>
-      <c r="AC11" t="inlineStr">
-        <is>
-          <t>👀觀察</t>
-        </is>
-      </c>
-      <c r="AD11" t="inlineStr">
-        <is>
-          <t>偏多觀察</t>
-        </is>
-      </c>
-      <c r="AE11" t="inlineStr">
+        <v>22</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>22</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>50</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG11" t="inlineStr"/>
+      <c r="AH11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr"/>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>⚠️整理</t>
+        </is>
+      </c>
+      <c r="AK11" t="inlineStr">
+        <is>
+          <t>整理觀察</t>
+        </is>
+      </c>
+      <c r="AL11" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF11" t="inlineStr">
+      <c r="AM11" t="inlineStr">
         <is>
           <t>5日法人明顯買超、外資投信同步買超</t>
         </is>
       </c>
-      <c r="AG11" t="inlineStr">
-        <is>
-          <t>偏多觀察：跌破5日線、多頭排列、量能未放大、5日法人明顯買超、外資投信同步買超。條件不差，適合等待拉回或突破確認。</t>
+      <c r="AN11" t="inlineStr">
+        <is>
+          <t>整理觀察：跌破5日線、多頭排列、量能未放大、5日法人明顯買超、外資投信同步買超。多空訊號混合，建議降低追價衝動。</t>
         </is>
       </c>
     </row>
@@ -1842,31 +2027,46 @@
         <v>-4135930</v>
       </c>
       <c r="AB12" t="n">
-        <v>55</v>
-      </c>
-      <c r="AC12" t="inlineStr">
-        <is>
-          <t>👀觀察</t>
-        </is>
-      </c>
-      <c r="AD12" t="inlineStr">
-        <is>
-          <t>偏多觀察</t>
-        </is>
-      </c>
-      <c r="AE12" t="inlineStr">
+        <v>22</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>22</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>50</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG12" t="inlineStr"/>
+      <c r="AH12" t="inlineStr"/>
+      <c r="AI12" t="inlineStr"/>
+      <c r="AJ12" t="inlineStr">
+        <is>
+          <t>⚠️整理</t>
+        </is>
+      </c>
+      <c r="AK12" t="inlineStr">
+        <is>
+          <t>整理觀察</t>
+        </is>
+      </c>
+      <c r="AL12" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF12" t="inlineStr">
+      <c r="AM12" t="inlineStr">
         <is>
           <t>5日法人明顯買超、外資投信同步買超</t>
         </is>
       </c>
-      <c r="AG12" t="inlineStr">
-        <is>
-          <t>偏多觀察：跌破5日線、多頭排列、量能未放大、5日法人明顯買超、外資投信同步買超。條件不差，適合等待拉回或突破確認。</t>
+      <c r="AN12" t="inlineStr">
+        <is>
+          <t>整理觀察：跌破5日線、多頭排列、量能未放大、5日法人明顯買超、外資投信同步買超。多空訊號混合，建議降低追價衝動。</t>
         </is>
       </c>
     </row>
@@ -1959,31 +2159,46 @@
         <v>2688460</v>
       </c>
       <c r="AB13" t="n">
-        <v>55</v>
-      </c>
-      <c r="AC13" t="inlineStr">
-        <is>
-          <t>👀觀察</t>
-        </is>
-      </c>
-      <c r="AD13" t="inlineStr">
-        <is>
-          <t>偏多觀察</t>
-        </is>
-      </c>
-      <c r="AE13" t="inlineStr">
+        <v>22</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>22</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>50</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG13" t="inlineStr"/>
+      <c r="AH13" t="inlineStr"/>
+      <c r="AI13" t="inlineStr"/>
+      <c r="AJ13" t="inlineStr">
+        <is>
+          <t>⚠️整理</t>
+        </is>
+      </c>
+      <c r="AK13" t="inlineStr">
+        <is>
+          <t>整理觀察</t>
+        </is>
+      </c>
+      <c r="AL13" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF13" t="inlineStr">
+      <c r="AM13" t="inlineStr">
         <is>
           <t>5日法人明顯買超、外資投信同步買超</t>
         </is>
       </c>
-      <c r="AG13" t="inlineStr">
-        <is>
-          <t>偏多觀察：跌破5日線、多頭排列、量能未放大、5日法人明顯買超、外資投信同步買超。條件不差，適合等待拉回或突破確認。</t>
+      <c r="AN13" t="inlineStr">
+        <is>
+          <t>整理觀察：跌破5日線、多頭排列、量能未放大、5日法人明顯買超、外資投信同步買超。多空訊號混合，建議降低追價衝動。</t>
         </is>
       </c>
     </row>
@@ -2076,31 +2291,46 @@
         <v>1252083</v>
       </c>
       <c r="AB14" t="n">
-        <v>55</v>
-      </c>
-      <c r="AC14" t="inlineStr">
-        <is>
-          <t>👀觀察</t>
-        </is>
-      </c>
-      <c r="AD14" t="inlineStr">
-        <is>
-          <t>偏多觀察</t>
-        </is>
-      </c>
-      <c r="AE14" t="inlineStr">
+        <v>22</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>22</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>50</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG14" t="inlineStr"/>
+      <c r="AH14" t="inlineStr"/>
+      <c r="AI14" t="inlineStr"/>
+      <c r="AJ14" t="inlineStr">
+        <is>
+          <t>⚠️整理</t>
+        </is>
+      </c>
+      <c r="AK14" t="inlineStr">
+        <is>
+          <t>整理觀察</t>
+        </is>
+      </c>
+      <c r="AL14" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF14" t="inlineStr">
+      <c r="AM14" t="inlineStr">
         <is>
           <t>5日法人明顯買超、外資投信同步買超</t>
         </is>
       </c>
-      <c r="AG14" t="inlineStr">
-        <is>
-          <t>偏多觀察：跌破5日線、多頭排列、量能未放大、5日法人明顯買超、外資投信同步買超。條件不差，適合等待拉回或突破確認。</t>
+      <c r="AN14" t="inlineStr">
+        <is>
+          <t>整理觀察：跌破5日線、多頭排列、量能未放大、5日法人明顯買超、外資投信同步買超。多空訊號混合，建議降低追價衝動。</t>
         </is>
       </c>
     </row>
@@ -2193,31 +2423,46 @@
         <v>112652</v>
       </c>
       <c r="AB15" t="n">
-        <v>55</v>
-      </c>
-      <c r="AC15" t="inlineStr">
-        <is>
-          <t>👀觀察</t>
-        </is>
-      </c>
-      <c r="AD15" t="inlineStr">
-        <is>
-          <t>偏多觀察</t>
-        </is>
-      </c>
-      <c r="AE15" t="inlineStr">
+        <v>22</v>
+      </c>
+      <c r="AC15" t="n">
+        <v>22</v>
+      </c>
+      <c r="AD15" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>50</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG15" t="inlineStr"/>
+      <c r="AH15" t="inlineStr"/>
+      <c r="AI15" t="inlineStr"/>
+      <c r="AJ15" t="inlineStr">
+        <is>
+          <t>⚠️整理</t>
+        </is>
+      </c>
+      <c r="AK15" t="inlineStr">
+        <is>
+          <t>整理觀察</t>
+        </is>
+      </c>
+      <c r="AL15" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF15" t="inlineStr">
+      <c r="AM15" t="inlineStr">
         <is>
           <t>5日法人明顯買超、外資投信同步買超</t>
         </is>
       </c>
-      <c r="AG15" t="inlineStr">
-        <is>
-          <t>偏多觀察：跌破5日線、多頭排列、量能未放大、5日法人明顯買超、外資投信同步買超。條件不差，適合等待拉回或突破確認。</t>
+      <c r="AN15" t="inlineStr">
+        <is>
+          <t>整理觀察：跌破5日線、多頭排列、量能未放大、5日法人明顯買超、外資投信同步買超。多空訊號混合，建議降低追價衝動。</t>
         </is>
       </c>
     </row>
@@ -2310,31 +2555,46 @@
         <v>-5556188</v>
       </c>
       <c r="AB16" t="n">
-        <v>55</v>
-      </c>
-      <c r="AC16" t="inlineStr">
-        <is>
-          <t>👀觀察</t>
-        </is>
-      </c>
-      <c r="AD16" t="inlineStr">
-        <is>
-          <t>偏多觀察</t>
-        </is>
-      </c>
-      <c r="AE16" t="inlineStr">
+        <v>22</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>22</v>
+      </c>
+      <c r="AD16" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE16" t="n">
+        <v>50</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG16" t="inlineStr"/>
+      <c r="AH16" t="inlineStr"/>
+      <c r="AI16" t="inlineStr"/>
+      <c r="AJ16" t="inlineStr">
+        <is>
+          <t>⚠️整理</t>
+        </is>
+      </c>
+      <c r="AK16" t="inlineStr">
+        <is>
+          <t>整理觀察</t>
+        </is>
+      </c>
+      <c r="AL16" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF16" t="inlineStr">
+      <c r="AM16" t="inlineStr">
         <is>
           <t>5日法人明顯買超、外資投信同步買超</t>
         </is>
       </c>
-      <c r="AG16" t="inlineStr">
-        <is>
-          <t>偏多觀察：跌破5日線、多頭排列、量能未放大、5日法人明顯買超、外資投信同步買超。條件不差，適合等待拉回或突破確認。</t>
+      <c r="AN16" t="inlineStr">
+        <is>
+          <t>整理觀察：跌破5日線、多頭排列、量能未放大、5日法人明顯買超、外資投信同步買超。多空訊號混合，建議降低追價衝動。</t>
         </is>
       </c>
     </row>
@@ -2427,31 +2687,46 @@
         <v>-2571</v>
       </c>
       <c r="AB17" t="n">
-        <v>45</v>
-      </c>
-      <c r="AC17" t="inlineStr">
-        <is>
-          <t>⚠️整理</t>
-        </is>
-      </c>
-      <c r="AD17" t="inlineStr">
-        <is>
-          <t>整理觀察</t>
-        </is>
-      </c>
-      <c r="AE17" t="inlineStr">
+        <v>18</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>18</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>25</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>20</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG17" t="inlineStr"/>
+      <c r="AH17" t="inlineStr"/>
+      <c r="AI17" t="inlineStr"/>
+      <c r="AJ17" t="inlineStr">
+        <is>
+          <t>❌避開</t>
+        </is>
+      </c>
+      <c r="AK17" t="inlineStr">
+        <is>
+          <t>觀望</t>
+        </is>
+      </c>
+      <c r="AL17" t="inlineStr">
         <is>
           <t>站上5日線、量能未放大、接近20日高點、接近20日低點</t>
         </is>
       </c>
-      <c r="AF17" t="inlineStr">
+      <c r="AM17" t="inlineStr">
         <is>
           <t>5日法人買超</t>
         </is>
       </c>
-      <c r="AG17" t="inlineStr">
-        <is>
-          <t>整理觀察：站上5日線、量能未放大、接近20日高點、接近20日低點、5日法人買超。多空訊號混合，建議降低追價衝動。</t>
+      <c r="AN17" t="inlineStr">
+        <is>
+          <t>風險偏高：站上5日線、量能未放大、接近20日高點、接近20日低點、5日法人買超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
@@ -2544,31 +2819,46 @@
         <v>-1207489</v>
       </c>
       <c r="AB18" t="n">
-        <v>45</v>
-      </c>
-      <c r="AC18" t="inlineStr">
-        <is>
-          <t>⚠️整理</t>
-        </is>
-      </c>
-      <c r="AD18" t="inlineStr">
-        <is>
-          <t>整理觀察</t>
-        </is>
-      </c>
-      <c r="AE18" t="inlineStr">
+        <v>18</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>18</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>15</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>30</v>
+      </c>
+      <c r="AF18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG18" t="inlineStr"/>
+      <c r="AH18" t="inlineStr"/>
+      <c r="AI18" t="inlineStr"/>
+      <c r="AJ18" t="inlineStr">
+        <is>
+          <t>❌避開</t>
+        </is>
+      </c>
+      <c r="AK18" t="inlineStr">
+        <is>
+          <t>觀望</t>
+        </is>
+      </c>
+      <c r="AL18" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能溫和放大</t>
         </is>
       </c>
-      <c r="AF18" t="inlineStr">
+      <c r="AM18" t="inlineStr">
         <is>
           <t>5日法人明顯買超、投信買外資賣</t>
         </is>
       </c>
-      <c r="AG18" t="inlineStr">
-        <is>
-          <t>整理觀察：跌破5日線、多頭排列、量能溫和放大、5日法人明顯買超、投信買外資賣。多空訊號混合，建議降低追價衝動。</t>
+      <c r="AN18" t="inlineStr">
+        <is>
+          <t>風險偏高：跌破5日線、多頭排列、量能溫和放大、5日法人明顯買超、投信買外資賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
@@ -2661,31 +2951,46 @@
         <v>-117849</v>
       </c>
       <c r="AB19" t="n">
-        <v>40</v>
-      </c>
-      <c r="AC19" t="inlineStr">
-        <is>
-          <t>⚠️整理</t>
-        </is>
-      </c>
-      <c r="AD19" t="inlineStr">
-        <is>
-          <t>整理觀察</t>
-        </is>
-      </c>
-      <c r="AE19" t="inlineStr">
+        <v>16</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>16</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>-10</v>
+      </c>
+      <c r="AE19" t="n">
+        <v>50</v>
+      </c>
+      <c r="AF19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG19" t="inlineStr"/>
+      <c r="AH19" t="inlineStr"/>
+      <c r="AI19" t="inlineStr"/>
+      <c r="AJ19" t="inlineStr">
+        <is>
+          <t>❌避開</t>
+        </is>
+      </c>
+      <c r="AK19" t="inlineStr">
+        <is>
+          <t>觀望</t>
+        </is>
+      </c>
+      <c r="AL19" t="inlineStr">
         <is>
           <t>跌破5日線、量能溫和放大</t>
         </is>
       </c>
-      <c r="AF19" t="inlineStr">
+      <c r="AM19" t="inlineStr">
         <is>
           <t>法人連續偏買、5日法人買超、外資買投信賣</t>
         </is>
       </c>
-      <c r="AG19" t="inlineStr">
-        <is>
-          <t>整理觀察：跌破5日線、量能溫和放大、法人連續偏買、5日法人買超、外資買投信賣。多空訊號混合，建議降低追價衝動。</t>
+      <c r="AN19" t="inlineStr">
+        <is>
+          <t>風險偏高：跌破5日線、量能溫和放大、法人連續偏買、5日法人買超、外資買投信賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
@@ -2778,31 +3083,46 @@
         <v>4134585</v>
       </c>
       <c r="AB20" t="n">
-        <v>35</v>
-      </c>
-      <c r="AC20" t="inlineStr">
-        <is>
-          <t>⚠️整理</t>
-        </is>
-      </c>
-      <c r="AD20" t="inlineStr">
-        <is>
-          <t>整理觀察</t>
-        </is>
-      </c>
-      <c r="AE20" t="inlineStr">
+        <v>14</v>
+      </c>
+      <c r="AC20" t="n">
+        <v>14</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>30</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG20" t="inlineStr"/>
+      <c r="AH20" t="inlineStr"/>
+      <c r="AI20" t="inlineStr"/>
+      <c r="AJ20" t="inlineStr">
+        <is>
+          <t>❌避開</t>
+        </is>
+      </c>
+      <c r="AK20" t="inlineStr">
+        <is>
+          <t>觀望</t>
+        </is>
+      </c>
+      <c r="AL20" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF20" t="inlineStr">
+      <c r="AM20" t="inlineStr">
         <is>
           <t>5日法人明顯買超、投信買外資賣</t>
         </is>
       </c>
-      <c r="AG20" t="inlineStr">
-        <is>
-          <t>整理觀察：跌破5日線、多頭排列、量能未放大、5日法人明顯買超、投信買外資賣。多空訊號混合，建議降低追價衝動。</t>
+      <c r="AN20" t="inlineStr">
+        <is>
+          <t>風險偏高：跌破5日線、多頭排列、量能未放大、5日法人明顯買超、投信買外資賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
@@ -2895,31 +3215,46 @@
         <v>605989</v>
       </c>
       <c r="AB21" t="n">
-        <v>35</v>
-      </c>
-      <c r="AC21" t="inlineStr">
-        <is>
-          <t>⚠️整理</t>
-        </is>
-      </c>
-      <c r="AD21" t="inlineStr">
-        <is>
-          <t>整理觀察</t>
-        </is>
-      </c>
-      <c r="AE21" t="inlineStr">
+        <v>14</v>
+      </c>
+      <c r="AC21" t="n">
+        <v>14</v>
+      </c>
+      <c r="AD21" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE21" t="n">
+        <v>30</v>
+      </c>
+      <c r="AF21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG21" t="inlineStr"/>
+      <c r="AH21" t="inlineStr"/>
+      <c r="AI21" t="inlineStr"/>
+      <c r="AJ21" t="inlineStr">
+        <is>
+          <t>❌避開</t>
+        </is>
+      </c>
+      <c r="AK21" t="inlineStr">
+        <is>
+          <t>觀望</t>
+        </is>
+      </c>
+      <c r="AL21" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF21" t="inlineStr">
+      <c r="AM21" t="inlineStr">
         <is>
           <t>5日法人明顯買超</t>
         </is>
       </c>
-      <c r="AG21" t="inlineStr">
-        <is>
-          <t>整理觀察：跌破5日線、多頭排列、量能未放大、5日法人明顯買超。多空訊號混合，建議降低追價衝動。</t>
+      <c r="AN21" t="inlineStr">
+        <is>
+          <t>風險偏高：跌破5日線、多頭排列、量能未放大、5日法人明顯買超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
@@ -3012,31 +3347,46 @@
         <v>2584386</v>
       </c>
       <c r="AB22" t="n">
-        <v>35</v>
-      </c>
-      <c r="AC22" t="inlineStr">
-        <is>
-          <t>⚠️整理</t>
-        </is>
-      </c>
-      <c r="AD22" t="inlineStr">
-        <is>
-          <t>整理觀察</t>
-        </is>
-      </c>
-      <c r="AE22" t="inlineStr">
+        <v>14</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>14</v>
+      </c>
+      <c r="AD22" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE22" t="n">
+        <v>30</v>
+      </c>
+      <c r="AF22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG22" t="inlineStr"/>
+      <c r="AH22" t="inlineStr"/>
+      <c r="AI22" t="inlineStr"/>
+      <c r="AJ22" t="inlineStr">
+        <is>
+          <t>❌避開</t>
+        </is>
+      </c>
+      <c r="AK22" t="inlineStr">
+        <is>
+          <t>觀望</t>
+        </is>
+      </c>
+      <c r="AL22" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF22" t="inlineStr">
+      <c r="AM22" t="inlineStr">
         <is>
           <t>5日法人明顯買超</t>
         </is>
       </c>
-      <c r="AG22" t="inlineStr">
-        <is>
-          <t>整理觀察：跌破5日線、多頭排列、量能未放大、5日法人明顯買超。多空訊號混合，建議降低追價衝動。</t>
+      <c r="AN22" t="inlineStr">
+        <is>
+          <t>風險偏高：跌破5日線、多頭排列、量能未放大、5日法人明顯買超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
@@ -3129,31 +3479,46 @@
         <v>-628128</v>
       </c>
       <c r="AB23" t="n">
-        <v>35</v>
-      </c>
-      <c r="AC23" t="inlineStr">
-        <is>
-          <t>⚠️整理</t>
-        </is>
-      </c>
-      <c r="AD23" t="inlineStr">
-        <is>
-          <t>整理觀察</t>
-        </is>
-      </c>
-      <c r="AE23" t="inlineStr">
+        <v>14</v>
+      </c>
+      <c r="AC23" t="n">
+        <v>14</v>
+      </c>
+      <c r="AD23" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE23" t="n">
+        <v>30</v>
+      </c>
+      <c r="AF23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG23" t="inlineStr"/>
+      <c r="AH23" t="inlineStr"/>
+      <c r="AI23" t="inlineStr"/>
+      <c r="AJ23" t="inlineStr">
+        <is>
+          <t>❌避開</t>
+        </is>
+      </c>
+      <c r="AK23" t="inlineStr">
+        <is>
+          <t>觀望</t>
+        </is>
+      </c>
+      <c r="AL23" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF23" t="inlineStr">
+      <c r="AM23" t="inlineStr">
         <is>
           <t>5日法人明顯買超、外資買投信賣</t>
         </is>
       </c>
-      <c r="AG23" t="inlineStr">
-        <is>
-          <t>整理觀察：跌破5日線、多頭排列、量能未放大、5日法人明顯買超、外資買投信賣。多空訊號混合，建議降低追價衝動。</t>
+      <c r="AN23" t="inlineStr">
+        <is>
+          <t>風險偏高：跌破5日線、多頭排列、量能未放大、5日法人明顯買超、外資買投信賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
@@ -3246,31 +3611,46 @@
         <v>752682</v>
       </c>
       <c r="AB24" t="n">
-        <v>35</v>
-      </c>
-      <c r="AC24" t="inlineStr">
-        <is>
-          <t>⚠️整理</t>
-        </is>
-      </c>
-      <c r="AD24" t="inlineStr">
-        <is>
-          <t>整理觀察</t>
-        </is>
-      </c>
-      <c r="AE24" t="inlineStr">
+        <v>14</v>
+      </c>
+      <c r="AC24" t="n">
+        <v>14</v>
+      </c>
+      <c r="AD24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE24" t="n">
+        <v>30</v>
+      </c>
+      <c r="AF24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG24" t="inlineStr"/>
+      <c r="AH24" t="inlineStr"/>
+      <c r="AI24" t="inlineStr"/>
+      <c r="AJ24" t="inlineStr">
+        <is>
+          <t>❌避開</t>
+        </is>
+      </c>
+      <c r="AK24" t="inlineStr">
+        <is>
+          <t>觀望</t>
+        </is>
+      </c>
+      <c r="AL24" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF24" t="inlineStr">
+      <c r="AM24" t="inlineStr">
         <is>
           <t>5日法人明顯買超、投信買外資賣</t>
         </is>
       </c>
-      <c r="AG24" t="inlineStr">
-        <is>
-          <t>整理觀察：跌破5日線、多頭排列、量能未放大、5日法人明顯買超、投信買外資賣。多空訊號混合，建議降低追價衝動。</t>
+      <c r="AN24" t="inlineStr">
+        <is>
+          <t>風險偏高：跌破5日線、多頭排列、量能未放大、5日法人明顯買超、投信買外資賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
@@ -3363,31 +3743,46 @@
         <v>-192017</v>
       </c>
       <c r="AB25" t="n">
-        <v>25</v>
-      </c>
-      <c r="AC25" t="inlineStr">
-        <is>
-          <t>⚠️整理</t>
-        </is>
-      </c>
-      <c r="AD25" t="inlineStr">
-        <is>
-          <t>整理觀察</t>
-        </is>
-      </c>
-      <c r="AE25" t="inlineStr">
+        <v>10</v>
+      </c>
+      <c r="AC25" t="n">
+        <v>10</v>
+      </c>
+      <c r="AD25" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE25" t="n">
+        <v>20</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG25" t="inlineStr"/>
+      <c r="AH25" t="inlineStr"/>
+      <c r="AI25" t="inlineStr"/>
+      <c r="AJ25" t="inlineStr">
+        <is>
+          <t>❌避開</t>
+        </is>
+      </c>
+      <c r="AK25" t="inlineStr">
+        <is>
+          <t>觀望</t>
+        </is>
+      </c>
+      <c r="AL25" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF25" t="inlineStr">
+      <c r="AM25" t="inlineStr">
         <is>
           <t>5日法人買超、外資買投信賣</t>
         </is>
       </c>
-      <c r="AG25" t="inlineStr">
-        <is>
-          <t>整理觀察：跌破5日線、多頭排列、量能未放大、5日法人買超、外資買投信賣。多空訊號混合，建議降低追價衝動。</t>
+      <c r="AN25" t="inlineStr">
+        <is>
+          <t>風險偏高：跌破5日線、多頭排列、量能未放大、5日法人買超、外資買投信賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
@@ -3480,31 +3875,46 @@
         <v>1057775</v>
       </c>
       <c r="AB26" t="n">
-        <v>20</v>
-      </c>
-      <c r="AC26" t="inlineStr">
-        <is>
-          <t>⚠️整理</t>
-        </is>
-      </c>
-      <c r="AD26" t="inlineStr">
-        <is>
-          <t>整理觀察</t>
-        </is>
-      </c>
-      <c r="AE26" t="inlineStr">
+        <v>8</v>
+      </c>
+      <c r="AC26" t="n">
+        <v>8</v>
+      </c>
+      <c r="AD26" t="n">
+        <v>-10</v>
+      </c>
+      <c r="AE26" t="n">
+        <v>30</v>
+      </c>
+      <c r="AF26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG26" t="inlineStr"/>
+      <c r="AH26" t="inlineStr"/>
+      <c r="AI26" t="inlineStr"/>
+      <c r="AJ26" t="inlineStr">
+        <is>
+          <t>❌避開</t>
+        </is>
+      </c>
+      <c r="AK26" t="inlineStr">
+        <is>
+          <t>觀望</t>
+        </is>
+      </c>
+      <c r="AL26" t="inlineStr">
         <is>
           <t>跌破5日線、量能溫和放大</t>
         </is>
       </c>
-      <c r="AF26" t="inlineStr">
+      <c r="AM26" t="inlineStr">
         <is>
           <t>5日法人明顯買超、外資買投信賣</t>
         </is>
       </c>
-      <c r="AG26" t="inlineStr">
-        <is>
-          <t>整理觀察：跌破5日線、量能溫和放大、5日法人明顯買超、外資買投信賣。多空訊號混合，建議降低追價衝動。</t>
+      <c r="AN26" t="inlineStr">
+        <is>
+          <t>風險偏高：跌破5日線、量能溫和放大、5日法人明顯買超、外資買投信賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
@@ -3597,29 +4007,44 @@
         <v>-15524</v>
       </c>
       <c r="AB27" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC27" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="AC27" t="n">
+        <v>4</v>
+      </c>
+      <c r="AD27" t="n">
+        <v>15</v>
+      </c>
+      <c r="AE27" t="n">
+        <v>-5</v>
+      </c>
+      <c r="AF27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG27" t="inlineStr"/>
+      <c r="AH27" t="inlineStr"/>
+      <c r="AI27" t="inlineStr"/>
+      <c r="AJ27" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD27" t="inlineStr">
+      <c r="AK27" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE27" t="inlineStr">
+      <c r="AL27" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能溫和放大</t>
         </is>
       </c>
-      <c r="AF27" t="inlineStr">
+      <c r="AM27" t="inlineStr">
         <is>
           <t>短線籌碼止穩、5日法人賣超、投信買外資賣</t>
         </is>
       </c>
-      <c r="AG27" t="inlineStr">
+      <c r="AN27" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、多頭排列、量能溫和放大、短線籌碼止穩、5日法人賣超、投信買外資賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -3714,29 +4139,44 @@
         <v>-569170</v>
       </c>
       <c r="AB28" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC28" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="AC28" t="n">
+        <v>4</v>
+      </c>
+      <c r="AD28" t="n">
+        <v>-20</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>30</v>
+      </c>
+      <c r="AF28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG28" t="inlineStr"/>
+      <c r="AH28" t="inlineStr"/>
+      <c r="AI28" t="inlineStr"/>
+      <c r="AJ28" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD28" t="inlineStr">
+      <c r="AK28" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE28" t="inlineStr">
+      <c r="AL28" t="inlineStr">
         <is>
           <t>跌破5日線、量能未放大</t>
         </is>
       </c>
-      <c r="AF28" t="inlineStr">
+      <c r="AM28" t="inlineStr">
         <is>
           <t>5日法人明顯買超、外資買投信賣</t>
         </is>
       </c>
-      <c r="AG28" t="inlineStr">
+      <c r="AN28" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、量能未放大、5日法人明顯買超、外資買投信賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -3831,29 +4271,44 @@
         <v>-127096</v>
       </c>
       <c r="AB29" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC29" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="AC29" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD29" t="n">
+        <v>-55</v>
+      </c>
+      <c r="AE29" t="n">
+        <v>60</v>
+      </c>
+      <c r="AF29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG29" t="inlineStr"/>
+      <c r="AH29" t="inlineStr"/>
+      <c r="AI29" t="inlineStr"/>
+      <c r="AJ29" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD29" t="inlineStr">
+      <c r="AK29" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE29" t="inlineStr">
+      <c r="AL29" t="inlineStr">
         <is>
           <t>跌破5日線、空頭排列、量能未放大、接近20日低點</t>
         </is>
       </c>
-      <c r="AF29" t="inlineStr">
+      <c r="AM29" t="inlineStr">
         <is>
           <t>法人連續偏買、5日法人明顯買超</t>
         </is>
       </c>
-      <c r="AG29" t="inlineStr">
+      <c r="AN29" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、空頭排列、量能未放大、接近20日低點、法人連續偏買、5日法人明顯買超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -3948,29 +4403,44 @@
         <v>4471704</v>
       </c>
       <c r="AB30" t="n">
-        <v>5</v>
-      </c>
-      <c r="AC30" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="AC30" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD30" t="n">
+        <v>20</v>
+      </c>
+      <c r="AE30" t="n">
+        <v>-15</v>
+      </c>
+      <c r="AF30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG30" t="inlineStr"/>
+      <c r="AH30" t="inlineStr"/>
+      <c r="AI30" t="inlineStr"/>
+      <c r="AJ30" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD30" t="inlineStr">
+      <c r="AK30" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE30" t="inlineStr">
+      <c r="AL30" t="inlineStr">
         <is>
           <t>站上5日線、量能未放大</t>
         </is>
       </c>
-      <c r="AF30" t="inlineStr">
+      <c r="AM30" t="inlineStr">
         <is>
           <t>短線籌碼止穩、5日法人明顯賣超、投信買外資賣</t>
         </is>
       </c>
-      <c r="AG30" t="inlineStr">
+      <c r="AN30" t="inlineStr">
         <is>
           <t>風險偏高：站上5日線、量能未放大、短線籌碼止穩、5日法人明顯賣超、投信買外資賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -4067,27 +4537,42 @@
       <c r="AB31" t="n">
         <v>0</v>
       </c>
-      <c r="AC31" t="inlineStr">
+      <c r="AC31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD31" t="n">
+        <v>-20</v>
+      </c>
+      <c r="AE31" t="n">
+        <v>20</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG31" t="inlineStr"/>
+      <c r="AH31" t="inlineStr"/>
+      <c r="AI31" t="inlineStr"/>
+      <c r="AJ31" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD31" t="inlineStr">
+      <c r="AK31" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE31" t="inlineStr">
+      <c r="AL31" t="inlineStr">
         <is>
           <t>跌破5日線、量能未放大</t>
         </is>
       </c>
-      <c r="AF31" t="inlineStr">
+      <c r="AM31" t="inlineStr">
         <is>
           <t>5日法人買超</t>
         </is>
       </c>
-      <c r="AG31" t="inlineStr">
+      <c r="AN31" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、量能未放大、5日法人買超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -4182,29 +4667,44 @@
         <v>-267465</v>
       </c>
       <c r="AB32" t="n">
-        <v>-5</v>
-      </c>
-      <c r="AC32" t="inlineStr">
+        <v>-2</v>
+      </c>
+      <c r="AC32" t="n">
+        <v>-2</v>
+      </c>
+      <c r="AD32" t="n">
+        <v>55</v>
+      </c>
+      <c r="AE32" t="n">
+        <v>-60</v>
+      </c>
+      <c r="AF32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG32" t="inlineStr"/>
+      <c r="AH32" t="inlineStr"/>
+      <c r="AI32" t="inlineStr"/>
+      <c r="AJ32" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD32" t="inlineStr">
+      <c r="AK32" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE32" t="inlineStr">
+      <c r="AL32" t="inlineStr">
         <is>
           <t>站上5日線、多頭排列、量能溫和放大</t>
         </is>
       </c>
-      <c r="AF32" t="inlineStr">
+      <c r="AM32" t="inlineStr">
         <is>
           <t>法人連續偏賣、中期買超轉短線賣壓、5日法人小幅賣超、投信買外資賣</t>
         </is>
       </c>
-      <c r="AG32" t="inlineStr">
+      <c r="AN32" t="inlineStr">
         <is>
           <t>風險偏高：站上5日線、多頭排列、量能溫和放大、法人連續偏賣、中期買超轉短線賣壓、5日法人小幅賣超、投信買外資賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -4299,29 +4799,44 @@
         <v>-46653750</v>
       </c>
       <c r="AB33" t="n">
-        <v>-10</v>
-      </c>
-      <c r="AC33" t="inlineStr">
+        <v>-4</v>
+      </c>
+      <c r="AC33" t="n">
+        <v>-4</v>
+      </c>
+      <c r="AD33" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE33" t="n">
+        <v>-15</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG33" t="inlineStr"/>
+      <c r="AH33" t="inlineStr"/>
+      <c r="AI33" t="inlineStr"/>
+      <c r="AJ33" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD33" t="inlineStr">
+      <c r="AK33" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE33" t="inlineStr">
+      <c r="AL33" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF33" t="inlineStr">
+      <c r="AM33" t="inlineStr">
         <is>
           <t>短線籌碼止穩、5日法人明顯賣超、投信買外資賣</t>
         </is>
       </c>
-      <c r="AG33" t="inlineStr">
+      <c r="AN33" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、多頭排列、量能未放大、短線籌碼止穩、5日法人明顯賣超、投信買外資賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -4416,29 +4931,44 @@
         <v>2300265</v>
       </c>
       <c r="AB34" t="n">
-        <v>-10</v>
-      </c>
-      <c r="AC34" t="inlineStr">
+        <v>-4</v>
+      </c>
+      <c r="AC34" t="n">
+        <v>-4</v>
+      </c>
+      <c r="AD34" t="n">
+        <v>45</v>
+      </c>
+      <c r="AE34" t="n">
+        <v>-55</v>
+      </c>
+      <c r="AF34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG34" t="inlineStr"/>
+      <c r="AH34" t="inlineStr"/>
+      <c r="AI34" t="inlineStr"/>
+      <c r="AJ34" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD34" t="inlineStr">
+      <c r="AK34" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE34" t="inlineStr">
+      <c r="AL34" t="inlineStr">
         <is>
           <t>站上5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF34" t="inlineStr">
+      <c r="AM34" t="inlineStr">
         <is>
           <t>法人連續偏賣、5日法人明顯賣超、投信買外資賣</t>
         </is>
       </c>
-      <c r="AG34" t="inlineStr">
+      <c r="AN34" t="inlineStr">
         <is>
           <t>風險偏高：站上5日線、多頭排列、量能未放大、法人連續偏賣、5日法人明顯賣超、投信買外資賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -4533,29 +5063,44 @@
         <v>933873</v>
       </c>
       <c r="AB35" t="n">
-        <v>-10</v>
-      </c>
-      <c r="AC35" t="inlineStr">
+        <v>-4</v>
+      </c>
+      <c r="AC35" t="n">
+        <v>-4</v>
+      </c>
+      <c r="AD35" t="n">
+        <v>45</v>
+      </c>
+      <c r="AE35" t="n">
+        <v>-55</v>
+      </c>
+      <c r="AF35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG35" t="inlineStr"/>
+      <c r="AH35" t="inlineStr"/>
+      <c r="AI35" t="inlineStr"/>
+      <c r="AJ35" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD35" t="inlineStr">
+      <c r="AK35" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE35" t="inlineStr">
+      <c r="AL35" t="inlineStr">
         <is>
           <t>站上5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF35" t="inlineStr">
+      <c r="AM35" t="inlineStr">
         <is>
           <t>法人連續偏賣、5日法人明顯賣超</t>
         </is>
       </c>
-      <c r="AG35" t="inlineStr">
+      <c r="AN35" t="inlineStr">
         <is>
           <t>風險偏高：站上5日線、多頭排列、量能未放大、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -4650,29 +5195,44 @@
         <v>-85904</v>
       </c>
       <c r="AB36" t="n">
-        <v>-15</v>
-      </c>
-      <c r="AC36" t="inlineStr">
+        <v>-6</v>
+      </c>
+      <c r="AC36" t="n">
+        <v>-6</v>
+      </c>
+      <c r="AD36" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE36" t="n">
+        <v>-20</v>
+      </c>
+      <c r="AF36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG36" t="inlineStr"/>
+      <c r="AH36" t="inlineStr"/>
+      <c r="AI36" t="inlineStr"/>
+      <c r="AJ36" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD36" t="inlineStr">
+      <c r="AK36" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE36" t="inlineStr">
+      <c r="AL36" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF36" t="inlineStr">
+      <c r="AM36" t="inlineStr">
         <is>
           <t>5日法人賣超</t>
         </is>
       </c>
-      <c r="AG36" t="inlineStr">
+      <c r="AN36" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、多頭排列、量能未放大、5日法人賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -4767,29 +5327,44 @@
         <v>-2184700</v>
       </c>
       <c r="AB37" t="n">
-        <v>-20</v>
-      </c>
-      <c r="AC37" t="inlineStr">
+        <v>-8</v>
+      </c>
+      <c r="AC37" t="n">
+        <v>-8</v>
+      </c>
+      <c r="AD37" t="n">
+        <v>15</v>
+      </c>
+      <c r="AE37" t="n">
+        <v>-35</v>
+      </c>
+      <c r="AF37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG37" t="inlineStr"/>
+      <c r="AH37" t="inlineStr"/>
+      <c r="AI37" t="inlineStr"/>
+      <c r="AJ37" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD37" t="inlineStr">
+      <c r="AK37" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE37" t="inlineStr">
+      <c r="AL37" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能溫和放大</t>
         </is>
       </c>
-      <c r="AF37" t="inlineStr">
+      <c r="AM37" t="inlineStr">
         <is>
           <t>中期買超轉短線賣壓、5日法人小幅賣超、外資買投信賣</t>
         </is>
       </c>
-      <c r="AG37" t="inlineStr">
+      <c r="AN37" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、多頭排列、量能溫和放大、中期買超轉短線賣壓、5日法人小幅賣超、外資買投信賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -4884,29 +5459,44 @@
         <v>-552608</v>
       </c>
       <c r="AB38" t="n">
+        <v>-8</v>
+      </c>
+      <c r="AC38" t="n">
+        <v>-8</v>
+      </c>
+      <c r="AD38" t="n">
         <v>-20</v>
       </c>
-      <c r="AC38" t="inlineStr">
+      <c r="AE38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG38" t="inlineStr"/>
+      <c r="AH38" t="inlineStr"/>
+      <c r="AI38" t="inlineStr"/>
+      <c r="AJ38" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD38" t="inlineStr">
+      <c r="AK38" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE38" t="inlineStr">
+      <c r="AL38" t="inlineStr">
         <is>
           <t>跌破5日線、量能未放大</t>
         </is>
       </c>
-      <c r="AF38" t="inlineStr">
+      <c r="AM38" t="inlineStr">
         <is>
           <t>籌碼中性、外資買投信賣</t>
         </is>
       </c>
-      <c r="AG38" t="inlineStr">
+      <c r="AN38" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、量能未放大、籌碼中性、外資買投信賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -5001,29 +5591,44 @@
         <v>-281077</v>
       </c>
       <c r="AB39" t="n">
-        <v>-25</v>
-      </c>
-      <c r="AC39" t="inlineStr">
+        <v>-10</v>
+      </c>
+      <c r="AC39" t="n">
+        <v>-10</v>
+      </c>
+      <c r="AD39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE39" t="n">
+        <v>-30</v>
+      </c>
+      <c r="AF39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG39" t="inlineStr"/>
+      <c r="AH39" t="inlineStr"/>
+      <c r="AI39" t="inlineStr"/>
+      <c r="AJ39" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD39" t="inlineStr">
+      <c r="AK39" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE39" t="inlineStr">
+      <c r="AL39" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF39" t="inlineStr">
+      <c r="AM39" t="inlineStr">
         <is>
           <t>5日法人明顯賣超、投信買外資賣</t>
         </is>
       </c>
-      <c r="AG39" t="inlineStr">
+      <c r="AN39" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、多頭排列、量能未放大、5日法人明顯賣超、投信買外資賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -5118,29 +5723,44 @@
         <v>-4976</v>
       </c>
       <c r="AB40" t="n">
-        <v>-35</v>
-      </c>
-      <c r="AC40" t="inlineStr">
+        <v>-14</v>
+      </c>
+      <c r="AC40" t="n">
+        <v>-14</v>
+      </c>
+      <c r="AD40" t="n">
+        <v>-20</v>
+      </c>
+      <c r="AE40" t="n">
+        <v>-15</v>
+      </c>
+      <c r="AF40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG40" t="inlineStr"/>
+      <c r="AH40" t="inlineStr"/>
+      <c r="AI40" t="inlineStr"/>
+      <c r="AJ40" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD40" t="inlineStr">
+      <c r="AK40" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE40" t="inlineStr">
+      <c r="AL40" t="inlineStr">
         <is>
           <t>跌破5日線、量能未放大</t>
         </is>
       </c>
-      <c r="AF40" t="inlineStr">
+      <c r="AM40" t="inlineStr">
         <is>
           <t>短線籌碼止穩、5日法人明顯賣超、投信買外資賣</t>
         </is>
       </c>
-      <c r="AG40" t="inlineStr">
+      <c r="AN40" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、量能未放大、短線籌碼止穩、5日法人明顯賣超、投信買外資賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -5235,29 +5855,44 @@
         <v>4679571</v>
       </c>
       <c r="AB41" t="n">
-        <v>-40</v>
-      </c>
-      <c r="AC41" t="inlineStr">
+        <v>-16</v>
+      </c>
+      <c r="AC41" t="n">
+        <v>-16</v>
+      </c>
+      <c r="AD41" t="n">
+        <v>15</v>
+      </c>
+      <c r="AE41" t="n">
+        <v>-55</v>
+      </c>
+      <c r="AF41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG41" t="inlineStr"/>
+      <c r="AH41" t="inlineStr"/>
+      <c r="AI41" t="inlineStr"/>
+      <c r="AJ41" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD41" t="inlineStr">
+      <c r="AK41" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE41" t="inlineStr">
+      <c r="AL41" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能溫和放大</t>
         </is>
       </c>
-      <c r="AF41" t="inlineStr">
+      <c r="AM41" t="inlineStr">
         <is>
           <t>法人連續偏賣、5日法人明顯賣超、投信買外資賣</t>
         </is>
       </c>
-      <c r="AG41" t="inlineStr">
+      <c r="AN41" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、多頭排列、量能溫和放大、法人連續偏賣、5日法人明顯賣超、投信買外資賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -5352,29 +5987,44 @@
         <v>23177890</v>
       </c>
       <c r="AB42" t="n">
-        <v>-40</v>
-      </c>
-      <c r="AC42" t="inlineStr">
+        <v>-16</v>
+      </c>
+      <c r="AC42" t="n">
+        <v>-16</v>
+      </c>
+      <c r="AD42" t="n">
+        <v>-10</v>
+      </c>
+      <c r="AE42" t="n">
+        <v>-30</v>
+      </c>
+      <c r="AF42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG42" t="inlineStr"/>
+      <c r="AH42" t="inlineStr"/>
+      <c r="AI42" t="inlineStr"/>
+      <c r="AJ42" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD42" t="inlineStr">
+      <c r="AK42" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE42" t="inlineStr">
+      <c r="AL42" t="inlineStr">
         <is>
           <t>跌破5日線、量能溫和放大</t>
         </is>
       </c>
-      <c r="AF42" t="inlineStr">
+      <c r="AM42" t="inlineStr">
         <is>
           <t>5日法人明顯賣超、外資買投信賣</t>
         </is>
       </c>
-      <c r="AG42" t="inlineStr">
+      <c r="AN42" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、量能溫和放大、5日法人明顯賣超、外資買投信賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -5469,29 +6119,44 @@
         <v>-120035</v>
       </c>
       <c r="AB43" t="n">
-        <v>-40</v>
-      </c>
-      <c r="AC43" t="inlineStr">
+        <v>-16</v>
+      </c>
+      <c r="AC43" t="n">
+        <v>-16</v>
+      </c>
+      <c r="AD43" t="n">
+        <v>-20</v>
+      </c>
+      <c r="AE43" t="n">
+        <v>-20</v>
+      </c>
+      <c r="AF43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG43" t="inlineStr"/>
+      <c r="AH43" t="inlineStr"/>
+      <c r="AI43" t="inlineStr"/>
+      <c r="AJ43" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD43" t="inlineStr">
+      <c r="AK43" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE43" t="inlineStr">
+      <c r="AL43" t="inlineStr">
         <is>
           <t>跌破5日線、量能未放大</t>
         </is>
       </c>
-      <c r="AF43" t="inlineStr">
+      <c r="AM43" t="inlineStr">
         <is>
           <t>5日法人賣超、投信買外資賣</t>
         </is>
       </c>
-      <c r="AG43" t="inlineStr">
+      <c r="AN43" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、量能未放大、5日法人賣超、投信買外資賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -5586,29 +6251,44 @@
         <v>4412359</v>
       </c>
       <c r="AB44" t="n">
-        <v>-40</v>
-      </c>
-      <c r="AC44" t="inlineStr">
+        <v>-16</v>
+      </c>
+      <c r="AC44" t="n">
+        <v>-16</v>
+      </c>
+      <c r="AD44" t="n">
+        <v>15</v>
+      </c>
+      <c r="AE44" t="n">
+        <v>-55</v>
+      </c>
+      <c r="AF44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG44" t="inlineStr"/>
+      <c r="AH44" t="inlineStr"/>
+      <c r="AI44" t="inlineStr"/>
+      <c r="AJ44" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD44" t="inlineStr">
+      <c r="AK44" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE44" t="inlineStr">
+      <c r="AL44" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能溫和放大</t>
         </is>
       </c>
-      <c r="AF44" t="inlineStr">
+      <c r="AM44" t="inlineStr">
         <is>
           <t>法人連續偏賣、5日法人明顯賣超、投信買外資賣</t>
         </is>
       </c>
-      <c r="AG44" t="inlineStr">
+      <c r="AN44" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、多頭排列、量能溫和放大、法人連續偏賣、5日法人明顯賣超、投信買外資賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -5703,29 +6383,44 @@
         <v>161799</v>
       </c>
       <c r="AB45" t="n">
-        <v>-45</v>
-      </c>
-      <c r="AC45" t="inlineStr">
+        <v>-18</v>
+      </c>
+      <c r="AC45" t="n">
+        <v>-18</v>
+      </c>
+      <c r="AD45" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE45" t="n">
+        <v>-50</v>
+      </c>
+      <c r="AF45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG45" t="inlineStr"/>
+      <c r="AH45" t="inlineStr"/>
+      <c r="AI45" t="inlineStr"/>
+      <c r="AJ45" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD45" t="inlineStr">
+      <c r="AK45" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE45" t="inlineStr">
+      <c r="AL45" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF45" t="inlineStr">
+      <c r="AM45" t="inlineStr">
         <is>
           <t>5日法人明顯賣超、外資投信同步賣超</t>
         </is>
       </c>
-      <c r="AG45" t="inlineStr">
+      <c r="AN45" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、多頭排列、量能未放大、5日法人明顯賣超、外資投信同步賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -5820,29 +6515,44 @@
         <v>-1998547</v>
       </c>
       <c r="AB46" t="n">
-        <v>-45</v>
-      </c>
-      <c r="AC46" t="inlineStr">
+        <v>-18</v>
+      </c>
+      <c r="AC46" t="n">
+        <v>-18</v>
+      </c>
+      <c r="AD46" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE46" t="n">
+        <v>-50</v>
+      </c>
+      <c r="AF46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG46" t="inlineStr"/>
+      <c r="AH46" t="inlineStr"/>
+      <c r="AI46" t="inlineStr"/>
+      <c r="AJ46" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD46" t="inlineStr">
+      <c r="AK46" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE46" t="inlineStr">
+      <c r="AL46" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF46" t="inlineStr">
+      <c r="AM46" t="inlineStr">
         <is>
           <t>5日法人明顯賣超、外資投信同步賣超</t>
         </is>
       </c>
-      <c r="AG46" t="inlineStr">
+      <c r="AN46" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、多頭排列、量能未放大、5日法人明顯賣超、外資投信同步賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -5937,29 +6647,44 @@
         <v>-2443069</v>
       </c>
       <c r="AB47" t="n">
-        <v>-50</v>
-      </c>
-      <c r="AC47" t="inlineStr">
+        <v>-20</v>
+      </c>
+      <c r="AC47" t="n">
+        <v>-20</v>
+      </c>
+      <c r="AD47" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE47" t="n">
+        <v>-55</v>
+      </c>
+      <c r="AF47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG47" t="inlineStr"/>
+      <c r="AH47" t="inlineStr"/>
+      <c r="AI47" t="inlineStr"/>
+      <c r="AJ47" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD47" t="inlineStr">
+      <c r="AK47" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE47" t="inlineStr">
+      <c r="AL47" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF47" t="inlineStr">
+      <c r="AM47" t="inlineStr">
         <is>
           <t>法人連續偏賣、5日法人明顯賣超</t>
         </is>
       </c>
-      <c r="AG47" t="inlineStr">
+      <c r="AN47" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、多頭排列、量能未放大、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -6054,29 +6779,44 @@
         <v>-467292</v>
       </c>
       <c r="AB48" t="n">
-        <v>-50</v>
-      </c>
-      <c r="AC48" t="inlineStr">
+        <v>-20</v>
+      </c>
+      <c r="AC48" t="n">
+        <v>-20</v>
+      </c>
+      <c r="AD48" t="n">
+        <v>-20</v>
+      </c>
+      <c r="AE48" t="n">
+        <v>-30</v>
+      </c>
+      <c r="AF48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG48" t="inlineStr"/>
+      <c r="AH48" t="inlineStr"/>
+      <c r="AI48" t="inlineStr"/>
+      <c r="AJ48" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD48" t="inlineStr">
+      <c r="AK48" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE48" t="inlineStr">
+      <c r="AL48" t="inlineStr">
         <is>
           <t>跌破5日線、量能未放大</t>
         </is>
       </c>
-      <c r="AF48" t="inlineStr">
+      <c r="AM48" t="inlineStr">
         <is>
           <t>5日法人明顯賣超、投信買外資賣</t>
         </is>
       </c>
-      <c r="AG48" t="inlineStr">
+      <c r="AN48" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、量能未放大、5日法人明顯賣超、投信買外資賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -6171,29 +6911,44 @@
         <v>-588912</v>
       </c>
       <c r="AB49" t="n">
-        <v>-50</v>
-      </c>
-      <c r="AC49" t="inlineStr">
+        <v>-20</v>
+      </c>
+      <c r="AC49" t="n">
+        <v>-20</v>
+      </c>
+      <c r="AD49" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE49" t="n">
+        <v>-55</v>
+      </c>
+      <c r="AF49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG49" t="inlineStr"/>
+      <c r="AH49" t="inlineStr"/>
+      <c r="AI49" t="inlineStr"/>
+      <c r="AJ49" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD49" t="inlineStr">
+      <c r="AK49" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE49" t="inlineStr">
+      <c r="AL49" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF49" t="inlineStr">
+      <c r="AM49" t="inlineStr">
         <is>
           <t>法人連續偏賣、5日法人明顯賣超、外資買投信賣</t>
         </is>
       </c>
-      <c r="AG49" t="inlineStr">
+      <c r="AN49" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、多頭排列、量能未放大、法人連續偏賣、5日法人明顯賣超、外資買投信賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -6288,29 +7043,44 @@
         <v>2885066</v>
       </c>
       <c r="AB50" t="n">
-        <v>-55</v>
-      </c>
-      <c r="AC50" t="inlineStr">
+        <v>-22</v>
+      </c>
+      <c r="AC50" t="n">
+        <v>-22</v>
+      </c>
+      <c r="AD50" t="n">
+        <v>20</v>
+      </c>
+      <c r="AE50" t="n">
+        <v>-75</v>
+      </c>
+      <c r="AF50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG50" t="inlineStr"/>
+      <c r="AH50" t="inlineStr"/>
+      <c r="AI50" t="inlineStr"/>
+      <c r="AJ50" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD50" t="inlineStr">
+      <c r="AK50" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE50" t="inlineStr">
+      <c r="AL50" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、成交量放大</t>
         </is>
       </c>
-      <c r="AF50" t="inlineStr">
+      <c r="AM50" t="inlineStr">
         <is>
           <t>中期買超轉短線賣壓、5日法人明顯賣超、外資投信同步賣超</t>
         </is>
       </c>
-      <c r="AG50" t="inlineStr">
+      <c r="AN50" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、多頭排列、成交量放大、中期買超轉短線賣壓、5日法人明顯賣超、外資投信同步賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -6405,29 +7175,44 @@
         <v>-149507</v>
       </c>
       <c r="AB51" t="n">
-        <v>-60</v>
-      </c>
-      <c r="AC51" t="inlineStr">
+        <v>-24</v>
+      </c>
+      <c r="AC51" t="n">
+        <v>-24</v>
+      </c>
+      <c r="AD51" t="n">
+        <v>-30</v>
+      </c>
+      <c r="AE51" t="n">
+        <v>-30</v>
+      </c>
+      <c r="AF51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG51" t="inlineStr"/>
+      <c r="AH51" t="inlineStr"/>
+      <c r="AI51" t="inlineStr"/>
+      <c r="AJ51" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD51" t="inlineStr">
+      <c r="AK51" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE51" t="inlineStr">
+      <c r="AL51" t="inlineStr">
         <is>
           <t>跌破5日線、量能未放大、接近20日低點</t>
         </is>
       </c>
-      <c r="AF51" t="inlineStr">
+      <c r="AM51" t="inlineStr">
         <is>
           <t>5日法人明顯賣超</t>
         </is>
       </c>
-      <c r="AG51" t="inlineStr">
+      <c r="AN51" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、量能未放大、接近20日低點、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -6522,29 +7307,44 @@
         <v>-280802</v>
       </c>
       <c r="AB52" t="n">
-        <v>-60</v>
-      </c>
-      <c r="AC52" t="inlineStr">
+        <v>-24</v>
+      </c>
+      <c r="AC52" t="n">
+        <v>-24</v>
+      </c>
+      <c r="AD52" t="n">
+        <v>-10</v>
+      </c>
+      <c r="AE52" t="n">
+        <v>-50</v>
+      </c>
+      <c r="AF52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG52" t="inlineStr"/>
+      <c r="AH52" t="inlineStr"/>
+      <c r="AI52" t="inlineStr"/>
+      <c r="AJ52" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD52" t="inlineStr">
+      <c r="AK52" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE52" t="inlineStr">
+      <c r="AL52" t="inlineStr">
         <is>
           <t>跌破5日線、量能溫和放大</t>
         </is>
       </c>
-      <c r="AF52" t="inlineStr">
+      <c r="AM52" t="inlineStr">
         <is>
           <t>5日法人明顯賣超、外資投信同步賣超</t>
         </is>
       </c>
-      <c r="AG52" t="inlineStr">
+      <c r="AN52" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、量能溫和放大、5日法人明顯賣超、外資投信同步賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -6639,29 +7439,44 @@
         <v>303643</v>
       </c>
       <c r="AB53" t="n">
-        <v>-60</v>
-      </c>
-      <c r="AC53" t="inlineStr">
+        <v>-24</v>
+      </c>
+      <c r="AC53" t="n">
+        <v>-24</v>
+      </c>
+      <c r="AD53" t="n">
+        <v>-10</v>
+      </c>
+      <c r="AE53" t="n">
+        <v>-50</v>
+      </c>
+      <c r="AF53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG53" t="inlineStr"/>
+      <c r="AH53" t="inlineStr"/>
+      <c r="AI53" t="inlineStr"/>
+      <c r="AJ53" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD53" t="inlineStr">
+      <c r="AK53" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE53" t="inlineStr">
+      <c r="AL53" t="inlineStr">
         <is>
           <t>跌破5日線、量能溫和放大</t>
         </is>
       </c>
-      <c r="AF53" t="inlineStr">
+      <c r="AM53" t="inlineStr">
         <is>
           <t>5日法人明顯賣超、外資投信同步賣超</t>
         </is>
       </c>
-      <c r="AG53" t="inlineStr">
+      <c r="AN53" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、量能溫和放大、5日法人明顯賣超、外資投信同步賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -6670,37 +7485,37 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>3105.TWO</t>
+          <t>3081.TWO</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>穩懋</t>
+          <t>聯亞</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>483.5</v>
+        <v>2655</v>
       </c>
       <c r="D54" t="n">
-        <v>507</v>
+        <v>2665</v>
       </c>
       <c r="E54" t="n">
-        <v>525.5</v>
+        <v>2756</v>
       </c>
       <c r="F54" t="n">
-        <v>504.9</v>
+        <v>2743.75</v>
       </c>
       <c r="G54" t="n">
-        <v>30445000</v>
+        <v>3094000</v>
       </c>
       <c r="H54" t="n">
-        <v>31281800</v>
+        <v>2418200</v>
       </c>
       <c r="I54" t="n">
-        <v>588</v>
+        <v>3215</v>
       </c>
       <c r="J54" t="n">
-        <v>436</v>
+        <v>2445</v>
       </c>
       <c r="K54" t="inlineStr">
         <is>
@@ -6711,113 +7526,128 @@
         <v>0</v>
       </c>
       <c r="M54" t="n">
-        <v>-5488502</v>
+        <v>-554317</v>
       </c>
       <c r="N54" t="n">
-        <v>-9353559</v>
+        <v>-1229802</v>
       </c>
       <c r="O54" t="n">
-        <v>-10995269</v>
+        <v>-1950372</v>
       </c>
       <c r="P54" t="n">
         <v>0</v>
       </c>
       <c r="Q54" t="n">
-        <v>-4438850</v>
+        <v>-458374</v>
       </c>
       <c r="R54" t="n">
-        <v>-6776494</v>
+        <v>-739509</v>
       </c>
       <c r="S54" t="n">
-        <v>-9455532</v>
+        <v>-1711064</v>
       </c>
       <c r="T54" t="n">
         <v>0</v>
       </c>
       <c r="U54" t="n">
-        <v>-141276</v>
+        <v>67299</v>
       </c>
       <c r="V54" t="n">
-        <v>-1019439</v>
+        <v>-286201</v>
       </c>
       <c r="W54" t="n">
-        <v>-1370765</v>
+        <v>-44623</v>
       </c>
       <c r="X54" t="n">
         <v>0</v>
       </c>
       <c r="Y54" t="n">
-        <v>-908376</v>
+        <v>-163242</v>
       </c>
       <c r="Z54" t="n">
-        <v>-1557626</v>
+        <v>-204092</v>
       </c>
       <c r="AA54" t="n">
-        <v>-168972</v>
+        <v>-194685</v>
       </c>
       <c r="AB54" t="n">
-        <v>-70</v>
-      </c>
-      <c r="AC54" t="inlineStr">
+        <v>-24</v>
+      </c>
+      <c r="AC54" t="n">
+        <v>-24</v>
+      </c>
+      <c r="AD54" t="n">
+        <v>-10</v>
+      </c>
+      <c r="AE54" t="n">
+        <v>-50</v>
+      </c>
+      <c r="AF54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG54" t="inlineStr"/>
+      <c r="AH54" t="inlineStr"/>
+      <c r="AI54" t="inlineStr"/>
+      <c r="AJ54" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD54" t="inlineStr">
+      <c r="AK54" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE54" t="inlineStr">
-        <is>
-          <t>跌破5日線、量能未放大</t>
-        </is>
-      </c>
-      <c r="AF54" t="inlineStr">
+      <c r="AL54" t="inlineStr">
+        <is>
+          <t>跌破5日線、量能溫和放大</t>
+        </is>
+      </c>
+      <c r="AM54" t="inlineStr">
         <is>
           <t>5日法人明顯賣超、外資投信同步賣超</t>
         </is>
       </c>
-      <c r="AG54" t="inlineStr">
-        <is>
-          <t>風險偏高：跌破5日線、量能未放大、5日法人明顯賣超、外資投信同步賣超。目前不適合積極追蹤，等待結構改善。</t>
+      <c r="AN54" t="inlineStr">
+        <is>
+          <t>風險偏高：跌破5日線、量能溫和放大、5日法人明顯賣超、外資投信同步賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2374.TW</t>
+          <t>3105.TWO</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>佳能</t>
+          <t>穩懋</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>79.7</v>
+        <v>483.5</v>
       </c>
       <c r="D55" t="n">
-        <v>81.88</v>
+        <v>507</v>
       </c>
       <c r="E55" t="n">
-        <v>81.81</v>
+        <v>525.5</v>
       </c>
       <c r="F55" t="n">
-        <v>81.42</v>
+        <v>504.9</v>
       </c>
       <c r="G55" t="n">
-        <v>15546534</v>
+        <v>30445000</v>
       </c>
       <c r="H55" t="n">
-        <v>13920640</v>
+        <v>31281800</v>
       </c>
       <c r="I55" t="n">
-        <v>86.40000000000001</v>
+        <v>588</v>
       </c>
       <c r="J55" t="n">
-        <v>77.2</v>
+        <v>436</v>
       </c>
       <c r="K55" t="inlineStr">
         <is>
@@ -6825,116 +7655,131 @@
         </is>
       </c>
       <c r="L55" t="n">
-        <v>-3501402</v>
+        <v>0</v>
       </c>
       <c r="M55" t="n">
-        <v>-6216003</v>
+        <v>-5488502</v>
       </c>
       <c r="N55" t="n">
-        <v>-7481768</v>
+        <v>-9353559</v>
       </c>
       <c r="O55" t="n">
-        <v>-8582233</v>
+        <v>-10995269</v>
       </c>
       <c r="P55" t="n">
-        <v>-3399304</v>
+        <v>0</v>
       </c>
       <c r="Q55" t="n">
-        <v>-5890258</v>
+        <v>-4438850</v>
       </c>
       <c r="R55" t="n">
-        <v>-7253249</v>
+        <v>-6776494</v>
       </c>
       <c r="S55" t="n">
-        <v>-8333523</v>
+        <v>-9455532</v>
       </c>
       <c r="T55" t="n">
-        <v>-1000</v>
+        <v>0</v>
       </c>
       <c r="U55" t="n">
-        <v>-1000</v>
+        <v>-141276</v>
       </c>
       <c r="V55" t="n">
-        <v>-1000</v>
+        <v>-1019439</v>
       </c>
       <c r="W55" t="n">
-        <v>-2000</v>
+        <v>-1370765</v>
       </c>
       <c r="X55" t="n">
-        <v>-101098</v>
+        <v>0</v>
       </c>
       <c r="Y55" t="n">
-        <v>-324745</v>
+        <v>-908376</v>
       </c>
       <c r="Z55" t="n">
-        <v>-227519</v>
+        <v>-1557626</v>
       </c>
       <c r="AA55" t="n">
-        <v>-246710</v>
+        <v>-168972</v>
       </c>
       <c r="AB55" t="n">
-        <v>-70</v>
-      </c>
-      <c r="AC55" t="inlineStr">
+        <v>-28</v>
+      </c>
+      <c r="AC55" t="n">
+        <v>-28</v>
+      </c>
+      <c r="AD55" t="n">
+        <v>-20</v>
+      </c>
+      <c r="AE55" t="n">
+        <v>-50</v>
+      </c>
+      <c r="AF55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG55" t="inlineStr"/>
+      <c r="AH55" t="inlineStr"/>
+      <c r="AI55" t="inlineStr"/>
+      <c r="AJ55" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD55" t="inlineStr">
+      <c r="AK55" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE55" t="inlineStr">
-        <is>
-          <t>跌破5日線、多頭排列、量能溫和放大、接近20日低點</t>
-        </is>
-      </c>
-      <c r="AF55" t="inlineStr">
-        <is>
-          <t>法人連續偏賣、5日法人明顯賣超、外資投信同步賣超</t>
-        </is>
-      </c>
-      <c r="AG55" t="inlineStr">
-        <is>
-          <t>風險偏高：跌破5日線、多頭排列、量能溫和放大、接近20日低點、法人連續偏賣、5日法人明顯賣超、外資投信同步賣超。目前不適合積極追蹤，等待結構改善。</t>
+      <c r="AL55" t="inlineStr">
+        <is>
+          <t>跌破5日線、量能未放大</t>
+        </is>
+      </c>
+      <c r="AM55" t="inlineStr">
+        <is>
+          <t>5日法人明顯賣超、外資投信同步賣超</t>
+        </is>
+      </c>
+      <c r="AN55" t="inlineStr">
+        <is>
+          <t>風險偏高：跌破5日線、量能未放大、5日法人明顯賣超、外資投信同步賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>3211.TWO</t>
+          <t>2374.TW</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>順達</t>
+          <t>佳能</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>423</v>
+        <v>79.7</v>
       </c>
       <c r="D56" t="n">
-        <v>439.8</v>
+        <v>81.88</v>
       </c>
       <c r="E56" t="n">
-        <v>443.7</v>
+        <v>81.81</v>
       </c>
       <c r="F56" t="n">
-        <v>409.07</v>
+        <v>81.42</v>
       </c>
       <c r="G56" t="n">
-        <v>10396000</v>
+        <v>15546534</v>
       </c>
       <c r="H56" t="n">
-        <v>12556200</v>
+        <v>13920640</v>
       </c>
       <c r="I56" t="n">
-        <v>492.5</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="J56" t="n">
-        <v>343</v>
+        <v>77.2</v>
       </c>
       <c r="K56" t="inlineStr">
         <is>
@@ -6942,116 +7787,131 @@
         </is>
       </c>
       <c r="L56" t="n">
-        <v>0</v>
+        <v>-3501402</v>
       </c>
       <c r="M56" t="n">
-        <v>709158</v>
+        <v>-6216003</v>
       </c>
       <c r="N56" t="n">
-        <v>-2262989</v>
+        <v>-7481768</v>
       </c>
       <c r="O56" t="n">
-        <v>8288668</v>
+        <v>-8582233</v>
       </c>
       <c r="P56" t="n">
-        <v>0</v>
+        <v>-3399304</v>
       </c>
       <c r="Q56" t="n">
-        <v>1534533</v>
+        <v>-5890258</v>
       </c>
       <c r="R56" t="n">
-        <v>-434369</v>
+        <v>-7253249</v>
       </c>
       <c r="S56" t="n">
-        <v>11800430</v>
+        <v>-8333523</v>
       </c>
       <c r="T56" t="n">
-        <v>0</v>
+        <v>-1000</v>
       </c>
       <c r="U56" t="n">
-        <v>-692000</v>
+        <v>-1000</v>
       </c>
       <c r="V56" t="n">
-        <v>-1650000</v>
+        <v>-1000</v>
       </c>
       <c r="W56" t="n">
-        <v>-3609000</v>
+        <v>-2000</v>
       </c>
       <c r="X56" t="n">
-        <v>0</v>
+        <v>-101098</v>
       </c>
       <c r="Y56" t="n">
-        <v>-133375</v>
+        <v>-324745</v>
       </c>
       <c r="Z56" t="n">
-        <v>-178620</v>
+        <v>-227519</v>
       </c>
       <c r="AA56" t="n">
-        <v>97238</v>
+        <v>-246710</v>
       </c>
       <c r="AB56" t="n">
-        <v>-70</v>
-      </c>
-      <c r="AC56" t="inlineStr">
+        <v>-28</v>
+      </c>
+      <c r="AC56" t="n">
+        <v>-28</v>
+      </c>
+      <c r="AD56" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE56" t="n">
+        <v>-75</v>
+      </c>
+      <c r="AF56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG56" t="inlineStr"/>
+      <c r="AH56" t="inlineStr"/>
+      <c r="AI56" t="inlineStr"/>
+      <c r="AJ56" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD56" t="inlineStr">
+      <c r="AK56" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE56" t="inlineStr">
-        <is>
-          <t>跌破5日線、量能未放大</t>
-        </is>
-      </c>
-      <c r="AF56" t="inlineStr">
-        <is>
-          <t>5日法人明顯賣超、外資投信同步賣超</t>
-        </is>
-      </c>
-      <c r="AG56" t="inlineStr">
-        <is>
-          <t>風險偏高：跌破5日線、量能未放大、5日法人明顯賣超、外資投信同步賣超。目前不適合積極追蹤，等待結構改善。</t>
+      <c r="AL56" t="inlineStr">
+        <is>
+          <t>跌破5日線、多頭排列、量能溫和放大、接近20日低點</t>
+        </is>
+      </c>
+      <c r="AM56" t="inlineStr">
+        <is>
+          <t>法人連續偏賣、5日法人明顯賣超、外資投信同步賣超</t>
+        </is>
+      </c>
+      <c r="AN56" t="inlineStr">
+        <is>
+          <t>風險偏高：跌破5日線、多頭排列、量能溫和放大、接近20日低點、法人連續偏賣、5日法人明顯賣超、外資投信同步賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>3081.TWO</t>
+          <t>3211.TWO</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>聯亞</t>
+          <t>順達</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>2615</v>
+        <v>423</v>
       </c>
       <c r="D57" t="n">
-        <v>2847</v>
+        <v>439.8</v>
       </c>
       <c r="E57" t="n">
-        <v>2728</v>
+        <v>443.7</v>
       </c>
       <c r="F57" t="n">
-        <v>2752.25</v>
+        <v>409.07</v>
       </c>
       <c r="G57" t="n">
-        <v>2144000</v>
+        <v>10396000</v>
       </c>
       <c r="H57" t="n">
-        <v>2878200</v>
+        <v>12556200</v>
       </c>
       <c r="I57" t="n">
-        <v>3215</v>
+        <v>492.5</v>
       </c>
       <c r="J57" t="n">
-        <v>2460</v>
+        <v>343</v>
       </c>
       <c r="K57" t="inlineStr">
         <is>
@@ -7062,74 +7922,89 @@
         <v>0</v>
       </c>
       <c r="M57" t="n">
-        <v>-554317</v>
+        <v>709158</v>
       </c>
       <c r="N57" t="n">
-        <v>-1229802</v>
+        <v>-2262989</v>
       </c>
       <c r="O57" t="n">
-        <v>-1950372</v>
+        <v>8288668</v>
       </c>
       <c r="P57" t="n">
         <v>0</v>
       </c>
       <c r="Q57" t="n">
-        <v>-458374</v>
+        <v>1534533</v>
       </c>
       <c r="R57" t="n">
-        <v>-739509</v>
+        <v>-434369</v>
       </c>
       <c r="S57" t="n">
-        <v>-1711064</v>
+        <v>11800430</v>
       </c>
       <c r="T57" t="n">
         <v>0</v>
       </c>
       <c r="U57" t="n">
-        <v>67299</v>
+        <v>-692000</v>
       </c>
       <c r="V57" t="n">
-        <v>-286201</v>
+        <v>-1650000</v>
       </c>
       <c r="W57" t="n">
-        <v>-44623</v>
+        <v>-3609000</v>
       </c>
       <c r="X57" t="n">
         <v>0</v>
       </c>
       <c r="Y57" t="n">
-        <v>-163242</v>
+        <v>-133375</v>
       </c>
       <c r="Z57" t="n">
-        <v>-204092</v>
+        <v>-178620</v>
       </c>
       <c r="AA57" t="n">
-        <v>-194685</v>
+        <v>97238</v>
       </c>
       <c r="AB57" t="n">
-        <v>-70</v>
-      </c>
-      <c r="AC57" t="inlineStr">
+        <v>-28</v>
+      </c>
+      <c r="AC57" t="n">
+        <v>-28</v>
+      </c>
+      <c r="AD57" t="n">
+        <v>-20</v>
+      </c>
+      <c r="AE57" t="n">
+        <v>-50</v>
+      </c>
+      <c r="AF57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG57" t="inlineStr"/>
+      <c r="AH57" t="inlineStr"/>
+      <c r="AI57" t="inlineStr"/>
+      <c r="AJ57" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD57" t="inlineStr">
+      <c r="AK57" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE57" t="inlineStr">
+      <c r="AL57" t="inlineStr">
         <is>
           <t>跌破5日線、量能未放大</t>
         </is>
       </c>
-      <c r="AF57" t="inlineStr">
+      <c r="AM57" t="inlineStr">
         <is>
           <t>5日法人明顯賣超、外資投信同步賣超</t>
         </is>
       </c>
-      <c r="AG57" t="inlineStr">
+      <c r="AN57" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、量能未放大、5日法人明顯賣超、外資投信同步賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -7224,29 +8099,44 @@
         <v>-114322</v>
       </c>
       <c r="AB58" t="n">
-        <v>-75</v>
-      </c>
-      <c r="AC58" t="inlineStr">
+        <v>-30</v>
+      </c>
+      <c r="AC58" t="n">
+        <v>-30</v>
+      </c>
+      <c r="AD58" t="n">
+        <v>-20</v>
+      </c>
+      <c r="AE58" t="n">
+        <v>-55</v>
+      </c>
+      <c r="AF58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG58" t="inlineStr"/>
+      <c r="AH58" t="inlineStr"/>
+      <c r="AI58" t="inlineStr"/>
+      <c r="AJ58" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD58" t="inlineStr">
+      <c r="AK58" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE58" t="inlineStr">
+      <c r="AL58" t="inlineStr">
         <is>
           <t>跌破5日線、量能未放大</t>
         </is>
       </c>
-      <c r="AF58" t="inlineStr">
+      <c r="AM58" t="inlineStr">
         <is>
           <t>法人連續偏賣、5日法人明顯賣超</t>
         </is>
       </c>
-      <c r="AG58" t="inlineStr">
+      <c r="AN58" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、量能未放大、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -7341,29 +8231,44 @@
         <v>299741</v>
       </c>
       <c r="AB59" t="n">
-        <v>-75</v>
-      </c>
-      <c r="AC59" t="inlineStr">
+        <v>-30</v>
+      </c>
+      <c r="AC59" t="n">
+        <v>-30</v>
+      </c>
+      <c r="AD59" t="n">
+        <v>-20</v>
+      </c>
+      <c r="AE59" t="n">
+        <v>-55</v>
+      </c>
+      <c r="AF59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG59" t="inlineStr"/>
+      <c r="AH59" t="inlineStr"/>
+      <c r="AI59" t="inlineStr"/>
+      <c r="AJ59" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD59" t="inlineStr">
+      <c r="AK59" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE59" t="inlineStr">
+      <c r="AL59" t="inlineStr">
         <is>
           <t>跌破5日線、量能未放大</t>
         </is>
       </c>
-      <c r="AF59" t="inlineStr">
+      <c r="AM59" t="inlineStr">
         <is>
           <t>法人連續偏賣、5日法人明顯賣超</t>
         </is>
       </c>
-      <c r="AG59" t="inlineStr">
+      <c r="AN59" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、量能未放大、法人連續偏賣、5日法人明顯賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -7458,29 +8363,44 @@
         <v>-5558309</v>
       </c>
       <c r="AB60" t="n">
-        <v>-75</v>
-      </c>
-      <c r="AC60" t="inlineStr">
+        <v>-30</v>
+      </c>
+      <c r="AC60" t="n">
+        <v>-30</v>
+      </c>
+      <c r="AD60" t="n">
+        <v>-20</v>
+      </c>
+      <c r="AE60" t="n">
+        <v>-55</v>
+      </c>
+      <c r="AF60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG60" t="inlineStr"/>
+      <c r="AH60" t="inlineStr"/>
+      <c r="AI60" t="inlineStr"/>
+      <c r="AJ60" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD60" t="inlineStr">
+      <c r="AK60" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE60" t="inlineStr">
+      <c r="AL60" t="inlineStr">
         <is>
           <t>跌破5日線、量能未放大</t>
         </is>
       </c>
-      <c r="AF60" t="inlineStr">
+      <c r="AM60" t="inlineStr">
         <is>
           <t>法人連續偏賣、5日法人明顯賣超、投信買外資賣</t>
         </is>
       </c>
-      <c r="AG60" t="inlineStr">
+      <c r="AN60" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、量能未放大、法人連續偏賣、5日法人明顯賣超、投信買外資賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -7575,29 +8495,44 @@
         <v>-1831866</v>
       </c>
       <c r="AB61" t="n">
-        <v>-75</v>
-      </c>
-      <c r="AC61" t="inlineStr">
+        <v>-30</v>
+      </c>
+      <c r="AC61" t="n">
+        <v>-30</v>
+      </c>
+      <c r="AD61" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE61" t="n">
+        <v>-80</v>
+      </c>
+      <c r="AF61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG61" t="inlineStr"/>
+      <c r="AH61" t="inlineStr"/>
+      <c r="AI61" t="inlineStr"/>
+      <c r="AJ61" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD61" t="inlineStr">
+      <c r="AK61" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE61" t="inlineStr">
+      <c r="AL61" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF61" t="inlineStr">
+      <c r="AM61" t="inlineStr">
         <is>
           <t>法人連續偏賣、中期買超轉短線賣壓、5日法人明顯賣超、投信買外資賣</t>
         </is>
       </c>
-      <c r="AG61" t="inlineStr">
+      <c r="AN61" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、多頭排列、量能未放大、法人連續偏賣、中期買超轉短線賣壓、5日法人明顯賣超、投信買外資賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -7692,29 +8627,44 @@
         <v>-133932</v>
       </c>
       <c r="AB62" t="n">
-        <v>-75</v>
-      </c>
-      <c r="AC62" t="inlineStr">
+        <v>-30</v>
+      </c>
+      <c r="AC62" t="n">
+        <v>-30</v>
+      </c>
+      <c r="AD62" t="n">
+        <v>-45</v>
+      </c>
+      <c r="AE62" t="n">
+        <v>-30</v>
+      </c>
+      <c r="AF62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG62" t="inlineStr"/>
+      <c r="AH62" t="inlineStr"/>
+      <c r="AI62" t="inlineStr"/>
+      <c r="AJ62" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD62" t="inlineStr">
+      <c r="AK62" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE62" t="inlineStr">
+      <c r="AL62" t="inlineStr">
         <is>
           <t>跌破5日線、空頭排列、量能溫和放大、接近20日低點</t>
         </is>
       </c>
-      <c r="AF62" t="inlineStr">
+      <c r="AM62" t="inlineStr">
         <is>
           <t>5日法人明顯賣超、投信買外資賣</t>
         </is>
       </c>
-      <c r="AG62" t="inlineStr">
+      <c r="AN62" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、空頭排列、量能溫和放大、接近20日低點、5日法人明顯賣超、投信買外資賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -7809,29 +8759,44 @@
         <v>661872</v>
       </c>
       <c r="AB63" t="n">
-        <v>-75</v>
-      </c>
-      <c r="AC63" t="inlineStr">
+        <v>-30</v>
+      </c>
+      <c r="AC63" t="n">
+        <v>-30</v>
+      </c>
+      <c r="AD63" t="n">
+        <v>-20</v>
+      </c>
+      <c r="AE63" t="n">
+        <v>-55</v>
+      </c>
+      <c r="AF63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG63" t="inlineStr"/>
+      <c r="AH63" t="inlineStr"/>
+      <c r="AI63" t="inlineStr"/>
+      <c r="AJ63" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD63" t="inlineStr">
+      <c r="AK63" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE63" t="inlineStr">
+      <c r="AL63" t="inlineStr">
         <is>
           <t>跌破5日線、量能未放大</t>
         </is>
       </c>
-      <c r="AF63" t="inlineStr">
+      <c r="AM63" t="inlineStr">
         <is>
           <t>法人連續偏賣、5日法人明顯賣超、外資買投信賣</t>
         </is>
       </c>
-      <c r="AG63" t="inlineStr">
+      <c r="AN63" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、量能未放大、法人連續偏賣、5日法人明顯賣超、外資買投信賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -7926,29 +8891,44 @@
         <v>-5852851</v>
       </c>
       <c r="AB64" t="n">
-        <v>-85</v>
-      </c>
-      <c r="AC64" t="inlineStr">
+        <v>-34</v>
+      </c>
+      <c r="AC64" t="n">
+        <v>-34</v>
+      </c>
+      <c r="AD64" t="n">
+        <v>-10</v>
+      </c>
+      <c r="AE64" t="n">
+        <v>-75</v>
+      </c>
+      <c r="AF64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG64" t="inlineStr"/>
+      <c r="AH64" t="inlineStr"/>
+      <c r="AI64" t="inlineStr"/>
+      <c r="AJ64" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD64" t="inlineStr">
+      <c r="AK64" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE64" t="inlineStr">
+      <c r="AL64" t="inlineStr">
         <is>
           <t>跌破5日線、量能溫和放大</t>
         </is>
       </c>
-      <c r="AF64" t="inlineStr">
+      <c r="AM64" t="inlineStr">
         <is>
           <t>法人連續偏賣、5日法人明顯賣超、外資投信同步賣超</t>
         </is>
       </c>
-      <c r="AG64" t="inlineStr">
+      <c r="AN64" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、量能溫和放大、法人連續偏賣、5日法人明顯賣超、外資投信同步賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -8043,29 +9023,44 @@
         <v>242708</v>
       </c>
       <c r="AB65" t="n">
-        <v>-85</v>
-      </c>
-      <c r="AC65" t="inlineStr">
+        <v>-34</v>
+      </c>
+      <c r="AC65" t="n">
+        <v>-34</v>
+      </c>
+      <c r="AD65" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE65" t="n">
+        <v>-90</v>
+      </c>
+      <c r="AF65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG65" t="inlineStr"/>
+      <c r="AH65" t="inlineStr"/>
+      <c r="AI65" t="inlineStr"/>
+      <c r="AJ65" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD65" t="inlineStr">
+      <c r="AK65" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE65" t="inlineStr">
+      <c r="AL65" t="inlineStr">
         <is>
           <t>跌破5日線、多頭排列、量能未放大</t>
         </is>
       </c>
-      <c r="AF65" t="inlineStr">
+      <c r="AM65" t="inlineStr">
         <is>
           <t>法人連續偏賣、中期買超轉短線賣壓、5日法人賣超、外資投信同步賣超</t>
         </is>
       </c>
-      <c r="AG65" t="inlineStr">
+      <c r="AN65" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、多頭排列、量能未放大、法人連續偏賣、中期買超轉短線賣壓、5日法人賣超、外資投信同步賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -8160,29 +9155,44 @@
         <v>-1736198</v>
       </c>
       <c r="AB66" t="n">
-        <v>-90</v>
-      </c>
-      <c r="AC66" t="inlineStr">
+        <v>-36</v>
+      </c>
+      <c r="AC66" t="n">
+        <v>-36</v>
+      </c>
+      <c r="AD66" t="n">
+        <v>-10</v>
+      </c>
+      <c r="AE66" t="n">
+        <v>-80</v>
+      </c>
+      <c r="AF66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG66" t="inlineStr"/>
+      <c r="AH66" t="inlineStr"/>
+      <c r="AI66" t="inlineStr"/>
+      <c r="AJ66" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD66" t="inlineStr">
+      <c r="AK66" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE66" t="inlineStr">
+      <c r="AL66" t="inlineStr">
         <is>
           <t>跌破5日線、量能溫和放大</t>
         </is>
       </c>
-      <c r="AF66" t="inlineStr">
+      <c r="AM66" t="inlineStr">
         <is>
           <t>法人連續偏賣、中期買超轉短線賣壓、5日法人明顯賣超、外資買投信賣</t>
         </is>
       </c>
-      <c r="AG66" t="inlineStr">
+      <c r="AN66" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、量能溫和放大、法人連續偏賣、中期買超轉短線賣壓、5日法人明顯賣超、外資買投信賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -8277,29 +9287,44 @@
         <v>-1335444</v>
       </c>
       <c r="AB67" t="n">
-        <v>-95</v>
-      </c>
-      <c r="AC67" t="inlineStr">
+        <v>-38</v>
+      </c>
+      <c r="AC67" t="n">
+        <v>-38</v>
+      </c>
+      <c r="AD67" t="n">
+        <v>-20</v>
+      </c>
+      <c r="AE67" t="n">
+        <v>-75</v>
+      </c>
+      <c r="AF67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG67" t="inlineStr"/>
+      <c r="AH67" t="inlineStr"/>
+      <c r="AI67" t="inlineStr"/>
+      <c r="AJ67" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD67" t="inlineStr">
+      <c r="AK67" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE67" t="inlineStr">
+      <c r="AL67" t="inlineStr">
         <is>
           <t>跌破5日線、量能未放大</t>
         </is>
       </c>
-      <c r="AF67" t="inlineStr">
+      <c r="AM67" t="inlineStr">
         <is>
           <t>法人連續偏賣、5日法人明顯賣超、外資投信同步賣超</t>
         </is>
       </c>
-      <c r="AG67" t="inlineStr">
+      <c r="AN67" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、量能未放大、法人連續偏賣、5日法人明顯賣超、外資投信同步賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -8394,29 +9419,44 @@
         <v>163202</v>
       </c>
       <c r="AB68" t="n">
-        <v>-95</v>
-      </c>
-      <c r="AC68" t="inlineStr">
+        <v>-38</v>
+      </c>
+      <c r="AC68" t="n">
+        <v>-38</v>
+      </c>
+      <c r="AD68" t="n">
+        <v>-20</v>
+      </c>
+      <c r="AE68" t="n">
+        <v>-75</v>
+      </c>
+      <c r="AF68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG68" t="inlineStr"/>
+      <c r="AH68" t="inlineStr"/>
+      <c r="AI68" t="inlineStr"/>
+      <c r="AJ68" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD68" t="inlineStr">
+      <c r="AK68" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE68" t="inlineStr">
+      <c r="AL68" t="inlineStr">
         <is>
           <t>跌破5日線、量能溫和放大、接近20日低點</t>
         </is>
       </c>
-      <c r="AF68" t="inlineStr">
+      <c r="AM68" t="inlineStr">
         <is>
           <t>法人連續偏賣、5日法人明顯賣超、外資投信同步賣超</t>
         </is>
       </c>
-      <c r="AG68" t="inlineStr">
+      <c r="AN68" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、量能溫和放大、接近20日低點、法人連續偏賣、5日法人明顯賣超、外資投信同步賣超。目前不適合積極追蹤，等待結構改善。</t>
         </is>
@@ -8511,29 +9551,44 @@
         <v>74827</v>
       </c>
       <c r="AB69" t="n">
-        <v>-100</v>
-      </c>
-      <c r="AC69" t="inlineStr">
+        <v>-40</v>
+      </c>
+      <c r="AC69" t="n">
+        <v>-40</v>
+      </c>
+      <c r="AD69" t="n">
+        <v>-20</v>
+      </c>
+      <c r="AE69" t="n">
+        <v>-80</v>
+      </c>
+      <c r="AF69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG69" t="inlineStr"/>
+      <c r="AH69" t="inlineStr"/>
+      <c r="AI69" t="inlineStr"/>
+      <c r="AJ69" t="inlineStr">
         <is>
           <t>❌避開</t>
         </is>
       </c>
-      <c r="AD69" t="inlineStr">
+      <c r="AK69" t="inlineStr">
         <is>
           <t>觀望</t>
         </is>
       </c>
-      <c r="AE69" t="inlineStr">
+      <c r="AL69" t="inlineStr">
         <is>
           <t>跌破5日線、量能未放大</t>
         </is>
       </c>
-      <c r="AF69" t="inlineStr">
+      <c r="AM69" t="inlineStr">
         <is>
           <t>法人連續偏賣、中期買超轉短線賣壓、5日法人明顯賣超、投信買外資賣</t>
         </is>
       </c>
-      <c r="AG69" t="inlineStr">
+      <c r="AN69" t="inlineStr">
         <is>
           <t>風險偏高：跌破5日線、量能未放大、法人連續偏賣、中期買超轉短線賣壓、5日法人明顯賣超、投信買外資賣。目前不適合積極追蹤，等待結構改善。</t>
         </is>

</xml_diff>

<commit_message>
update stock analysis data
</commit_message>
<xml_diff>
--- a/output/stock_analysis_result.xlsx
+++ b/output/stock_analysis_result.xlsx
@@ -938,10 +938,10 @@
         <v>32.96</v>
       </c>
       <c r="H4" t="n">
-        <v>37049127</v>
+        <v>37194127</v>
       </c>
       <c r="I4" t="n">
-        <v>30001308</v>
+        <v>30030308</v>
       </c>
       <c r="J4" t="n">
         <v>34.15</v>
@@ -2797,10 +2797,10 @@
         <v>154.4</v>
       </c>
       <c r="H17" t="n">
-        <v>30590982</v>
+        <v>30591982</v>
       </c>
       <c r="I17" t="n">
-        <v>28139896</v>
+        <v>28140096</v>
       </c>
       <c r="J17" t="n">
         <v>166</v>
@@ -3369,10 +3369,10 @@
         <v>42.67</v>
       </c>
       <c r="H21" t="n">
-        <v>26911949</v>
+        <v>26966949</v>
       </c>
       <c r="I21" t="n">
-        <v>64999561</v>
+        <v>65010561</v>
       </c>
       <c r="J21" t="n">
         <v>45.65</v>
@@ -3512,10 +3512,10 @@
         <v>248.15</v>
       </c>
       <c r="H22" t="n">
-        <v>37889704</v>
+        <v>39074704</v>
       </c>
       <c r="I22" t="n">
-        <v>40028658</v>
+        <v>40265658</v>
       </c>
       <c r="J22" t="n">
         <v>275.5</v>
@@ -4370,10 +4370,10 @@
         <v>128.78</v>
       </c>
       <c r="H28" t="n">
-        <v>26395566</v>
+        <v>26571566</v>
       </c>
       <c r="I28" t="n">
-        <v>26106715</v>
+        <v>26141915</v>
       </c>
       <c r="J28" t="n">
         <v>141</v>
@@ -5514,10 +5514,10 @@
         <v>69.48999999999999</v>
       </c>
       <c r="H36" t="n">
-        <v>49676897</v>
+        <v>50699897</v>
       </c>
       <c r="I36" t="n">
-        <v>75454312</v>
+        <v>75658912</v>
       </c>
       <c r="J36" t="n">
         <v>73.59999999999999</v>
@@ -5800,10 +5800,10 @@
         <v>174.97</v>
       </c>
       <c r="H38" t="n">
-        <v>134089840</v>
+        <v>134345840</v>
       </c>
       <c r="I38" t="n">
-        <v>131846709</v>
+        <v>131897909</v>
       </c>
       <c r="J38" t="n">
         <v>230</v>
@@ -8088,10 +8088,10 @@
         <v>2433</v>
       </c>
       <c r="H54" t="n">
-        <v>29493604</v>
+        <v>30538604</v>
       </c>
       <c r="I54" t="n">
-        <v>35201525</v>
+        <v>35410525</v>
       </c>
       <c r="J54" t="n">
         <v>2535</v>
@@ -9661,10 +9661,10 @@
         <v>336.15</v>
       </c>
       <c r="H65" t="n">
-        <v>5403663</v>
+        <v>5415663</v>
       </c>
       <c r="I65" t="n">
-        <v>4717079</v>
+        <v>4719479</v>
       </c>
       <c r="J65" t="n">
         <v>353</v>
@@ -12378,10 +12378,10 @@
         <v>2470.25</v>
       </c>
       <c r="H84" t="n">
-        <v>1265880</v>
+        <v>1274880</v>
       </c>
       <c r="I84" t="n">
-        <v>2276775</v>
+        <v>2278575</v>
       </c>
       <c r="J84" t="n">
         <v>2825</v>
@@ -13091,10 +13091,10 @@
         <v>949.25</v>
       </c>
       <c r="H89" t="n">
-        <v>27529533</v>
+        <v>27974533</v>
       </c>
       <c r="I89" t="n">
-        <v>32155522</v>
+        <v>32244522</v>
       </c>
       <c r="J89" t="n">
         <v>1115</v>
@@ -15379,10 +15379,10 @@
         <v>4117.75</v>
       </c>
       <c r="H105" t="n">
-        <v>5889689</v>
+        <v>6009689</v>
       </c>
       <c r="I105" t="n">
-        <v>8017389</v>
+        <v>8041389</v>
       </c>
       <c r="J105" t="n">
         <v>4785</v>

</xml_diff>